<commit_message>
Add consent columns in table description
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2131" uniqueCount="2131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2140" uniqueCount="2140">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -5987,10 +5987,37 @@
     <t xml:space="preserve">scope/text</t>
   </si>
   <si>
+    <t xml:space="preserve">cons_category_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_category_version</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_category_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_category_display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_category_text</t>
+  </si>
+  <si>
     <t xml:space="preserve">cons_datetime</t>
   </si>
   <si>
     <t xml:space="preserve">dateTime</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_policy_authority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy/authority</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cons_policy_uri</t>
+  </si>
+  <si>
+    <t xml:space="preserve">policy/uri</t>
   </si>
   <si>
     <t xml:space="preserve">cons_provision_type</t>
@@ -23301,22 +23328,20 @@
         <v>1991</v>
       </c>
       <c r="C1251" t="s">
-        <v>1992</v>
+        <v>251</v>
       </c>
       <c r="D1251"/>
-      <c r="E1251" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1251"/>
       <c r="F1251"/>
       <c r="G1251"/>
     </row>
     <row r="1252">
       <c r="A1252"/>
       <c r="B1252" t="s">
-        <v>1993</v>
+        <v>1992</v>
       </c>
       <c r="C1252" t="s">
-        <v>1994</v>
+        <v>253</v>
       </c>
       <c r="D1252"/>
       <c r="E1252"/>
@@ -23326,40 +23351,36 @@
     <row r="1253">
       <c r="A1253"/>
       <c r="B1253" t="s">
-        <v>1995</v>
+        <v>1993</v>
       </c>
       <c r="C1253" t="s">
-        <v>1996</v>
+        <v>255</v>
       </c>
       <c r="D1253"/>
-      <c r="E1253" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1253"/>
       <c r="F1253"/>
       <c r="G1253"/>
     </row>
     <row r="1254">
       <c r="A1254"/>
       <c r="B1254" t="s">
-        <v>1997</v>
+        <v>1994</v>
       </c>
       <c r="C1254" t="s">
-        <v>1998</v>
+        <v>257</v>
       </c>
       <c r="D1254"/>
-      <c r="E1254" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1254"/>
       <c r="F1254"/>
       <c r="G1254"/>
     </row>
     <row r="1255">
       <c r="A1255"/>
       <c r="B1255" t="s">
-        <v>1999</v>
+        <v>1995</v>
       </c>
       <c r="C1255" t="s">
-        <v>2000</v>
+        <v>259</v>
       </c>
       <c r="D1255"/>
       <c r="E1255"/>
@@ -23369,23 +23390,25 @@
     <row r="1256">
       <c r="A1256"/>
       <c r="B1256" t="s">
-        <v>2001</v>
+        <v>1996</v>
       </c>
       <c r="C1256" t="s">
-        <v>2002</v>
+        <v>1997</v>
       </c>
       <c r="D1256"/>
-      <c r="E1256"/>
+      <c r="E1256" t="s">
+        <v>18</v>
+      </c>
       <c r="F1256"/>
       <c r="G1256"/>
     </row>
     <row r="1257">
       <c r="A1257"/>
       <c r="B1257" t="s">
-        <v>2003</v>
+        <v>1998</v>
       </c>
       <c r="C1257" t="s">
-        <v>2004</v>
+        <v>1999</v>
       </c>
       <c r="D1257"/>
       <c r="E1257"/>
@@ -23395,10 +23418,10 @@
     <row r="1258">
       <c r="A1258"/>
       <c r="B1258" t="s">
-        <v>2005</v>
+        <v>2000</v>
       </c>
       <c r="C1258" t="s">
-        <v>2006</v>
+        <v>2001</v>
       </c>
       <c r="D1258"/>
       <c r="E1258"/>
@@ -23408,10 +23431,10 @@
     <row r="1259">
       <c r="A1259"/>
       <c r="B1259" t="s">
-        <v>2007</v>
+        <v>2002</v>
       </c>
       <c r="C1259" t="s">
-        <v>2008</v>
+        <v>2003</v>
       </c>
       <c r="D1259"/>
       <c r="E1259"/>
@@ -23421,36 +23444,40 @@
     <row r="1260">
       <c r="A1260"/>
       <c r="B1260" t="s">
-        <v>2009</v>
+        <v>2004</v>
       </c>
       <c r="C1260" t="s">
-        <v>2010</v>
+        <v>2005</v>
       </c>
       <c r="D1260"/>
-      <c r="E1260"/>
+      <c r="E1260" t="s">
+        <v>18</v>
+      </c>
       <c r="F1260"/>
       <c r="G1260"/>
     </row>
     <row r="1261">
       <c r="A1261"/>
       <c r="B1261" t="s">
-        <v>2011</v>
+        <v>2006</v>
       </c>
       <c r="C1261" t="s">
-        <v>2012</v>
+        <v>2007</v>
       </c>
       <c r="D1261"/>
-      <c r="E1261"/>
+      <c r="E1261" t="s">
+        <v>18</v>
+      </c>
       <c r="F1261"/>
       <c r="G1261"/>
     </row>
     <row r="1262">
       <c r="A1262"/>
       <c r="B1262" t="s">
-        <v>2013</v>
+        <v>2008</v>
       </c>
       <c r="C1262" t="s">
-        <v>2014</v>
+        <v>2009</v>
       </c>
       <c r="D1262"/>
       <c r="E1262"/>
@@ -23460,10 +23487,10 @@
     <row r="1263">
       <c r="A1263"/>
       <c r="B1263" t="s">
-        <v>2015</v>
+        <v>2010</v>
       </c>
       <c r="C1263" t="s">
-        <v>2016</v>
+        <v>2011</v>
       </c>
       <c r="D1263"/>
       <c r="E1263"/>
@@ -23473,10 +23500,10 @@
     <row r="1264">
       <c r="A1264"/>
       <c r="B1264" t="s">
-        <v>2017</v>
+        <v>2012</v>
       </c>
       <c r="C1264" t="s">
-        <v>2018</v>
+        <v>2013</v>
       </c>
       <c r="D1264"/>
       <c r="E1264"/>
@@ -23486,10 +23513,10 @@
     <row r="1265">
       <c r="A1265"/>
       <c r="B1265" t="s">
-        <v>2019</v>
+        <v>2014</v>
       </c>
       <c r="C1265" t="s">
-        <v>2020</v>
+        <v>2015</v>
       </c>
       <c r="D1265"/>
       <c r="E1265"/>
@@ -23499,10 +23526,10 @@
     <row r="1266">
       <c r="A1266"/>
       <c r="B1266" t="s">
-        <v>2021</v>
+        <v>2016</v>
       </c>
       <c r="C1266" t="s">
-        <v>2022</v>
+        <v>2017</v>
       </c>
       <c r="D1266"/>
       <c r="E1266"/>
@@ -23512,10 +23539,10 @@
     <row r="1267">
       <c r="A1267"/>
       <c r="B1267" t="s">
-        <v>2023</v>
+        <v>2018</v>
       </c>
       <c r="C1267" t="s">
-        <v>2024</v>
+        <v>2019</v>
       </c>
       <c r="D1267"/>
       <c r="E1267"/>
@@ -23525,10 +23552,10 @@
     <row r="1268">
       <c r="A1268"/>
       <c r="B1268" t="s">
-        <v>2025</v>
+        <v>2020</v>
       </c>
       <c r="C1268" t="s">
-        <v>2026</v>
+        <v>2021</v>
       </c>
       <c r="D1268"/>
       <c r="E1268"/>
@@ -23538,10 +23565,10 @@
     <row r="1269">
       <c r="A1269"/>
       <c r="B1269" t="s">
-        <v>2027</v>
+        <v>2022</v>
       </c>
       <c r="C1269" t="s">
-        <v>2028</v>
+        <v>2023</v>
       </c>
       <c r="D1269"/>
       <c r="E1269"/>
@@ -23551,10 +23578,10 @@
     <row r="1270">
       <c r="A1270"/>
       <c r="B1270" t="s">
-        <v>2029</v>
+        <v>2024</v>
       </c>
       <c r="C1270" t="s">
-        <v>2030</v>
+        <v>2025</v>
       </c>
       <c r="D1270"/>
       <c r="E1270"/>
@@ -23564,10 +23591,10 @@
     <row r="1271">
       <c r="A1271"/>
       <c r="B1271" t="s">
-        <v>2031</v>
+        <v>2026</v>
       </c>
       <c r="C1271" t="s">
-        <v>2032</v>
+        <v>2027</v>
       </c>
       <c r="D1271"/>
       <c r="E1271"/>
@@ -23577,10 +23604,10 @@
     <row r="1272">
       <c r="A1272"/>
       <c r="B1272" t="s">
-        <v>2033</v>
+        <v>2028</v>
       </c>
       <c r="C1272" t="s">
-        <v>2034</v>
+        <v>2029</v>
       </c>
       <c r="D1272"/>
       <c r="E1272"/>
@@ -23590,10 +23617,10 @@
     <row r="1273">
       <c r="A1273"/>
       <c r="B1273" t="s">
-        <v>2035</v>
+        <v>2030</v>
       </c>
       <c r="C1273" t="s">
-        <v>2036</v>
+        <v>2031</v>
       </c>
       <c r="D1273"/>
       <c r="E1273"/>
@@ -23603,10 +23630,10 @@
     <row r="1274">
       <c r="A1274"/>
       <c r="B1274" t="s">
-        <v>2037</v>
+        <v>2032</v>
       </c>
       <c r="C1274" t="s">
-        <v>2038</v>
+        <v>2033</v>
       </c>
       <c r="D1274"/>
       <c r="E1274"/>
@@ -23616,10 +23643,10 @@
     <row r="1275">
       <c r="A1275"/>
       <c r="B1275" t="s">
-        <v>2039</v>
+        <v>2034</v>
       </c>
       <c r="C1275" t="s">
-        <v>2040</v>
+        <v>2035</v>
       </c>
       <c r="D1275"/>
       <c r="E1275"/>
@@ -23629,40 +23656,36 @@
     <row r="1276">
       <c r="A1276"/>
       <c r="B1276" t="s">
-        <v>2041</v>
+        <v>2036</v>
       </c>
       <c r="C1276" t="s">
-        <v>2042</v>
+        <v>2037</v>
       </c>
       <c r="D1276"/>
-      <c r="E1276" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1276"/>
       <c r="F1276"/>
       <c r="G1276"/>
     </row>
     <row r="1277">
       <c r="A1277"/>
       <c r="B1277" t="s">
-        <v>2043</v>
+        <v>2038</v>
       </c>
       <c r="C1277" t="s">
-        <v>2044</v>
+        <v>2039</v>
       </c>
       <c r="D1277"/>
-      <c r="E1277" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1277"/>
       <c r="F1277"/>
       <c r="G1277"/>
     </row>
     <row r="1278">
       <c r="A1278"/>
       <c r="B1278" t="s">
-        <v>2045</v>
+        <v>2040</v>
       </c>
       <c r="C1278" t="s">
-        <v>2046</v>
+        <v>2041</v>
       </c>
       <c r="D1278"/>
       <c r="E1278"/>
@@ -23672,40 +23695,36 @@
     <row r="1279">
       <c r="A1279"/>
       <c r="B1279" t="s">
-        <v>2047</v>
+        <v>2042</v>
       </c>
       <c r="C1279" t="s">
-        <v>2048</v>
+        <v>2043</v>
       </c>
       <c r="D1279"/>
-      <c r="E1279" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1279"/>
       <c r="F1279"/>
       <c r="G1279"/>
     </row>
     <row r="1280">
       <c r="A1280"/>
       <c r="B1280" t="s">
-        <v>2049</v>
+        <v>2044</v>
       </c>
       <c r="C1280" t="s">
-        <v>2050</v>
+        <v>2045</v>
       </c>
       <c r="D1280"/>
-      <c r="E1280" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1280"/>
       <c r="F1280"/>
       <c r="G1280"/>
     </row>
     <row r="1281">
       <c r="A1281"/>
       <c r="B1281" t="s">
-        <v>2051</v>
+        <v>2046</v>
       </c>
       <c r="C1281" t="s">
-        <v>2052</v>
+        <v>2047</v>
       </c>
       <c r="D1281"/>
       <c r="E1281"/>
@@ -23715,10 +23734,10 @@
     <row r="1282">
       <c r="A1282"/>
       <c r="B1282" t="s">
-        <v>2053</v>
+        <v>2048</v>
       </c>
       <c r="C1282" t="s">
-        <v>2054</v>
+        <v>2049</v>
       </c>
       <c r="D1282"/>
       <c r="E1282"/>
@@ -23728,36 +23747,40 @@
     <row r="1283">
       <c r="A1283"/>
       <c r="B1283" t="s">
-        <v>2055</v>
+        <v>2050</v>
       </c>
       <c r="C1283" t="s">
-        <v>2056</v>
+        <v>2051</v>
       </c>
       <c r="D1283"/>
-      <c r="E1283"/>
+      <c r="E1283" t="s">
+        <v>18</v>
+      </c>
       <c r="F1283"/>
       <c r="G1283"/>
     </row>
     <row r="1284">
       <c r="A1284"/>
       <c r="B1284" t="s">
-        <v>2057</v>
+        <v>2052</v>
       </c>
       <c r="C1284" t="s">
-        <v>2058</v>
+        <v>2053</v>
       </c>
       <c r="D1284"/>
-      <c r="E1284"/>
+      <c r="E1284" t="s">
+        <v>18</v>
+      </c>
       <c r="F1284"/>
       <c r="G1284"/>
     </row>
     <row r="1285">
       <c r="A1285"/>
       <c r="B1285" t="s">
-        <v>2059</v>
+        <v>2054</v>
       </c>
       <c r="C1285" t="s">
-        <v>2060</v>
+        <v>2055</v>
       </c>
       <c r="D1285"/>
       <c r="E1285"/>
@@ -23767,36 +23790,40 @@
     <row r="1286">
       <c r="A1286"/>
       <c r="B1286" t="s">
-        <v>2061</v>
+        <v>2056</v>
       </c>
       <c r="C1286" t="s">
-        <v>2062</v>
+        <v>2057</v>
       </c>
       <c r="D1286"/>
-      <c r="E1286"/>
+      <c r="E1286" t="s">
+        <v>18</v>
+      </c>
       <c r="F1286"/>
       <c r="G1286"/>
     </row>
     <row r="1287">
       <c r="A1287"/>
       <c r="B1287" t="s">
-        <v>2063</v>
+        <v>2058</v>
       </c>
       <c r="C1287" t="s">
-        <v>2064</v>
+        <v>2059</v>
       </c>
       <c r="D1287"/>
-      <c r="E1287"/>
+      <c r="E1287" t="s">
+        <v>18</v>
+      </c>
       <c r="F1287"/>
       <c r="G1287"/>
     </row>
     <row r="1288">
       <c r="A1288"/>
       <c r="B1288" t="s">
-        <v>2065</v>
+        <v>2060</v>
       </c>
       <c r="C1288" t="s">
-        <v>2066</v>
+        <v>2061</v>
       </c>
       <c r="D1288"/>
       <c r="E1288"/>
@@ -23806,10 +23833,10 @@
     <row r="1289">
       <c r="A1289"/>
       <c r="B1289" t="s">
-        <v>2067</v>
+        <v>2062</v>
       </c>
       <c r="C1289" t="s">
-        <v>2068</v>
+        <v>2063</v>
       </c>
       <c r="D1289"/>
       <c r="E1289"/>
@@ -23819,10 +23846,10 @@
     <row r="1290">
       <c r="A1290"/>
       <c r="B1290" t="s">
-        <v>2069</v>
+        <v>2064</v>
       </c>
       <c r="C1290" t="s">
-        <v>2070</v>
+        <v>2065</v>
       </c>
       <c r="D1290"/>
       <c r="E1290"/>
@@ -23832,10 +23859,10 @@
     <row r="1291">
       <c r="A1291"/>
       <c r="B1291" t="s">
-        <v>2071</v>
+        <v>2066</v>
       </c>
       <c r="C1291" t="s">
-        <v>2072</v>
+        <v>2067</v>
       </c>
       <c r="D1291"/>
       <c r="E1291"/>
@@ -23845,10 +23872,10 @@
     <row r="1292">
       <c r="A1292"/>
       <c r="B1292" t="s">
-        <v>2073</v>
+        <v>2068</v>
       </c>
       <c r="C1292" t="s">
-        <v>2074</v>
+        <v>2069</v>
       </c>
       <c r="D1292"/>
       <c r="E1292"/>
@@ -23858,10 +23885,10 @@
     <row r="1293">
       <c r="A1293"/>
       <c r="B1293" t="s">
-        <v>2075</v>
+        <v>2070</v>
       </c>
       <c r="C1293" t="s">
-        <v>2076</v>
+        <v>2071</v>
       </c>
       <c r="D1293"/>
       <c r="E1293"/>
@@ -23871,10 +23898,10 @@
     <row r="1294">
       <c r="A1294"/>
       <c r="B1294" t="s">
-        <v>2077</v>
+        <v>2072</v>
       </c>
       <c r="C1294" t="s">
-        <v>2078</v>
+        <v>2073</v>
       </c>
       <c r="D1294"/>
       <c r="E1294"/>
@@ -23884,10 +23911,10 @@
     <row r="1295">
       <c r="A1295"/>
       <c r="B1295" t="s">
-        <v>2079</v>
+        <v>2074</v>
       </c>
       <c r="C1295" t="s">
-        <v>2080</v>
+        <v>2075</v>
       </c>
       <c r="D1295"/>
       <c r="E1295"/>
@@ -23897,10 +23924,10 @@
     <row r="1296">
       <c r="A1296"/>
       <c r="B1296" t="s">
-        <v>2081</v>
+        <v>2076</v>
       </c>
       <c r="C1296" t="s">
-        <v>2082</v>
+        <v>2077</v>
       </c>
       <c r="D1296"/>
       <c r="E1296"/>
@@ -23910,10 +23937,10 @@
     <row r="1297">
       <c r="A1297"/>
       <c r="B1297" t="s">
-        <v>2083</v>
+        <v>2078</v>
       </c>
       <c r="C1297" t="s">
-        <v>2084</v>
+        <v>2079</v>
       </c>
       <c r="D1297"/>
       <c r="E1297"/>
@@ -23923,10 +23950,10 @@
     <row r="1298">
       <c r="A1298"/>
       <c r="B1298" t="s">
-        <v>2085</v>
+        <v>2080</v>
       </c>
       <c r="C1298" t="s">
-        <v>2086</v>
+        <v>2081</v>
       </c>
       <c r="D1298"/>
       <c r="E1298"/>
@@ -23936,10 +23963,10 @@
     <row r="1299">
       <c r="A1299"/>
       <c r="B1299" t="s">
-        <v>2087</v>
+        <v>2082</v>
       </c>
       <c r="C1299" t="s">
-        <v>2088</v>
+        <v>2083</v>
       </c>
       <c r="D1299"/>
       <c r="E1299"/>
@@ -23949,10 +23976,10 @@
     <row r="1300">
       <c r="A1300"/>
       <c r="B1300" t="s">
-        <v>2089</v>
+        <v>2084</v>
       </c>
       <c r="C1300" t="s">
-        <v>2090</v>
+        <v>2085</v>
       </c>
       <c r="D1300"/>
       <c r="E1300"/>
@@ -23962,10 +23989,10 @@
     <row r="1301">
       <c r="A1301"/>
       <c r="B1301" t="s">
-        <v>2091</v>
+        <v>2086</v>
       </c>
       <c r="C1301" t="s">
-        <v>2092</v>
+        <v>2087</v>
       </c>
       <c r="D1301"/>
       <c r="E1301"/>
@@ -23975,51 +24002,49 @@
     <row r="1302">
       <c r="A1302"/>
       <c r="B1302" t="s">
-        <v>2093</v>
+        <v>2088</v>
       </c>
       <c r="C1302" t="s">
-        <v>2094</v>
+        <v>2089</v>
       </c>
       <c r="D1302"/>
-      <c r="E1302" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1302"/>
       <c r="F1302"/>
       <c r="G1302"/>
     </row>
     <row r="1303">
       <c r="A1303"/>
       <c r="B1303" t="s">
-        <v>2095</v>
+        <v>2090</v>
       </c>
       <c r="C1303" t="s">
-        <v>2096</v>
+        <v>2091</v>
       </c>
       <c r="D1303"/>
-      <c r="E1303" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1303"/>
       <c r="F1303"/>
       <c r="G1303"/>
     </row>
     <row r="1304">
       <c r="A1304"/>
-      <c r="B1304"/>
-      <c r="C1304"/>
+      <c r="B1304" t="s">
+        <v>2092</v>
+      </c>
+      <c r="C1304" t="s">
+        <v>2093</v>
+      </c>
       <c r="D1304"/>
       <c r="E1304"/>
       <c r="F1304"/>
       <c r="G1304"/>
     </row>
     <row r="1305">
-      <c r="A1305" t="s">
-        <v>122</v>
-      </c>
+      <c r="A1305"/>
       <c r="B1305" t="s">
-        <v>123</v>
+        <v>2094</v>
       </c>
       <c r="C1305" t="s">
-        <v>13</v>
+        <v>2095</v>
       </c>
       <c r="D1305"/>
       <c r="E1305"/>
@@ -24029,10 +24054,10 @@
     <row r="1306">
       <c r="A1306"/>
       <c r="B1306" t="s">
+        <v>2096</v>
+      </c>
+      <c r="C1306" t="s">
         <v>2097</v>
-      </c>
-      <c r="C1306" t="s">
-        <v>15</v>
       </c>
       <c r="D1306"/>
       <c r="E1306"/>
@@ -24045,22 +24070,20 @@
         <v>2098</v>
       </c>
       <c r="C1307" t="s">
-        <v>17</v>
+        <v>2099</v>
       </c>
       <c r="D1307"/>
-      <c r="E1307" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1307"/>
       <c r="F1307"/>
       <c r="G1307"/>
     </row>
     <row r="1308">
       <c r="A1308"/>
       <c r="B1308" t="s">
-        <v>2099</v>
+        <v>2100</v>
       </c>
       <c r="C1308" t="s">
-        <v>20</v>
+        <v>2101</v>
       </c>
       <c r="D1308"/>
       <c r="E1308"/>
@@ -24070,49 +24093,51 @@
     <row r="1309">
       <c r="A1309"/>
       <c r="B1309" t="s">
-        <v>2100</v>
+        <v>2102</v>
       </c>
       <c r="C1309" t="s">
-        <v>22</v>
+        <v>2103</v>
       </c>
       <c r="D1309"/>
-      <c r="E1309"/>
+      <c r="E1309" t="s">
+        <v>18</v>
+      </c>
       <c r="F1309"/>
       <c r="G1309"/>
     </row>
     <row r="1310">
       <c r="A1310"/>
       <c r="B1310" t="s">
-        <v>2101</v>
+        <v>2104</v>
       </c>
       <c r="C1310" t="s">
-        <v>24</v>
+        <v>2105</v>
       </c>
       <c r="D1310"/>
-      <c r="E1310"/>
+      <c r="E1310" t="s">
+        <v>18</v>
+      </c>
       <c r="F1310"/>
       <c r="G1310"/>
     </row>
     <row r="1311">
       <c r="A1311"/>
-      <c r="B1311" t="s">
-        <v>2102</v>
-      </c>
-      <c r="C1311" t="s">
-        <v>26</v>
-      </c>
+      <c r="B1311"/>
+      <c r="C1311"/>
       <c r="D1311"/>
       <c r="E1311"/>
       <c r="F1311"/>
       <c r="G1311"/>
     </row>
     <row r="1312">
-      <c r="A1312"/>
+      <c r="A1312" t="s">
+        <v>122</v>
+      </c>
       <c r="B1312" t="s">
-        <v>2103</v>
+        <v>123</v>
       </c>
       <c r="C1312" t="s">
-        <v>28</v>
+        <v>13</v>
       </c>
       <c r="D1312"/>
       <c r="E1312"/>
@@ -24122,10 +24147,10 @@
     <row r="1313">
       <c r="A1313"/>
       <c r="B1313" t="s">
-        <v>2104</v>
+        <v>2106</v>
       </c>
       <c r="C1313" t="s">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="D1313"/>
       <c r="E1313"/>
@@ -24135,23 +24160,25 @@
     <row r="1314">
       <c r="A1314"/>
       <c r="B1314" t="s">
-        <v>2105</v>
+        <v>2107</v>
       </c>
       <c r="C1314" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="D1314"/>
-      <c r="E1314"/>
+      <c r="E1314" t="s">
+        <v>18</v>
+      </c>
       <c r="F1314"/>
       <c r="G1314"/>
     </row>
     <row r="1315">
       <c r="A1315"/>
       <c r="B1315" t="s">
-        <v>2106</v>
+        <v>2108</v>
       </c>
       <c r="C1315" t="s">
-        <v>34</v>
+        <v>20</v>
       </c>
       <c r="D1315"/>
       <c r="E1315"/>
@@ -24161,10 +24188,10 @@
     <row r="1316">
       <c r="A1316"/>
       <c r="B1316" t="s">
-        <v>2107</v>
+        <v>2109</v>
       </c>
       <c r="C1316" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="D1316"/>
       <c r="E1316"/>
@@ -24174,40 +24201,36 @@
     <row r="1317">
       <c r="A1317"/>
       <c r="B1317" t="s">
-        <v>2108</v>
+        <v>2110</v>
       </c>
       <c r="C1317" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="D1317"/>
-      <c r="E1317" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1317"/>
       <c r="F1317"/>
       <c r="G1317"/>
     </row>
     <row r="1318">
       <c r="A1318"/>
       <c r="B1318" t="s">
-        <v>2109</v>
+        <v>2111</v>
       </c>
       <c r="C1318" t="s">
-        <v>40</v>
+        <v>26</v>
       </c>
       <c r="D1318"/>
-      <c r="E1318" t="s">
-        <v>18</v>
-      </c>
+      <c r="E1318"/>
       <c r="F1318"/>
       <c r="G1318"/>
     </row>
     <row r="1319">
       <c r="A1319"/>
       <c r="B1319" t="s">
-        <v>2110</v>
+        <v>2112</v>
       </c>
       <c r="C1319" t="s">
-        <v>50</v>
+        <v>28</v>
       </c>
       <c r="D1319"/>
       <c r="E1319"/>
@@ -24217,10 +24240,10 @@
     <row r="1320">
       <c r="A1320"/>
       <c r="B1320" t="s">
-        <v>2111</v>
+        <v>2113</v>
       </c>
       <c r="C1320" t="s">
-        <v>2112</v>
+        <v>30</v>
       </c>
       <c r="D1320"/>
       <c r="E1320"/>
@@ -24230,10 +24253,10 @@
     <row r="1321">
       <c r="A1321"/>
       <c r="B1321" t="s">
-        <v>2113</v>
+        <v>2114</v>
       </c>
       <c r="C1321" t="s">
-        <v>2114</v>
+        <v>32</v>
       </c>
       <c r="D1321"/>
       <c r="E1321"/>
@@ -24246,7 +24269,7 @@
         <v>2115</v>
       </c>
       <c r="C1322" t="s">
-        <v>2116</v>
+        <v>34</v>
       </c>
       <c r="D1322"/>
       <c r="E1322"/>
@@ -24256,10 +24279,10 @@
     <row r="1323">
       <c r="A1323"/>
       <c r="B1323" t="s">
-        <v>2117</v>
+        <v>2116</v>
       </c>
       <c r="C1323" t="s">
-        <v>2118</v>
+        <v>36</v>
       </c>
       <c r="D1323"/>
       <c r="E1323"/>
@@ -24269,36 +24292,40 @@
     <row r="1324">
       <c r="A1324"/>
       <c r="B1324" t="s">
-        <v>2119</v>
+        <v>2117</v>
       </c>
       <c r="C1324" t="s">
-        <v>2120</v>
+        <v>38</v>
       </c>
       <c r="D1324"/>
-      <c r="E1324"/>
+      <c r="E1324" t="s">
+        <v>18</v>
+      </c>
       <c r="F1324"/>
       <c r="G1324"/>
     </row>
     <row r="1325">
       <c r="A1325"/>
       <c r="B1325" t="s">
-        <v>2121</v>
+        <v>2118</v>
       </c>
       <c r="C1325" t="s">
-        <v>2122</v>
+        <v>40</v>
       </c>
       <c r="D1325"/>
-      <c r="E1325"/>
+      <c r="E1325" t="s">
+        <v>18</v>
+      </c>
       <c r="F1325"/>
       <c r="G1325"/>
     </row>
     <row r="1326">
       <c r="A1326"/>
       <c r="B1326" t="s">
-        <v>2123</v>
+        <v>2119</v>
       </c>
       <c r="C1326" t="s">
-        <v>2124</v>
+        <v>50</v>
       </c>
       <c r="D1326"/>
       <c r="E1326"/>
@@ -24308,10 +24335,10 @@
     <row r="1327">
       <c r="A1327"/>
       <c r="B1327" t="s">
-        <v>2125</v>
+        <v>2120</v>
       </c>
       <c r="C1327" t="s">
-        <v>2126</v>
+        <v>2121</v>
       </c>
       <c r="D1327"/>
       <c r="E1327"/>
@@ -24320,22 +24347,24 @@
     </row>
     <row r="1328">
       <c r="A1328"/>
-      <c r="B1328"/>
-      <c r="C1328"/>
+      <c r="B1328" t="s">
+        <v>2122</v>
+      </c>
+      <c r="C1328" t="s">
+        <v>2123</v>
+      </c>
       <c r="D1328"/>
       <c r="E1328"/>
       <c r="F1328"/>
       <c r="G1328"/>
     </row>
     <row r="1329">
-      <c r="A1329" t="s">
-        <v>2127</v>
-      </c>
+      <c r="A1329"/>
       <c r="B1329" t="s">
-        <v>2128</v>
+        <v>2124</v>
       </c>
       <c r="C1329" t="s">
-        <v>2128</v>
+        <v>2125</v>
       </c>
       <c r="D1329"/>
       <c r="E1329"/>
@@ -24345,10 +24374,10 @@
     <row r="1330">
       <c r="A1330"/>
       <c r="B1330" t="s">
-        <v>2129</v>
+        <v>2126</v>
       </c>
       <c r="C1330" t="s">
-        <v>2129</v>
+        <v>2127</v>
       </c>
       <c r="D1330"/>
       <c r="E1330"/>
@@ -24358,15 +24387,104 @@
     <row r="1331">
       <c r="A1331"/>
       <c r="B1331" t="s">
-        <v>2130</v>
+        <v>2128</v>
       </c>
       <c r="C1331" t="s">
-        <v>2130</v>
+        <v>2129</v>
       </c>
       <c r="D1331"/>
       <c r="E1331"/>
       <c r="F1331"/>
       <c r="G1331"/>
+    </row>
+    <row r="1332">
+      <c r="A1332"/>
+      <c r="B1332" t="s">
+        <v>2130</v>
+      </c>
+      <c r="C1332" t="s">
+        <v>2131</v>
+      </c>
+      <c r="D1332"/>
+      <c r="E1332"/>
+      <c r="F1332"/>
+      <c r="G1332"/>
+    </row>
+    <row r="1333">
+      <c r="A1333"/>
+      <c r="B1333" t="s">
+        <v>2132</v>
+      </c>
+      <c r="C1333" t="s">
+        <v>2133</v>
+      </c>
+      <c r="D1333"/>
+      <c r="E1333"/>
+      <c r="F1333"/>
+      <c r="G1333"/>
+    </row>
+    <row r="1334">
+      <c r="A1334"/>
+      <c r="B1334" t="s">
+        <v>2134</v>
+      </c>
+      <c r="C1334" t="s">
+        <v>2135</v>
+      </c>
+      <c r="D1334"/>
+      <c r="E1334"/>
+      <c r="F1334"/>
+      <c r="G1334"/>
+    </row>
+    <row r="1335">
+      <c r="A1335"/>
+      <c r="B1335"/>
+      <c r="C1335"/>
+      <c r="D1335"/>
+      <c r="E1335"/>
+      <c r="F1335"/>
+      <c r="G1335"/>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="s">
+        <v>2136</v>
+      </c>
+      <c r="B1336" t="s">
+        <v>2137</v>
+      </c>
+      <c r="C1336" t="s">
+        <v>2137</v>
+      </c>
+      <c r="D1336"/>
+      <c r="E1336"/>
+      <c r="F1336"/>
+      <c r="G1336"/>
+    </row>
+    <row r="1337">
+      <c r="A1337"/>
+      <c r="B1337" t="s">
+        <v>2138</v>
+      </c>
+      <c r="C1337" t="s">
+        <v>2138</v>
+      </c>
+      <c r="D1337"/>
+      <c r="E1337"/>
+      <c r="F1337"/>
+      <c r="G1337"/>
+    </row>
+    <row r="1338">
+      <c r="A1338"/>
+      <c r="B1338" t="s">
+        <v>2139</v>
+      </c>
+      <c r="C1338" t="s">
+        <v>2139</v>
+      </c>
+      <c r="D1338"/>
+      <c r="E1338"/>
+      <c r="F1338"/>
+      <c r="G1338"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
feat: load snapshot pseudonymization rule sources refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="table_description" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="snapshot_extensions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2149" uniqueCount="2149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2164" uniqueCount="2164">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -6468,6 +6469,51 @@
   </si>
   <si>
     <t xml:space="preserve">encounter_id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dieses Blatt beschreibt Snapshot-spezifische Anreicherungsspalten. Diese Spalten werden nicht beim normalen Toolchain-DB-Init erzeugt, sondern nur beim Aufbau pseudonymisierter Snapshot-DBs ergänzt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Snapshot-Prozess liest dieses Blatt zusätzlich zur normalen Table Description; operative Generatoren sollen es ignorieren.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TABLE_NAME</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLUMN_DESCRIPTION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COLUMN_TYPE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">observation</t>
+  </si>
+  <si>
+    <t xml:space="preserve">value_in_reference_unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Wert in Referenzeinheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">double precision</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep</t>
+  </si>
+  <si>
+    <t xml:space="preserve">reference_unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referenzeinheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">varchar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">primary_loinc_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Primary LOINC Code</t>
   </si>
 </sst>
 </file>
@@ -27021,4 +27067,117 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>2149</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2150</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+    </row>
+    <row r="4">
+      <c r="A4"/>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B5" t="s">
+        <v>6</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2152</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2153</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B6" t="s">
+        <v>2155</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2156</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2157</v>
+      </c>
+      <c r="E6" t="s">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2159</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2160</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2161</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2158</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2162</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2163</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2161</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2158</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add pseudonym mapping support refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2164" uniqueCount="2164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="2168">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -6514,6 +6514,18 @@
   </si>
   <si>
     <t xml:space="preserve">Primary LOINC Code</t>
+  </si>
+  <si>
+    <t>Dieses Blatt beschreibt Snapshot-spezifische Anreicherungsspalten.</t>
+  </si>
+  <si>
+    <t>Diese Spalten werden nicht beim normalen Toolchain-DB-Init erzeugt.</t>
+  </si>
+  <si>
+    <t>Der Snapshot-Prozess liest dieses Blatt zusätzlich zur normalen Table Description.</t>
+  </si>
+  <si>
+    <t>Operative Generatoren sollen dieses Blatt ignorieren.</t>
   </si>
 </sst>
 </file>
@@ -27070,114 +27082,132 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1"/>
-      <c r="C1"/>
-      <c r="D1"/>
-      <c r="E1"/>
+      <c r="B1" s="1"/>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
+      <c r="E1" s="1"/>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>2149</v>
-      </c>
-      <c r="B2"/>
-      <c r="C2"/>
-      <c r="D2"/>
-      <c r="E2"/>
+      <c r="A2" s="1" t="s">
+        <v>2164</v>
+      </c>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
     </row>
     <row r="3">
-      <c r="A3" t="s">
-        <v>2150</v>
-      </c>
-      <c r="B3"/>
-      <c r="C3"/>
-      <c r="D3"/>
-      <c r="E3"/>
+      <c r="A3" s="1" t="s">
+        <v>2165</v>
+      </c>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="1"/>
     </row>
     <row r="4">
-      <c r="A4"/>
-      <c r="B4"/>
-      <c r="C4"/>
-      <c r="D4"/>
-      <c r="E4"/>
+      <c r="A4" s="1" t="s">
+        <v>2166</v>
+      </c>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1"/>
+      <c r="D4" s="1"/>
+      <c r="E4" s="1"/>
     </row>
     <row r="5">
-      <c r="A5" t="s">
+      <c r="A5" s="1" t="s">
+        <v>2167</v>
+      </c>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1"/>
+      <c r="D5" s="1"/>
+      <c r="E5" s="1"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1"/>
+      <c r="B6" s="1"/>
+      <c r="C6" s="1"/>
+      <c r="D6" s="1"/>
+      <c r="E6" s="1"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
         <v>2151</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C7" s="1" t="s">
         <v>2152</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D7" s="1" t="s">
         <v>2153</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E7" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="s">
+    <row r="8">
+      <c r="A8" s="1" t="s">
         <v>2154</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" s="1" t="s">
         <v>2155</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C8" s="1" t="s">
         <v>2156</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D8" s="1" t="s">
         <v>2157</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E8" s="1" t="s">
         <v>2158</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="s">
+    <row r="9">
+      <c r="A9" s="1" t="s">
         <v>2154</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B9" s="1" t="s">
         <v>2159</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C9" s="1" t="s">
         <v>2160</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D9" s="1" t="s">
         <v>2161</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E9" s="1" t="s">
         <v>2158</v>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="s">
+    <row r="10">
+      <c r="A10" s="1" t="s">
         <v>2154</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B10" s="1" t="s">
         <v>2162</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C10" s="1" t="s">
         <v>2163</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D10" s="1" t="s">
         <v>2161</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E10" s="1" t="s">
         <v>2158</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" ns2:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: support table description extensions refs #1264
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -7,13 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="table_description" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="snapshot_extensions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="snapshot_extension" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2168" uniqueCount="2168">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="2182">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -6465,16 +6465,25 @@
     <t xml:space="preserve">ward_name</t>
   </si>
   <si>
+    <t xml:space="preserve">varchar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keep</t>
+  </si>
+  <si>
     <t xml:space="preserve">patient_id</t>
   </si>
   <si>
     <t xml:space="preserve">encounter_id</t>
   </si>
   <si>
-    <t xml:space="preserve">Dieses Blatt beschreibt Snapshot-spezifische Anreicherungsspalten. Diese Spalten werden nicht beim normalen Toolchain-DB-Init erzeugt, sondern nur beim Aufbau pseudonymisierter Snapshot-DBs ergänzt.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Der Snapshot-Prozess liest dieses Blatt zusätzlich zur normalen Table Description; operative Generatoren sollen es ignorieren.</t>
+    <t xml:space="preserve">Dieses Blatt beschreibt Snapshot-spezifische Anreicherungsspalten.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Diese Spalten werden nicht beim normalen Toolchain-DB-Init erzeugt.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Der Snapshot-Prozess liest dieses Blatt zusätzlich zur normalen Table Description.</t>
   </si>
   <si>
     <t xml:space="preserve">TABLE_NAME</t>
@@ -6486,46 +6495,79 @@
     <t xml:space="preserve">COLUMN_TYPE</t>
   </si>
   <si>
+    <t xml:space="preserve">medicationrequest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medreq_medication_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Codesystem der referenzierten Medication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medreq_medication_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Code der referenzierten Medication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medicationadministration</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medadm_medication_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medadm_medication_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medicationstatement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medstat_medication_system</t>
+  </si>
+  <si>
+    <t xml:space="preserve">medstat_medication_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fall</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fall_age_at_admission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alter bei Aufnahme des Falls in abgeschlossenen Jahren</t>
+  </si>
+  <si>
+    <t xml:space="preserve">encounter</t>
+  </si>
+  <si>
+    <t xml:space="preserve">enc_age_at_admission</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alter bei Beginn des Encounters in abgeschlossenen Jahren</t>
+  </si>
+  <si>
     <t xml:space="preserve">observation</t>
   </si>
   <si>
     <t xml:space="preserve">value_in_reference_unit</t>
   </si>
   <si>
-    <t xml:space="preserve">Wert in Referenzeinheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">double precision</t>
-  </si>
-  <si>
-    <t xml:space="preserve">keep</t>
+    <t xml:space="preserve">Observation-Wert in der Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">double</t>
   </si>
   <si>
     <t xml:space="preserve">reference_unit</t>
   </si>
   <si>
-    <t xml:space="preserve">Referenzeinheit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">varchar</t>
+    <t xml:space="preserve">Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
   </si>
   <si>
     <t xml:space="preserve">primary_loinc_code</t>
   </si>
   <si>
-    <t xml:space="preserve">Primary LOINC Code</t>
-  </si>
-  <si>
-    <t>Dieses Blatt beschreibt Snapshot-spezifische Anreicherungsspalten.</t>
-  </si>
-  <si>
-    <t>Diese Spalten werden nicht beim normalen Toolchain-DB-Init erzeugt.</t>
-  </si>
-  <si>
-    <t>Der Snapshot-Prozess liest dieses Blatt zusätzlich zur normalen Table Description.</t>
-  </si>
-  <si>
-    <t>Operative Generatoren sollen dieses Blatt ignorieren.</t>
+    <t xml:space="preserve">Primärer LOINC aus der LOINC-Mapping-Tabelle</t>
   </si>
 </sst>
 </file>
@@ -27022,58 +27064,60 @@
       <c r="H1335"/>
     </row>
     <row r="1336">
-      <c r="A1336"/>
-      <c r="B1336"/>
-      <c r="C1336"/>
+      <c r="A1336" t="s">
+        <v>2145</v>
+      </c>
+      <c r="B1336" t="s">
+        <v>2146</v>
+      </c>
+      <c r="C1336" t="s">
+        <v>2146</v>
+      </c>
       <c r="D1336"/>
-      <c r="E1336"/>
+      <c r="E1336" t="s">
+        <v>2147</v>
+      </c>
       <c r="F1336"/>
       <c r="G1336"/>
-      <c r="H1336"/>
+      <c r="H1336" t="s">
+        <v>2148</v>
+      </c>
     </row>
     <row r="1337">
-      <c r="A1337" t="s">
-        <v>2145</v>
-      </c>
+      <c r="A1337"/>
       <c r="B1337" t="s">
-        <v>2146</v>
+        <v>2149</v>
       </c>
       <c r="C1337" t="s">
-        <v>2146</v>
+        <v>2149</v>
       </c>
       <c r="D1337"/>
-      <c r="E1337"/>
+      <c r="E1337" t="s">
+        <v>2147</v>
+      </c>
       <c r="F1337"/>
       <c r="G1337"/>
-      <c r="H1337"/>
+      <c r="H1337" t="s">
+        <v>16</v>
+      </c>
     </row>
     <row r="1338">
       <c r="A1338"/>
       <c r="B1338" t="s">
+        <v>2150</v>
+      </c>
+      <c r="C1338" t="s">
+        <v>2150</v>
+      </c>
+      <c r="D1338"/>
+      <c r="E1338" t="s">
         <v>2147</v>
       </c>
-      <c r="C1338" t="s">
-        <v>2147</v>
-      </c>
-      <c r="D1338"/>
-      <c r="E1338"/>
       <c r="F1338"/>
       <c r="G1338"/>
-      <c r="H1338"/>
-    </row>
-    <row r="1339">
-      <c r="A1339"/>
-      <c r="B1339" t="s">
-        <v>2148</v>
-      </c>
-      <c r="C1339" t="s">
-        <v>2148</v>
-      </c>
-      <c r="D1339"/>
-      <c r="E1339"/>
-      <c r="F1339"/>
-      <c r="G1339"/>
-      <c r="H1339"/>
+      <c r="H1338" t="s">
+        <v>16</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -27082,132 +27126,259 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:ns2="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ns1:Ignorable="x14ac xr xr2 xr3">
-  <dimension ref="A1:E10"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
+      <c r="B1"/>
+      <c r="C1"/>
+      <c r="D1"/>
+      <c r="E1"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>2151</v>
+      </c>
+      <c r="B2"/>
+      <c r="C2"/>
+      <c r="D2"/>
+      <c r="E2"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>2152</v>
+      </c>
+      <c r="B3"/>
+      <c r="C3"/>
+      <c r="D3"/>
+      <c r="E3"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>2153</v>
+      </c>
+      <c r="B4"/>
+      <c r="C4"/>
+      <c r="D4"/>
+      <c r="E4"/>
+    </row>
+    <row r="5">
+      <c r="A5"/>
+      <c r="B5"/>
+      <c r="C5"/>
+      <c r="D5"/>
+      <c r="E5"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>2154</v>
+      </c>
+      <c r="B6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2155</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2156</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B7" t="s">
+        <v>2158</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2159</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E7" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>2157</v>
+      </c>
+      <c r="B8" t="s">
+        <v>2160</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2161</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E8" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B9" t="s">
+        <v>2163</v>
+      </c>
+      <c r="C9" t="s">
+        <v>2159</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E9" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>2162</v>
+      </c>
+      <c r="B10" t="s">
         <v>2164</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="1" t="s">
+      <c r="C10" t="s">
+        <v>2161</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E10" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
         <v>2165</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="1" t="s">
+      <c r="B11" t="s">
         <v>2166</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="1"/>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="1" t="s">
+      <c r="C11" t="s">
+        <v>2159</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E11" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>2165</v>
+      </c>
+      <c r="B12" t="s">
         <v>2167</v>
       </c>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="1"/>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="s">
-        <v>2151</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>2153</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="s">
-        <v>2154</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>2155</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>2156</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>2157</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>2158</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="s">
-        <v>2154</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>2159</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>2160</v>
-      </c>
-      <c r="D9" s="1" t="s">
+      <c r="C12" t="s">
         <v>2161</v>
       </c>
-      <c r="E9" s="1" t="s">
-        <v>2158</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="s">
-        <v>2154</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>2162</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>2163</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>2161</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>2158</v>
+      <c r="D12" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E12" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>2168</v>
+      </c>
+      <c r="B13" t="s">
+        <v>2169</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2170</v>
+      </c>
+      <c r="D13" t="s">
+        <v>104</v>
+      </c>
+      <c r="E13" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B14" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2173</v>
+      </c>
+      <c r="D14" t="s">
+        <v>104</v>
+      </c>
+      <c r="E14" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B15" t="s">
+        <v>2175</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2176</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2177</v>
+      </c>
+      <c r="E15" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B16" t="s">
+        <v>2178</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2179</v>
+      </c>
+      <c r="D16" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E16" t="s">
+        <v>2148</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B17" t="s">
+        <v>2180</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2181</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2147</v>
+      </c>
+      <c r="E17" t="s">
+        <v>2148</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" ns2:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: keep structural table description rows empty refs #1351
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -8337,9 +8337,7 @@
       <c r="E89"/>
       <c r="F89"/>
       <c r="G89"/>
-      <c r="H89" t="s">
-        <v>19</v>
-      </c>
+      <c r="H89"/>
     </row>
     <row r="90">
       <c r="A90" t="s">
@@ -8713,9 +8711,7 @@
       <c r="E112"/>
       <c r="F112"/>
       <c r="G112"/>
-      <c r="H112" t="s">
-        <v>19</v>
-      </c>
+      <c r="H112"/>
     </row>
     <row r="113">
       <c r="A113" t="s">
@@ -10755,9 +10751,7 @@
       <c r="E238"/>
       <c r="F238"/>
       <c r="G238"/>
-      <c r="H238" t="s">
-        <v>19</v>
-      </c>
+      <c r="H238"/>
     </row>
     <row r="239">
       <c r="A239" t="s">
@@ -11783,9 +11777,7 @@
       <c r="E301"/>
       <c r="F301"/>
       <c r="G301"/>
-      <c r="H301" t="s">
-        <v>19</v>
-      </c>
+      <c r="H301"/>
     </row>
     <row r="302">
       <c r="A302" t="s">
@@ -15715,9 +15707,7 @@
       <c r="E542"/>
       <c r="F542"/>
       <c r="G542"/>
-      <c r="H542" t="s">
-        <v>19</v>
-      </c>
+      <c r="H542"/>
     </row>
     <row r="543">
       <c r="A543" t="s">
@@ -17661,9 +17651,7 @@
       <c r="E662"/>
       <c r="F662"/>
       <c r="G662"/>
-      <c r="H662" t="s">
-        <v>19</v>
-      </c>
+      <c r="H662"/>
     </row>
     <row r="663">
       <c r="A663" t="s">
@@ -21341,9 +21329,7 @@
       <c r="E887"/>
       <c r="F887"/>
       <c r="G887"/>
-      <c r="H887" t="s">
-        <v>19</v>
-      </c>
+      <c r="H887"/>
     </row>
     <row r="888">
       <c r="A888" t="s">
@@ -23673,9 +23659,7 @@
       <c r="E1031"/>
       <c r="F1031"/>
       <c r="G1031"/>
-      <c r="H1031" t="s">
-        <v>19</v>
-      </c>
+      <c r="H1031"/>
     </row>
     <row r="1032">
       <c r="A1032" t="s">
@@ -24497,9 +24481,7 @@
       <c r="E1082"/>
       <c r="F1082"/>
       <c r="G1082"/>
-      <c r="H1082" t="s">
-        <v>19</v>
-      </c>
+      <c r="H1082"/>
     </row>
     <row r="1083">
       <c r="A1083" t="s">
@@ -25607,9 +25589,7 @@
       <c r="E1151"/>
       <c r="F1151"/>
       <c r="G1151"/>
-      <c r="H1151" t="s">
-        <v>19</v>
-      </c>
+      <c r="H1151"/>
     </row>
     <row r="1152">
       <c r="A1152" t="s">
@@ -26883,9 +26863,7 @@
       <c r="E1230"/>
       <c r="F1230"/>
       <c r="G1230"/>
-      <c r="H1230" t="s">
-        <v>19</v>
-      </c>
+      <c r="H1230"/>
     </row>
     <row r="1231">
       <c r="A1231" t="s">
@@ -28217,9 +28195,7 @@
       <c r="E1312"/>
       <c r="F1312"/>
       <c r="G1312"/>
-      <c r="H1312" t="s">
-        <v>19</v>
-      </c>
+      <c r="H1312"/>
     </row>
     <row r="1313">
       <c r="A1313" t="s">

</xml_diff>

<commit_message>
Improve snapshot analysis value fallback refs #1351
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2182" uniqueCount="2182">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="2184">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -6549,25 +6549,31 @@
     <t xml:space="preserve">observation</t>
   </si>
   <si>
-    <t xml:space="preserve">value_in_reference_unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Observation-Wert in der Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
+    <t xml:space="preserve">analysis_loinc_code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOINC-Code für die Auswertung: primärer LOINC aus dem Mapping, sonst ursprünglicher LOINC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">analysis_unit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Einheit des Analysewerts: Referenzeinheit bei erfolgreicher Umrechnung, sonst ursprüngliche Einheit</t>
+  </si>
+  <si>
+    <t xml:space="preserve">analysis_value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Analysewert in der Analyse-Einheit: umgerechneter Wert, sonst ursprünglicher Observation-Wert</t>
   </si>
   <si>
     <t xml:space="preserve">double</t>
   </si>
   <si>
-    <t xml:space="preserve">reference_unit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Referenzeinheit aus der LOINC-Mapping-Tabelle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">primary_loinc_code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Primärer LOINC aus der LOINC-Mapping-Tabelle</t>
+    <t xml:space="preserve">analysis_value_status</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Status der Herkunft des Analysewerts und der verwendeten Einheit</t>
   </si>
 </sst>
 </file>
@@ -28847,7 +28853,7 @@
         <v>2176</v>
       </c>
       <c r="D15" t="s">
-        <v>2177</v>
+        <v>2148</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -28858,10 +28864,10 @@
         <v>2174</v>
       </c>
       <c r="B16" t="s">
+        <v>2177</v>
+      </c>
+      <c r="C16" t="s">
         <v>2178</v>
-      </c>
-      <c r="C16" t="s">
-        <v>2179</v>
       </c>
       <c r="D16" t="s">
         <v>2148</v>
@@ -28875,15 +28881,32 @@
         <v>2174</v>
       </c>
       <c r="B17" t="s">
+        <v>2179</v>
+      </c>
+      <c r="C17" t="s">
         <v>2180</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>2181</v>
       </c>
-      <c r="D17" t="s">
+      <c r="E17" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>2174</v>
+      </c>
+      <c r="B18" t="s">
+        <v>2182</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2183</v>
+      </c>
+      <c r="D18" t="s">
         <v>2148</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E18" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Redact unapproved FHIR identifiers by default refs #1379
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -96,8 +96,11 @@
     <t xml:space="preserve">identifier/use</t>
   </si>
   <si>
-    <t xml:space="preserve">redactIf(type.coding.system == "http://fhir.de/CodeSystem/identifier-type-de-basis" &amp; type.coding.code in ["GKV", "PKV", "KVZ10"]);
-keep</t>
+    <t xml:space="preserve">keepIf(type.coding.system == "http://terminology.hl7.org/CodeSystem/v2-0203" &amp; type.coding.code == "VN");
+keepIf(type.coding.system == "http://terminology.hl7.org/CodeSystem/v2-0203" &amp; type.coding.code == "MR");
+keepIf(type.coding.system == "http://terminology.hl7.org/CodeSystem/v3-ObservationValue" &amp; type.coding.code == "PSEUDED");
+keepIf(type.coding.system == "http://terminology.hl7.org/CodeSystem/v3-ObservationValue" &amp; type.coding.code == "ANONYED");
+redact</t>
   </si>
   <si>
     <t xml:space="preserve">enc_identifier_type_system</t>
@@ -7087,7 +7090,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="12" ht="32" customHeight="1">
+    <row r="12" ht="77" customHeight="1">
       <c r="A12" s="1"/>
       <c r="B12" s="1" t="s">
         <v>25</v>
@@ -7103,7 +7106,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" ht="32" customHeight="1">
+    <row r="13" ht="77" customHeight="1">
       <c r="A13" s="1"/>
       <c r="B13" s="1" t="s">
         <v>28</v>
@@ -7119,7 +7122,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="14" ht="32" customHeight="1">
+    <row r="14" ht="77" customHeight="1">
       <c r="A14" s="1"/>
       <c r="B14" s="1" t="s">
         <v>30</v>
@@ -7135,7 +7138,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" ht="32" customHeight="1">
+    <row r="15" ht="77" customHeight="1">
       <c r="A15" s="1"/>
       <c r="B15" s="1" t="s">
         <v>32</v>
@@ -7151,7 +7154,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="16" ht="32" customHeight="1">
+    <row r="16" ht="77" customHeight="1">
       <c r="A16" s="1"/>
       <c r="B16" s="1" t="s">
         <v>34</v>
@@ -7167,7 +7170,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="17" ht="32" customHeight="1">
+    <row r="17" ht="77" customHeight="1">
       <c r="A17" s="1"/>
       <c r="B17" s="1" t="s">
         <v>36</v>
@@ -7183,7 +7186,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="18" ht="32" customHeight="1">
+    <row r="18" ht="77" customHeight="1">
       <c r="A18" s="1"/>
       <c r="B18" s="1" t="s">
         <v>38</v>
@@ -7215,7 +7218,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="20" ht="32" customHeight="1">
+    <row r="20" ht="77" customHeight="1">
       <c r="A20" s="1"/>
       <c r="B20" s="1" t="s">
         <v>43</v>
@@ -7233,7 +7236,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
+    <row r="21" ht="77" customHeight="1">
       <c r="A21" s="1"/>
       <c r="B21" s="1" t="s">
         <v>45</v>
@@ -8413,7 +8416,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="94" ht="32" customHeight="1">
+    <row r="94" ht="77" customHeight="1">
       <c r="A94" s="1"/>
       <c r="B94" s="1" t="s">
         <v>191</v>
@@ -8429,7 +8432,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="95" ht="32" customHeight="1">
+    <row r="95" ht="77" customHeight="1">
       <c r="A95" s="1"/>
       <c r="B95" s="1" t="s">
         <v>192</v>
@@ -8445,7 +8448,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="96" ht="32" customHeight="1">
+    <row r="96" ht="77" customHeight="1">
       <c r="A96" s="1"/>
       <c r="B96" s="1" t="s">
         <v>193</v>
@@ -8461,7 +8464,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="97" ht="32" customHeight="1">
+    <row r="97" ht="77" customHeight="1">
       <c r="A97" s="1"/>
       <c r="B97" s="1" t="s">
         <v>194</v>
@@ -8477,7 +8480,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="98" ht="32" customHeight="1">
+    <row r="98" ht="77" customHeight="1">
       <c r="A98" s="1"/>
       <c r="B98" s="1" t="s">
         <v>195</v>
@@ -8493,7 +8496,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="99" ht="32" customHeight="1">
+    <row r="99" ht="77" customHeight="1">
       <c r="A99" s="1"/>
       <c r="B99" s="1" t="s">
         <v>196</v>
@@ -8509,7 +8512,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="100" ht="32" customHeight="1">
+    <row r="100" ht="77" customHeight="1">
       <c r="A100" s="1"/>
       <c r="B100" s="1" t="s">
         <v>197</v>
@@ -8541,7 +8544,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="102" ht="32" customHeight="1">
+    <row r="102" ht="77" customHeight="1">
       <c r="A102" s="1"/>
       <c r="B102" s="1" t="s">
         <v>199</v>
@@ -8559,7 +8562,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="103" ht="32" customHeight="1">
+    <row r="103" ht="77" customHeight="1">
       <c r="A103" s="1"/>
       <c r="B103" s="1" t="s">
         <v>200</v>
@@ -8787,7 +8790,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="117" ht="32" customHeight="1">
+    <row r="117" ht="77" customHeight="1">
       <c r="A117" s="1"/>
       <c r="B117" s="1" t="s">
         <v>225</v>
@@ -8803,7 +8806,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="118" ht="32" customHeight="1">
+    <row r="118" ht="77" customHeight="1">
       <c r="A118" s="1"/>
       <c r="B118" s="1" t="s">
         <v>226</v>
@@ -8819,7 +8822,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="119" ht="32" customHeight="1">
+    <row r="119" ht="77" customHeight="1">
       <c r="A119" s="1"/>
       <c r="B119" s="1" t="s">
         <v>227</v>
@@ -8835,7 +8838,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="120" ht="32" customHeight="1">
+    <row r="120" ht="77" customHeight="1">
       <c r="A120" s="1"/>
       <c r="B120" s="1" t="s">
         <v>228</v>
@@ -8851,7 +8854,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="121" ht="32" customHeight="1">
+    <row r="121" ht="77" customHeight="1">
       <c r="A121" s="1"/>
       <c r="B121" s="1" t="s">
         <v>229</v>
@@ -8867,7 +8870,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="122" ht="32" customHeight="1">
+    <row r="122" ht="77" customHeight="1">
       <c r="A122" s="1"/>
       <c r="B122" s="1" t="s">
         <v>230</v>
@@ -8883,7 +8886,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="123" ht="32" customHeight="1">
+    <row r="123" ht="77" customHeight="1">
       <c r="A123" s="1"/>
       <c r="B123" s="1" t="s">
         <v>231</v>
@@ -8915,7 +8918,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="125" ht="32" customHeight="1">
+    <row r="125" ht="77" customHeight="1">
       <c r="A125" s="1"/>
       <c r="B125" s="1" t="s">
         <v>233</v>
@@ -8933,7 +8936,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="126" ht="32" customHeight="1">
+    <row r="126" ht="77" customHeight="1">
       <c r="A126" s="1"/>
       <c r="B126" s="1" t="s">
         <v>234</v>
@@ -10827,7 +10830,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="243" ht="32" customHeight="1">
+    <row r="243" ht="77" customHeight="1">
       <c r="A243" s="1"/>
       <c r="B243" s="1" t="s">
         <v>462</v>
@@ -10843,7 +10846,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="244" ht="32" customHeight="1">
+    <row r="244" ht="77" customHeight="1">
       <c r="A244" s="1"/>
       <c r="B244" s="1" t="s">
         <v>463</v>
@@ -10859,7 +10862,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="245" ht="32" customHeight="1">
+    <row r="245" ht="77" customHeight="1">
       <c r="A245" s="1"/>
       <c r="B245" s="1" t="s">
         <v>464</v>
@@ -10875,7 +10878,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="246" ht="32" customHeight="1">
+    <row r="246" ht="77" customHeight="1">
       <c r="A246" s="1"/>
       <c r="B246" s="1" t="s">
         <v>465</v>
@@ -10891,7 +10894,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="247" ht="32" customHeight="1">
+    <row r="247" ht="77" customHeight="1">
       <c r="A247" s="1"/>
       <c r="B247" s="1" t="s">
         <v>466</v>
@@ -10907,7 +10910,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="248" ht="32" customHeight="1">
+    <row r="248" ht="77" customHeight="1">
       <c r="A248" s="1"/>
       <c r="B248" s="1" t="s">
         <v>467</v>
@@ -10923,7 +10926,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="249" ht="32" customHeight="1">
+    <row r="249" ht="77" customHeight="1">
       <c r="A249" s="1"/>
       <c r="B249" s="1" t="s">
         <v>468</v>
@@ -10955,7 +10958,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="251" ht="32" customHeight="1">
+    <row r="251" ht="77" customHeight="1">
       <c r="A251" s="1"/>
       <c r="B251" s="1" t="s">
         <v>470</v>
@@ -10973,7 +10976,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="252" ht="32" customHeight="1">
+    <row r="252" ht="77" customHeight="1">
       <c r="A252" s="1"/>
       <c r="B252" s="1" t="s">
         <v>471</v>
@@ -11853,7 +11856,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="306" ht="32" customHeight="1">
+    <row r="306" ht="77" customHeight="1">
       <c r="A306" s="1"/>
       <c r="B306" s="1" t="s">
         <v>568</v>
@@ -11869,7 +11872,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="307" ht="32" customHeight="1">
+    <row r="307" ht="77" customHeight="1">
       <c r="A307" s="1"/>
       <c r="B307" s="1" t="s">
         <v>569</v>
@@ -11885,7 +11888,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="308" ht="32" customHeight="1">
+    <row r="308" ht="77" customHeight="1">
       <c r="A308" s="1"/>
       <c r="B308" s="1" t="s">
         <v>570</v>
@@ -11901,7 +11904,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="309" ht="32" customHeight="1">
+    <row r="309" ht="77" customHeight="1">
       <c r="A309" s="1"/>
       <c r="B309" s="1" t="s">
         <v>571</v>
@@ -11917,7 +11920,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="310" ht="32" customHeight="1">
+    <row r="310" ht="77" customHeight="1">
       <c r="A310" s="1"/>
       <c r="B310" s="1" t="s">
         <v>572</v>
@@ -11933,7 +11936,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="311" ht="32" customHeight="1">
+    <row r="311" ht="77" customHeight="1">
       <c r="A311" s="1"/>
       <c r="B311" s="1" t="s">
         <v>573</v>
@@ -11949,7 +11952,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="312" ht="32" customHeight="1">
+    <row r="312" ht="77" customHeight="1">
       <c r="A312" s="1"/>
       <c r="B312" s="1" t="s">
         <v>574</v>
@@ -11981,7 +11984,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="314" ht="32" customHeight="1">
+    <row r="314" ht="77" customHeight="1">
       <c r="A314" s="1"/>
       <c r="B314" s="1" t="s">
         <v>576</v>
@@ -11999,7 +12002,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="315" ht="32" customHeight="1">
+    <row r="315" ht="77" customHeight="1">
       <c r="A315" s="1"/>
       <c r="B315" s="1" t="s">
         <v>577</v>
@@ -15783,7 +15786,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="547" ht="32" customHeight="1">
+    <row r="547" ht="77" customHeight="1">
       <c r="A547" s="1"/>
       <c r="B547" s="1" t="s">
         <v>1013</v>
@@ -15799,7 +15802,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="548" ht="32" customHeight="1">
+    <row r="548" ht="77" customHeight="1">
       <c r="A548" s="1"/>
       <c r="B548" s="1" t="s">
         <v>1014</v>
@@ -15815,7 +15818,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="549" ht="32" customHeight="1">
+    <row r="549" ht="77" customHeight="1">
       <c r="A549" s="1"/>
       <c r="B549" s="1" t="s">
         <v>1015</v>
@@ -15831,7 +15834,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="550" ht="32" customHeight="1">
+    <row r="550" ht="77" customHeight="1">
       <c r="A550" s="1"/>
       <c r="B550" s="1" t="s">
         <v>1016</v>
@@ -15847,7 +15850,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="551" ht="32" customHeight="1">
+    <row r="551" ht="77" customHeight="1">
       <c r="A551" s="1"/>
       <c r="B551" s="1" t="s">
         <v>1017</v>
@@ -15863,7 +15866,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="552" ht="32" customHeight="1">
+    <row r="552" ht="77" customHeight="1">
       <c r="A552" s="1"/>
       <c r="B552" s="1" t="s">
         <v>1018</v>
@@ -15879,7 +15882,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="553" ht="32" customHeight="1">
+    <row r="553" ht="77" customHeight="1">
       <c r="A553" s="1"/>
       <c r="B553" s="1" t="s">
         <v>1019</v>
@@ -15911,7 +15914,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="555" ht="32" customHeight="1">
+    <row r="555" ht="77" customHeight="1">
       <c r="A555" s="1"/>
       <c r="B555" s="1" t="s">
         <v>1021</v>
@@ -15929,7 +15932,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="556" ht="32" customHeight="1">
+    <row r="556" ht="77" customHeight="1">
       <c r="A556" s="1"/>
       <c r="B556" s="1" t="s">
         <v>1022</v>
@@ -17727,7 +17730,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="667" ht="32" customHeight="1">
+    <row r="667" ht="77" customHeight="1">
       <c r="A667" s="1"/>
       <c r="B667" s="1" t="s">
         <v>1178</v>
@@ -17743,7 +17746,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="668" ht="32" customHeight="1">
+    <row r="668" ht="77" customHeight="1">
       <c r="A668" s="1"/>
       <c r="B668" s="1" t="s">
         <v>1179</v>
@@ -17759,7 +17762,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="669" ht="32" customHeight="1">
+    <row r="669" ht="77" customHeight="1">
       <c r="A669" s="1"/>
       <c r="B669" s="1" t="s">
         <v>1180</v>
@@ -17775,7 +17778,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="670" ht="32" customHeight="1">
+    <row r="670" ht="77" customHeight="1">
       <c r="A670" s="1"/>
       <c r="B670" s="1" t="s">
         <v>1181</v>
@@ -17791,7 +17794,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="671" ht="32" customHeight="1">
+    <row r="671" ht="77" customHeight="1">
       <c r="A671" s="1"/>
       <c r="B671" s="1" t="s">
         <v>1182</v>
@@ -17807,7 +17810,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="672" ht="32" customHeight="1">
+    <row r="672" ht="77" customHeight="1">
       <c r="A672" s="1"/>
       <c r="B672" s="1" t="s">
         <v>1183</v>
@@ -17823,7 +17826,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="673" ht="32" customHeight="1">
+    <row r="673" ht="77" customHeight="1">
       <c r="A673" s="1"/>
       <c r="B673" s="1" t="s">
         <v>1184</v>
@@ -17855,7 +17858,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="675" ht="32" customHeight="1">
+    <row r="675" ht="77" customHeight="1">
       <c r="A675" s="1"/>
       <c r="B675" s="1" t="s">
         <v>1186</v>
@@ -17873,7 +17876,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="676" ht="32" customHeight="1">
+    <row r="676" ht="77" customHeight="1">
       <c r="A676" s="1"/>
       <c r="B676" s="1" t="s">
         <v>1187</v>
@@ -21405,7 +21408,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="892" ht="32" customHeight="1">
+    <row r="892" ht="77" customHeight="1">
       <c r="A892" s="1"/>
       <c r="B892" s="1" t="s">
         <v>1532</v>
@@ -21421,7 +21424,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="893" ht="32" customHeight="1">
+    <row r="893" ht="77" customHeight="1">
       <c r="A893" s="1"/>
       <c r="B893" s="1" t="s">
         <v>1533</v>
@@ -21437,7 +21440,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="894" ht="32" customHeight="1">
+    <row r="894" ht="77" customHeight="1">
       <c r="A894" s="1"/>
       <c r="B894" s="1" t="s">
         <v>1534</v>
@@ -21453,7 +21456,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="895" ht="32" customHeight="1">
+    <row r="895" ht="77" customHeight="1">
       <c r="A895" s="1"/>
       <c r="B895" s="1" t="s">
         <v>1535</v>
@@ -21469,7 +21472,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="896" ht="32" customHeight="1">
+    <row r="896" ht="77" customHeight="1">
       <c r="A896" s="1"/>
       <c r="B896" s="1" t="s">
         <v>1536</v>
@@ -21485,7 +21488,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="897" ht="32" customHeight="1">
+    <row r="897" ht="77" customHeight="1">
       <c r="A897" s="1"/>
       <c r="B897" s="1" t="s">
         <v>1537</v>
@@ -21501,7 +21504,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="898" ht="32" customHeight="1">
+    <row r="898" ht="77" customHeight="1">
       <c r="A898" s="1"/>
       <c r="B898" s="1" t="s">
         <v>1538</v>
@@ -21533,7 +21536,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="900" ht="32" customHeight="1">
+    <row r="900" ht="77" customHeight="1">
       <c r="A900" s="1"/>
       <c r="B900" s="1" t="s">
         <v>1540</v>
@@ -21551,7 +21554,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="901" ht="32" customHeight="1">
+    <row r="901" ht="77" customHeight="1">
       <c r="A901" s="1"/>
       <c r="B901" s="1" t="s">
         <v>1541</v>
@@ -23735,7 +23738,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="1036" ht="32" customHeight="1">
+    <row r="1036" ht="77" customHeight="1">
       <c r="A1036" s="1"/>
       <c r="B1036" s="1" t="s">
         <v>1764</v>
@@ -23751,7 +23754,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1037" ht="32" customHeight="1">
+    <row r="1037" ht="77" customHeight="1">
       <c r="A1037" s="1"/>
       <c r="B1037" s="1" t="s">
         <v>1765</v>
@@ -23767,7 +23770,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1038" ht="32" customHeight="1">
+    <row r="1038" ht="77" customHeight="1">
       <c r="A1038" s="1"/>
       <c r="B1038" s="1" t="s">
         <v>1766</v>
@@ -23783,7 +23786,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1039" ht="32" customHeight="1">
+    <row r="1039" ht="77" customHeight="1">
       <c r="A1039" s="1"/>
       <c r="B1039" s="1" t="s">
         <v>1767</v>
@@ -23799,7 +23802,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1040" ht="32" customHeight="1">
+    <row r="1040" ht="77" customHeight="1">
       <c r="A1040" s="1"/>
       <c r="B1040" s="1" t="s">
         <v>1768</v>
@@ -23815,7 +23818,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1041" ht="32" customHeight="1">
+    <row r="1041" ht="77" customHeight="1">
       <c r="A1041" s="1"/>
       <c r="B1041" s="1" t="s">
         <v>1769</v>
@@ -23831,7 +23834,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1042" ht="32" customHeight="1">
+    <row r="1042" ht="77" customHeight="1">
       <c r="A1042" s="1"/>
       <c r="B1042" s="1" t="s">
         <v>1770</v>
@@ -23863,7 +23866,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="1044" ht="32" customHeight="1">
+    <row r="1044" ht="77" customHeight="1">
       <c r="A1044" s="1"/>
       <c r="B1044" s="1" t="s">
         <v>1772</v>
@@ -23881,7 +23884,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1045" ht="32" customHeight="1">
+    <row r="1045" ht="77" customHeight="1">
       <c r="A1045" s="1"/>
       <c r="B1045" s="1" t="s">
         <v>1773</v>
@@ -24557,7 +24560,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="1087" ht="32" customHeight="1">
+    <row r="1087" ht="77" customHeight="1">
       <c r="A1087" s="1"/>
       <c r="B1087" s="1" t="s">
         <v>1822</v>
@@ -24573,7 +24576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1088" ht="32" customHeight="1">
+    <row r="1088" ht="77" customHeight="1">
       <c r="A1088" s="1"/>
       <c r="B1088" s="1" t="s">
         <v>1823</v>
@@ -24589,7 +24592,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1089" ht="32" customHeight="1">
+    <row r="1089" ht="77" customHeight="1">
       <c r="A1089" s="1"/>
       <c r="B1089" s="1" t="s">
         <v>1824</v>
@@ -24605,7 +24608,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1090" ht="32" customHeight="1">
+    <row r="1090" ht="77" customHeight="1">
       <c r="A1090" s="1"/>
       <c r="B1090" s="1" t="s">
         <v>1825</v>
@@ -24621,7 +24624,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1091" ht="32" customHeight="1">
+    <row r="1091" ht="77" customHeight="1">
       <c r="A1091" s="1"/>
       <c r="B1091" s="1" t="s">
         <v>1826</v>
@@ -24637,7 +24640,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1092" ht="32" customHeight="1">
+    <row r="1092" ht="77" customHeight="1">
       <c r="A1092" s="1"/>
       <c r="B1092" s="1" t="s">
         <v>1827</v>
@@ -24653,7 +24656,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1093" ht="32" customHeight="1">
+    <row r="1093" ht="77" customHeight="1">
       <c r="A1093" s="1"/>
       <c r="B1093" s="1" t="s">
         <v>1828</v>
@@ -24685,7 +24688,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="1095" ht="32" customHeight="1">
+    <row r="1095" ht="77" customHeight="1">
       <c r="A1095" s="1"/>
       <c r="B1095" s="1" t="s">
         <v>1830</v>
@@ -24703,7 +24706,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1096" ht="32" customHeight="1">
+    <row r="1096" ht="77" customHeight="1">
       <c r="A1096" s="1"/>
       <c r="B1096" s="1" t="s">
         <v>1831</v>
@@ -25665,7 +25668,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="1156" ht="32" customHeight="1">
+    <row r="1156" ht="77" customHeight="1">
       <c r="A1156" s="1"/>
       <c r="B1156" s="1" t="s">
         <v>1896</v>
@@ -25681,7 +25684,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1157" ht="32" customHeight="1">
+    <row r="1157" ht="77" customHeight="1">
       <c r="A1157" s="1"/>
       <c r="B1157" s="1" t="s">
         <v>1897</v>
@@ -25697,7 +25700,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1158" ht="32" customHeight="1">
+    <row r="1158" ht="77" customHeight="1">
       <c r="A1158" s="1"/>
       <c r="B1158" s="1" t="s">
         <v>1898</v>
@@ -25713,7 +25716,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1159" ht="32" customHeight="1">
+    <row r="1159" ht="77" customHeight="1">
       <c r="A1159" s="1"/>
       <c r="B1159" s="1" t="s">
         <v>1899</v>
@@ -25729,7 +25732,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1160" ht="32" customHeight="1">
+    <row r="1160" ht="77" customHeight="1">
       <c r="A1160" s="1"/>
       <c r="B1160" s="1" t="s">
         <v>1900</v>
@@ -25745,7 +25748,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1161" ht="32" customHeight="1">
+    <row r="1161" ht="77" customHeight="1">
       <c r="A1161" s="1"/>
       <c r="B1161" s="1" t="s">
         <v>1901</v>
@@ -25761,7 +25764,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1162" ht="32" customHeight="1">
+    <row r="1162" ht="77" customHeight="1">
       <c r="A1162" s="1"/>
       <c r="B1162" s="1" t="s">
         <v>1902</v>
@@ -25793,7 +25796,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="1164" ht="32" customHeight="1">
+    <row r="1164" ht="77" customHeight="1">
       <c r="A1164" s="1"/>
       <c r="B1164" s="1" t="s">
         <v>1904</v>
@@ -25811,7 +25814,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1165" ht="32" customHeight="1">
+    <row r="1165" ht="77" customHeight="1">
       <c r="A1165" s="1"/>
       <c r="B1165" s="1" t="s">
         <v>1905</v>
@@ -26939,7 +26942,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="1235" ht="32" customHeight="1">
+    <row r="1235" ht="77" customHeight="1">
       <c r="A1235" s="1"/>
       <c r="B1235" s="1" t="s">
         <v>1978</v>
@@ -26955,7 +26958,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1236" ht="32" customHeight="1">
+    <row r="1236" ht="77" customHeight="1">
       <c r="A1236" s="1"/>
       <c r="B1236" s="1" t="s">
         <v>1979</v>
@@ -26971,7 +26974,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1237" ht="32" customHeight="1">
+    <row r="1237" ht="77" customHeight="1">
       <c r="A1237" s="1"/>
       <c r="B1237" s="1" t="s">
         <v>1980</v>
@@ -26987,7 +26990,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1238" ht="32" customHeight="1">
+    <row r="1238" ht="77" customHeight="1">
       <c r="A1238" s="1"/>
       <c r="B1238" s="1" t="s">
         <v>1981</v>
@@ -27003,7 +27006,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1239" ht="32" customHeight="1">
+    <row r="1239" ht="77" customHeight="1">
       <c r="A1239" s="1"/>
       <c r="B1239" s="1" t="s">
         <v>1982</v>
@@ -27019,7 +27022,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1240" ht="32" customHeight="1">
+    <row r="1240" ht="77" customHeight="1">
       <c r="A1240" s="1"/>
       <c r="B1240" s="1" t="s">
         <v>1983</v>
@@ -27035,7 +27038,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1241" ht="32" customHeight="1">
+    <row r="1241" ht="77" customHeight="1">
       <c r="A1241" s="1"/>
       <c r="B1241" s="1" t="s">
         <v>1984</v>
@@ -27067,7 +27070,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="1243" ht="32" customHeight="1">
+    <row r="1243" ht="77" customHeight="1">
       <c r="A1243" s="1"/>
       <c r="B1243" s="1" t="s">
         <v>1986</v>
@@ -27085,7 +27088,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1244" ht="32" customHeight="1">
+    <row r="1244" ht="77" customHeight="1">
       <c r="A1244" s="1"/>
       <c r="B1244" s="1" t="s">
         <v>1987</v>
@@ -28271,7 +28274,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="1317" ht="32" customHeight="1">
+    <row r="1317" ht="77" customHeight="1">
       <c r="A1317" s="1"/>
       <c r="B1317" s="1" t="s">
         <v>2119</v>
@@ -28287,7 +28290,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1318" ht="32" customHeight="1">
+    <row r="1318" ht="77" customHeight="1">
       <c r="A1318" s="1"/>
       <c r="B1318" s="1" t="s">
         <v>2120</v>
@@ -28303,7 +28306,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1319" ht="32" customHeight="1">
+    <row r="1319" ht="77" customHeight="1">
       <c r="A1319" s="1"/>
       <c r="B1319" s="1" t="s">
         <v>2121</v>
@@ -28319,7 +28322,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1320" ht="32" customHeight="1">
+    <row r="1320" ht="77" customHeight="1">
       <c r="A1320" s="1"/>
       <c r="B1320" s="1" t="s">
         <v>2122</v>
@@ -28335,7 +28338,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1321" ht="32" customHeight="1">
+    <row r="1321" ht="77" customHeight="1">
       <c r="A1321" s="1"/>
       <c r="B1321" s="1" t="s">
         <v>2123</v>
@@ -28351,7 +28354,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1322" ht="32" customHeight="1">
+    <row r="1322" ht="77" customHeight="1">
       <c r="A1322" s="1"/>
       <c r="B1322" s="1" t="s">
         <v>2124</v>
@@ -28367,7 +28370,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1323" ht="32" customHeight="1">
+    <row r="1323" ht="77" customHeight="1">
       <c r="A1323" s="1"/>
       <c r="B1323" s="1" t="s">
         <v>2125</v>
@@ -28399,7 +28402,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="1325" ht="32" customHeight="1">
+    <row r="1325" ht="77" customHeight="1">
       <c r="A1325" s="1"/>
       <c r="B1325" s="1" t="s">
         <v>2127</v>
@@ -28417,7 +28420,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="1326" ht="32" customHeight="1">
+    <row r="1326" ht="77" customHeight="1">
       <c r="A1326" s="1"/>
       <c r="B1326" s="1" t="s">
         <v>2128</v>

</xml_diff>

<commit_message>
Protect unapproved Observation codes refs #1340
</commit_message>
<xml_diff>
--- a/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
+++ b/R-cds2db/cds2db/inst/extdata/Table_Description.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2184" uniqueCount="2184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2190" uniqueCount="2190">
   <si>
     <t xml:space="preserve">Hint</t>
   </si>
@@ -4725,12 +4725,24 @@
     <t xml:space="preserve">obs_code_code</t>
   </si>
   <si>
+    <t xml:space="preserve">keepIf(system in ["http://loinc.org", "http://snomed.info/sct"]);
+cryptoHash</t>
+  </si>
+  <si>
     <t xml:space="preserve">obs_code_display</t>
   </si>
   <si>
+    <t xml:space="preserve">keepIf(system in ["http://loinc.org", "http://snomed.info/sct"]);
+redact</t>
+  </si>
+  <si>
     <t xml:space="preserve">obs_code_text</t>
   </si>
   <si>
+    <t xml:space="preserve">keepIf(coding.system in ["http://loinc.org", "http://snomed.info/sct"]);
+redact</t>
+  </si>
+  <si>
     <t xml:space="preserve">obs_effectivedatetime</t>
   </si>
   <si>
@@ -4896,16 +4908,28 @@
     <t xml:space="preserve">valueCodeableConcept/coding/code</t>
   </si>
   <si>
+    <t xml:space="preserve">keepIf(system in ["http://fhir.de/CodeSystem/bfarm/atc", "http://fhir.de/CodeSystem/ifa/pzn", "http://snomed.info/sct", "http://fhir.de/CodeSystem/ask"]);
+cryptoHash</t>
+  </si>
+  <si>
     <t xml:space="preserve">obs_valuecodeableconcept_display</t>
   </si>
   <si>
     <t xml:space="preserve">valueCodeableConcept/coding/display</t>
   </si>
   <si>
+    <t xml:space="preserve">keepIf(system in ["http://fhir.de/CodeSystem/bfarm/atc", "http://fhir.de/CodeSystem/ifa/pzn", "http://snomed.info/sct", "http://fhir.de/CodeSystem/ask"]);
+redact</t>
+  </si>
+  <si>
     <t xml:space="preserve">obs_valuecodeableconcept_text</t>
   </si>
   <si>
     <t xml:space="preserve">valueCodeableConcept/text</t>
+  </si>
+  <si>
+    <t xml:space="preserve">keepIf(coding.system in ["http://fhir.de/CodeSystem/bfarm/atc", "http://fhir.de/CodeSystem/ifa/pzn", "http://snomed.info/sct", "http://fhir.de/CodeSystem/ask"]);
+redact</t>
   </si>
   <si>
     <t xml:space="preserve">obs_dataabsentreason_system</t>
@@ -21940,58 +21964,58 @@
         <v>19</v>
       </c>
     </row>
-    <row r="925">
-      <c r="A925"/>
-      <c r="B925" t="s">
+    <row r="925" ht="32" customHeight="1">
+      <c r="A925" s="1"/>
+      <c r="B925" s="1" t="s">
         <v>1565</v>
       </c>
-      <c r="C925" t="s">
+      <c r="C925" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="D925"/>
-      <c r="E925"/>
-      <c r="F925"/>
-      <c r="G925"/>
-      <c r="H925" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="926">
-      <c r="A926"/>
-      <c r="B926" t="s">
+      <c r="D925" s="1"/>
+      <c r="E925" s="1"/>
+      <c r="F925" s="1"/>
+      <c r="G925" s="1"/>
+      <c r="H925" s="2" t="s">
         <v>1566</v>
       </c>
-      <c r="C926" t="s">
+    </row>
+    <row r="926" ht="32" customHeight="1">
+      <c r="A926" s="1"/>
+      <c r="B926" s="1" t="s">
+        <v>1567</v>
+      </c>
+      <c r="C926" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="D926"/>
-      <c r="E926"/>
-      <c r="F926"/>
-      <c r="G926"/>
-      <c r="H926" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="927">
-      <c r="A927"/>
-      <c r="B927" t="s">
-        <v>1567</v>
-      </c>
-      <c r="C927" t="s">
+      <c r="D926" s="1"/>
+      <c r="E926" s="1"/>
+      <c r="F926" s="1"/>
+      <c r="G926" s="1"/>
+      <c r="H926" s="2" t="s">
+        <v>1568</v>
+      </c>
+    </row>
+    <row r="927" ht="32" customHeight="1">
+      <c r="A927" s="1"/>
+      <c r="B927" s="1" t="s">
+        <v>1569</v>
+      </c>
+      <c r="C927" s="1" t="s">
         <v>289</v>
       </c>
-      <c r="D927"/>
-      <c r="E927"/>
-      <c r="F927"/>
-      <c r="G927"/>
-      <c r="H927" t="s">
-        <v>19</v>
+      <c r="D927" s="1"/>
+      <c r="E927" s="1"/>
+      <c r="F927" s="1"/>
+      <c r="G927" s="1"/>
+      <c r="H927" s="2" t="s">
+        <v>1570</v>
       </c>
     </row>
     <row r="928">
       <c r="A928"/>
       <c r="B928" t="s">
-        <v>1568</v>
+        <v>1571</v>
       </c>
       <c r="C928" t="s">
         <v>1058</v>
@@ -22009,10 +22033,10 @@
     <row r="929">
       <c r="A929"/>
       <c r="B929" t="s">
-        <v>1569</v>
+        <v>1572</v>
       </c>
       <c r="C929" t="s">
-        <v>1570</v>
+        <v>1573</v>
       </c>
       <c r="D929"/>
       <c r="E929" t="s">
@@ -22027,10 +22051,10 @@
     <row r="930">
       <c r="A930"/>
       <c r="B930" t="s">
-        <v>1571</v>
+        <v>1574</v>
       </c>
       <c r="C930" t="s">
-        <v>1572</v>
+        <v>1575</v>
       </c>
       <c r="D930"/>
       <c r="E930" t="s">
@@ -22045,10 +22069,10 @@
     <row r="931">
       <c r="A931"/>
       <c r="B931" t="s">
-        <v>1573</v>
+        <v>1576</v>
       </c>
       <c r="C931" t="s">
-        <v>1574</v>
+        <v>1577</v>
       </c>
       <c r="D931"/>
       <c r="E931"/>
@@ -22061,10 +22085,10 @@
     <row r="932">
       <c r="A932"/>
       <c r="B932" t="s">
-        <v>1575</v>
+        <v>1578</v>
       </c>
       <c r="C932" t="s">
-        <v>1576</v>
+        <v>1579</v>
       </c>
       <c r="D932"/>
       <c r="E932"/>
@@ -22077,10 +22101,10 @@
     <row r="933">
       <c r="A933"/>
       <c r="B933" t="s">
-        <v>1577</v>
+        <v>1580</v>
       </c>
       <c r="C933" t="s">
-        <v>1578</v>
+        <v>1581</v>
       </c>
       <c r="D933"/>
       <c r="E933"/>
@@ -22093,10 +22117,10 @@
     <row r="934">
       <c r="A934"/>
       <c r="B934" t="s">
-        <v>1579</v>
+        <v>1582</v>
       </c>
       <c r="C934" t="s">
-        <v>1580</v>
+        <v>1583</v>
       </c>
       <c r="D934"/>
       <c r="E934" t="s">
@@ -22111,10 +22135,10 @@
     <row r="935">
       <c r="A935"/>
       <c r="B935" t="s">
-        <v>1581</v>
+        <v>1584</v>
       </c>
       <c r="C935" t="s">
-        <v>1582</v>
+        <v>1585</v>
       </c>
       <c r="D935"/>
       <c r="E935"/>
@@ -22127,10 +22151,10 @@
     <row r="936">
       <c r="A936"/>
       <c r="B936" t="s">
-        <v>1583</v>
+        <v>1586</v>
       </c>
       <c r="C936" t="s">
-        <v>1584</v>
+        <v>1587</v>
       </c>
       <c r="D936"/>
       <c r="E936"/>
@@ -22143,10 +22167,10 @@
     <row r="937">
       <c r="A937"/>
       <c r="B937" t="s">
-        <v>1585</v>
+        <v>1588</v>
       </c>
       <c r="C937" t="s">
-        <v>1586</v>
+        <v>1589</v>
       </c>
       <c r="D937"/>
       <c r="E937"/>
@@ -22159,10 +22183,10 @@
     <row r="938">
       <c r="A938"/>
       <c r="B938" t="s">
-        <v>1587</v>
+        <v>1590</v>
       </c>
       <c r="C938" t="s">
-        <v>1588</v>
+        <v>1591</v>
       </c>
       <c r="D938"/>
       <c r="E938" t="s">
@@ -22177,10 +22201,10 @@
     <row r="939">
       <c r="A939"/>
       <c r="B939" t="s">
-        <v>1589</v>
+        <v>1592</v>
       </c>
       <c r="C939" t="s">
-        <v>1590</v>
+        <v>1593</v>
       </c>
       <c r="D939"/>
       <c r="E939"/>
@@ -22193,10 +22217,10 @@
     <row r="940">
       <c r="A940"/>
       <c r="B940" t="s">
-        <v>1591</v>
+        <v>1594</v>
       </c>
       <c r="C940" t="s">
-        <v>1592</v>
+        <v>1595</v>
       </c>
       <c r="D940"/>
       <c r="E940"/>
@@ -22209,10 +22233,10 @@
     <row r="941">
       <c r="A941"/>
       <c r="B941" t="s">
-        <v>1593</v>
+        <v>1596</v>
       </c>
       <c r="C941" t="s">
-        <v>1594</v>
+        <v>1597</v>
       </c>
       <c r="D941"/>
       <c r="E941"/>
@@ -22225,10 +22249,10 @@
     <row r="942">
       <c r="A942"/>
       <c r="B942" t="s">
-        <v>1595</v>
+        <v>1598</v>
       </c>
       <c r="C942" t="s">
-        <v>1596</v>
+        <v>1599</v>
       </c>
       <c r="D942"/>
       <c r="E942"/>
@@ -22241,10 +22265,10 @@
     <row r="943">
       <c r="A943"/>
       <c r="B943" t="s">
-        <v>1597</v>
+        <v>1600</v>
       </c>
       <c r="C943" t="s">
-        <v>1598</v>
+        <v>1601</v>
       </c>
       <c r="D943"/>
       <c r="E943" t="s">
@@ -22259,10 +22283,10 @@
     <row r="944">
       <c r="A944"/>
       <c r="B944" t="s">
-        <v>1599</v>
+        <v>1602</v>
       </c>
       <c r="C944" t="s">
-        <v>1600</v>
+        <v>1603</v>
       </c>
       <c r="D944"/>
       <c r="E944"/>
@@ -22275,10 +22299,10 @@
     <row r="945">
       <c r="A945"/>
       <c r="B945" t="s">
-        <v>1601</v>
+        <v>1604</v>
       </c>
       <c r="C945" t="s">
-        <v>1602</v>
+        <v>1605</v>
       </c>
       <c r="D945"/>
       <c r="E945"/>
@@ -22291,10 +22315,10 @@
     <row r="946">
       <c r="A946"/>
       <c r="B946" t="s">
-        <v>1603</v>
+        <v>1606</v>
       </c>
       <c r="C946" t="s">
-        <v>1604</v>
+        <v>1607</v>
       </c>
       <c r="D946"/>
       <c r="E946"/>
@@ -22307,10 +22331,10 @@
     <row r="947">
       <c r="A947"/>
       <c r="B947" t="s">
-        <v>1605</v>
+        <v>1608</v>
       </c>
       <c r="C947" t="s">
-        <v>1606</v>
+        <v>1609</v>
       </c>
       <c r="D947"/>
       <c r="E947"/>
@@ -22323,10 +22347,10 @@
     <row r="948">
       <c r="A948"/>
       <c r="B948" t="s">
-        <v>1607</v>
+        <v>1610</v>
       </c>
       <c r="C948" t="s">
-        <v>1608</v>
+        <v>1611</v>
       </c>
       <c r="D948"/>
       <c r="E948" t="s">
@@ -22341,10 +22365,10 @@
     <row r="949">
       <c r="A949"/>
       <c r="B949" t="s">
-        <v>1609</v>
+        <v>1612</v>
       </c>
       <c r="C949" t="s">
-        <v>1610</v>
+        <v>1613</v>
       </c>
       <c r="D949"/>
       <c r="E949"/>
@@ -22357,10 +22381,10 @@
     <row r="950">
       <c r="A950"/>
       <c r="B950" t="s">
-        <v>1611</v>
+        <v>1614</v>
       </c>
       <c r="C950" t="s">
-        <v>1612</v>
+        <v>1615</v>
       </c>
       <c r="D950"/>
       <c r="E950"/>
@@ -22373,10 +22397,10 @@
     <row r="951">
       <c r="A951"/>
       <c r="B951" t="s">
-        <v>1613</v>
+        <v>1616</v>
       </c>
       <c r="C951" t="s">
-        <v>1614</v>
+        <v>1617</v>
       </c>
       <c r="D951"/>
       <c r="E951"/>
@@ -22389,10 +22413,10 @@
     <row r="952">
       <c r="A952"/>
       <c r="B952" t="s">
-        <v>1615</v>
+        <v>1618</v>
       </c>
       <c r="C952" t="s">
-        <v>1616</v>
+        <v>1619</v>
       </c>
       <c r="D952"/>
       <c r="E952"/>
@@ -22405,10 +22429,10 @@
     <row r="953">
       <c r="A953"/>
       <c r="B953" t="s">
-        <v>1617</v>
+        <v>1620</v>
       </c>
       <c r="C953" t="s">
-        <v>1618</v>
+        <v>1621</v>
       </c>
       <c r="D953"/>
       <c r="E953"/>
@@ -22421,10 +22445,10 @@
     <row r="954">
       <c r="A954"/>
       <c r="B954" t="s">
-        <v>1619</v>
+        <v>1622</v>
       </c>
       <c r="C954" t="s">
-        <v>1620</v>
+        <v>1623</v>
       </c>
       <c r="D954"/>
       <c r="E954"/>
@@ -22434,61 +22458,61 @@
         <v>19</v>
       </c>
     </row>
-    <row r="955">
-      <c r="A955"/>
-      <c r="B955" t="s">
-        <v>1621</v>
-      </c>
-      <c r="C955" t="s">
-        <v>1622</v>
-      </c>
-      <c r="D955"/>
-      <c r="E955"/>
-      <c r="F955"/>
-      <c r="G955"/>
-      <c r="H955" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="956">
-      <c r="A956"/>
-      <c r="B956" t="s">
-        <v>1623</v>
-      </c>
-      <c r="C956" t="s">
+    <row r="955" ht="32" customHeight="1">
+      <c r="A955" s="1"/>
+      <c r="B955" s="1" t="s">
         <v>1624</v>
       </c>
-      <c r="D956"/>
-      <c r="E956"/>
-      <c r="F956"/>
-      <c r="G956"/>
-      <c r="H956" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="957">
-      <c r="A957"/>
-      <c r="B957" t="s">
+      <c r="C955" s="1" t="s">
         <v>1625</v>
       </c>
-      <c r="C957" t="s">
+      <c r="D955" s="1"/>
+      <c r="E955" s="1"/>
+      <c r="F955" s="1"/>
+      <c r="G955" s="1"/>
+      <c r="H955" s="2" t="s">
         <v>1626</v>
       </c>
-      <c r="D957"/>
-      <c r="E957"/>
-      <c r="F957"/>
-      <c r="G957"/>
-      <c r="H957" t="s">
-        <v>19</v>
+    </row>
+    <row r="956" ht="32" customHeight="1">
+      <c r="A956" s="1"/>
+      <c r="B956" s="1" t="s">
+        <v>1627</v>
+      </c>
+      <c r="C956" s="1" t="s">
+        <v>1628</v>
+      </c>
+      <c r="D956" s="1"/>
+      <c r="E956" s="1"/>
+      <c r="F956" s="1"/>
+      <c r="G956" s="1"/>
+      <c r="H956" s="2" t="s">
+        <v>1629</v>
+      </c>
+    </row>
+    <row r="957" ht="32" customHeight="1">
+      <c r="A957" s="1"/>
+      <c r="B957" s="1" t="s">
+        <v>1630</v>
+      </c>
+      <c r="C957" s="1" t="s">
+        <v>1631</v>
+      </c>
+      <c r="D957" s="1"/>
+      <c r="E957" s="1"/>
+      <c r="F957" s="1"/>
+      <c r="G957" s="1"/>
+      <c r="H957" s="2" t="s">
+        <v>1632</v>
       </c>
     </row>
     <row r="958">
       <c r="A958"/>
       <c r="B958" t="s">
-        <v>1627</v>
+        <v>1633</v>
       </c>
       <c r="C958" t="s">
-        <v>1628</v>
+        <v>1634</v>
       </c>
       <c r="D958"/>
       <c r="E958"/>
@@ -22501,10 +22525,10 @@
     <row r="959">
       <c r="A959"/>
       <c r="B959" t="s">
-        <v>1629</v>
+        <v>1635</v>
       </c>
       <c r="C959" t="s">
-        <v>1630</v>
+        <v>1636</v>
       </c>
       <c r="D959"/>
       <c r="E959"/>
@@ -22517,10 +22541,10 @@
     <row r="960">
       <c r="A960"/>
       <c r="B960" t="s">
-        <v>1631</v>
+        <v>1637</v>
       </c>
       <c r="C960" t="s">
-        <v>1632</v>
+        <v>1638</v>
       </c>
       <c r="D960"/>
       <c r="E960"/>
@@ -22533,10 +22557,10 @@
     <row r="961">
       <c r="A961"/>
       <c r="B961" t="s">
-        <v>1633</v>
+        <v>1639</v>
       </c>
       <c r="C961" t="s">
-        <v>1634</v>
+        <v>1640</v>
       </c>
       <c r="D961"/>
       <c r="E961"/>
@@ -22549,10 +22573,10 @@
     <row r="962">
       <c r="A962"/>
       <c r="B962" t="s">
-        <v>1635</v>
+        <v>1641</v>
       </c>
       <c r="C962" t="s">
-        <v>1636</v>
+        <v>1642</v>
       </c>
       <c r="D962"/>
       <c r="E962"/>
@@ -22565,7 +22589,7 @@
     <row r="963">
       <c r="A963"/>
       <c r="B963" t="s">
-        <v>1637</v>
+        <v>1643</v>
       </c>
       <c r="C963" t="s">
         <v>430</v>
@@ -22581,7 +22605,7 @@
     <row r="964">
       <c r="A964"/>
       <c r="B964" t="s">
-        <v>1638</v>
+        <v>1644</v>
       </c>
       <c r="C964" t="s">
         <v>432</v>
@@ -22597,7 +22621,7 @@
     <row r="965">
       <c r="A965"/>
       <c r="B965" t="s">
-        <v>1639</v>
+        <v>1645</v>
       </c>
       <c r="C965" t="s">
         <v>434</v>
@@ -22613,7 +22637,7 @@
     <row r="966" ht="77" customHeight="1">
       <c r="A966" s="1"/>
       <c r="B966" s="1" t="s">
-        <v>1640</v>
+        <v>1646</v>
       </c>
       <c r="C966" s="1" t="s">
         <v>436</v>
@@ -22629,7 +22653,7 @@
     <row r="967" ht="77" customHeight="1">
       <c r="A967" s="1"/>
       <c r="B967" s="1" t="s">
-        <v>1641</v>
+        <v>1647</v>
       </c>
       <c r="C967" s="1" t="s">
         <v>438</v>
@@ -22645,7 +22669,7 @@
     <row r="968" ht="77" customHeight="1">
       <c r="A968" s="1"/>
       <c r="B968" s="1" t="s">
-        <v>1642</v>
+        <v>1648</v>
       </c>
       <c r="C968" s="1" t="s">
         <v>440</v>
@@ -22661,7 +22685,7 @@
     <row r="969" ht="77" customHeight="1">
       <c r="A969" s="1"/>
       <c r="B969" s="1" t="s">
-        <v>1643</v>
+        <v>1649</v>
       </c>
       <c r="C969" s="1" t="s">
         <v>442</v>
@@ -22677,7 +22701,7 @@
     <row r="970" ht="77" customHeight="1">
       <c r="A970" s="1"/>
       <c r="B970" s="1" t="s">
-        <v>1644</v>
+        <v>1650</v>
       </c>
       <c r="C970" s="1" t="s">
         <v>444</v>
@@ -22693,7 +22717,7 @@
     <row r="971" ht="77" customHeight="1">
       <c r="A971" s="1"/>
       <c r="B971" s="1" t="s">
-        <v>1645</v>
+        <v>1651</v>
       </c>
       <c r="C971" s="1" t="s">
         <v>446</v>
@@ -22709,7 +22733,7 @@
     <row r="972" ht="77" customHeight="1">
       <c r="A972" s="1"/>
       <c r="B972" s="1" t="s">
-        <v>1646</v>
+        <v>1652</v>
       </c>
       <c r="C972" s="1" t="s">
         <v>448</v>
@@ -22725,7 +22749,7 @@
     <row r="973" ht="77" customHeight="1">
       <c r="A973" s="1"/>
       <c r="B973" s="1" t="s">
-        <v>1647</v>
+        <v>1653</v>
       </c>
       <c r="C973" s="1" t="s">
         <v>450</v>
@@ -22741,7 +22765,7 @@
     <row r="974">
       <c r="A974"/>
       <c r="B974" t="s">
-        <v>1648</v>
+        <v>1654</v>
       </c>
       <c r="C974" t="s">
         <v>452</v>
@@ -22757,7 +22781,7 @@
     <row r="975">
       <c r="A975"/>
       <c r="B975" t="s">
-        <v>1649</v>
+        <v>1655</v>
       </c>
       <c r="C975" t="s">
         <v>454</v>
@@ -22775,7 +22799,7 @@
     <row r="976">
       <c r="A976"/>
       <c r="B976" t="s">
-        <v>1650</v>
+        <v>1656</v>
       </c>
       <c r="C976" t="s">
         <v>456</v>
@@ -22791,10 +22815,10 @@
     <row r="977">
       <c r="A977"/>
       <c r="B977" t="s">
-        <v>1651</v>
+        <v>1657</v>
       </c>
       <c r="C977" t="s">
-        <v>1652</v>
+        <v>1658</v>
       </c>
       <c r="D977"/>
       <c r="E977"/>
@@ -22807,10 +22831,10 @@
     <row r="978">
       <c r="A978"/>
       <c r="B978" t="s">
-        <v>1653</v>
+        <v>1659</v>
       </c>
       <c r="C978" t="s">
-        <v>1654</v>
+        <v>1660</v>
       </c>
       <c r="D978"/>
       <c r="E978"/>
@@ -22823,10 +22847,10 @@
     <row r="979">
       <c r="A979"/>
       <c r="B979" t="s">
-        <v>1655</v>
+        <v>1661</v>
       </c>
       <c r="C979" t="s">
-        <v>1656</v>
+        <v>1662</v>
       </c>
       <c r="D979"/>
       <c r="E979"/>
@@ -22839,10 +22863,10 @@
     <row r="980">
       <c r="A980"/>
       <c r="B980" t="s">
-        <v>1657</v>
+        <v>1663</v>
       </c>
       <c r="C980" t="s">
-        <v>1658</v>
+        <v>1664</v>
       </c>
       <c r="D980"/>
       <c r="E980"/>
@@ -22855,10 +22879,10 @@
     <row r="981">
       <c r="A981"/>
       <c r="B981" t="s">
-        <v>1659</v>
+        <v>1665</v>
       </c>
       <c r="C981" t="s">
-        <v>1660</v>
+        <v>1666</v>
       </c>
       <c r="D981"/>
       <c r="E981"/>
@@ -22871,10 +22895,10 @@
     <row r="982">
       <c r="A982"/>
       <c r="B982" t="s">
-        <v>1661</v>
+        <v>1667</v>
       </c>
       <c r="C982" t="s">
-        <v>1662</v>
+        <v>1668</v>
       </c>
       <c r="D982"/>
       <c r="E982"/>
@@ -22887,10 +22911,10 @@
     <row r="983">
       <c r="A983"/>
       <c r="B983" t="s">
-        <v>1663</v>
+        <v>1669</v>
       </c>
       <c r="C983" t="s">
-        <v>1664</v>
+        <v>1670</v>
       </c>
       <c r="D983"/>
       <c r="E983"/>
@@ -22903,10 +22927,10 @@
     <row r="984" ht="77" customHeight="1">
       <c r="A984" s="1"/>
       <c r="B984" s="1" t="s">
-        <v>1665</v>
+        <v>1671</v>
       </c>
       <c r="C984" s="1" t="s">
-        <v>1666</v>
+        <v>1672</v>
       </c>
       <c r="D984" s="1"/>
       <c r="E984" s="1"/>
@@ -22919,10 +22943,10 @@
     <row r="985" ht="77" customHeight="1">
       <c r="A985" s="1"/>
       <c r="B985" s="1" t="s">
-        <v>1667</v>
+        <v>1673</v>
       </c>
       <c r="C985" s="1" t="s">
-        <v>1668</v>
+        <v>1674</v>
       </c>
       <c r="D985" s="1"/>
       <c r="E985" s="1"/>
@@ -22935,10 +22959,10 @@
     <row r="986" ht="77" customHeight="1">
       <c r="A986" s="1"/>
       <c r="B986" s="1" t="s">
-        <v>1669</v>
+        <v>1675</v>
       </c>
       <c r="C986" s="1" t="s">
-        <v>1670</v>
+        <v>1676</v>
       </c>
       <c r="D986" s="1"/>
       <c r="E986" s="1"/>
@@ -22951,10 +22975,10 @@
     <row r="987" ht="77" customHeight="1">
       <c r="A987" s="1"/>
       <c r="B987" s="1" t="s">
-        <v>1671</v>
+        <v>1677</v>
       </c>
       <c r="C987" s="1" t="s">
-        <v>1672</v>
+        <v>1678</v>
       </c>
       <c r="D987" s="1"/>
       <c r="E987" s="1"/>
@@ -22967,10 +22991,10 @@
     <row r="988" ht="77" customHeight="1">
       <c r="A988" s="1"/>
       <c r="B988" s="1" t="s">
-        <v>1673</v>
+        <v>1679</v>
       </c>
       <c r="C988" s="1" t="s">
-        <v>1674</v>
+        <v>1680</v>
       </c>
       <c r="D988" s="1"/>
       <c r="E988" s="1"/>
@@ -22983,10 +23007,10 @@
     <row r="989" ht="77" customHeight="1">
       <c r="A989" s="1"/>
       <c r="B989" s="1" t="s">
-        <v>1675</v>
+        <v>1681</v>
       </c>
       <c r="C989" s="1" t="s">
-        <v>1676</v>
+        <v>1682</v>
       </c>
       <c r="D989" s="1"/>
       <c r="E989" s="1"/>
@@ -22999,10 +23023,10 @@
     <row r="990" ht="77" customHeight="1">
       <c r="A990" s="1"/>
       <c r="B990" s="1" t="s">
-        <v>1677</v>
+        <v>1683</v>
       </c>
       <c r="C990" s="1" t="s">
-        <v>1678</v>
+        <v>1684</v>
       </c>
       <c r="D990" s="1"/>
       <c r="E990" s="1"/>
@@ -23015,10 +23039,10 @@
     <row r="991" ht="77" customHeight="1">
       <c r="A991" s="1"/>
       <c r="B991" s="1" t="s">
-        <v>1679</v>
+        <v>1685</v>
       </c>
       <c r="C991" s="1" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="D991" s="1"/>
       <c r="E991" s="1"/>
@@ -23031,10 +23055,10 @@
     <row r="992">
       <c r="A992"/>
       <c r="B992" t="s">
-        <v>1681</v>
+        <v>1687</v>
       </c>
       <c r="C992" t="s">
-        <v>1682</v>
+        <v>1688</v>
       </c>
       <c r="D992"/>
       <c r="E992"/>
@@ -23047,10 +23071,10 @@
     <row r="993">
       <c r="A993"/>
       <c r="B993" t="s">
-        <v>1683</v>
+        <v>1689</v>
       </c>
       <c r="C993" t="s">
-        <v>1684</v>
+        <v>1690</v>
       </c>
       <c r="D993"/>
       <c r="E993" t="s">
@@ -23065,10 +23089,10 @@
     <row r="994">
       <c r="A994"/>
       <c r="B994" t="s">
-        <v>1685</v>
+        <v>1691</v>
       </c>
       <c r="C994" t="s">
-        <v>1686</v>
+        <v>1692</v>
       </c>
       <c r="D994"/>
       <c r="E994"/>
@@ -23081,10 +23105,10 @@
     <row r="995">
       <c r="A995"/>
       <c r="B995" t="s">
-        <v>1687</v>
+        <v>1693</v>
       </c>
       <c r="C995" t="s">
-        <v>1688</v>
+        <v>1694</v>
       </c>
       <c r="D995"/>
       <c r="E995"/>
@@ -23097,10 +23121,10 @@
     <row r="996">
       <c r="A996"/>
       <c r="B996" t="s">
-        <v>1689</v>
+        <v>1695</v>
       </c>
       <c r="C996" t="s">
-        <v>1690</v>
+        <v>1696</v>
       </c>
       <c r="D996"/>
       <c r="E996"/>
@@ -23113,10 +23137,10 @@
     <row r="997">
       <c r="A997"/>
       <c r="B997" t="s">
-        <v>1691</v>
+        <v>1697</v>
       </c>
       <c r="C997" t="s">
-        <v>1692</v>
+        <v>1698</v>
       </c>
       <c r="D997"/>
       <c r="E997" t="s">
@@ -23131,10 +23155,10 @@
     <row r="998">
       <c r="A998"/>
       <c r="B998" t="s">
-        <v>1693</v>
+        <v>1699</v>
       </c>
       <c r="C998" t="s">
-        <v>1694</v>
+        <v>1700</v>
       </c>
       <c r="D998"/>
       <c r="E998"/>
@@ -23147,10 +23171,10 @@
     <row r="999">
       <c r="A999"/>
       <c r="B999" t="s">
-        <v>1695</v>
+        <v>1701</v>
       </c>
       <c r="C999" t="s">
-        <v>1696</v>
+        <v>1702</v>
       </c>
       <c r="D999"/>
       <c r="E999"/>
@@ -23163,10 +23187,10 @@
     <row r="1000">
       <c r="A1000"/>
       <c r="B1000" t="s">
-        <v>1697</v>
+        <v>1703</v>
       </c>
       <c r="C1000" t="s">
-        <v>1698</v>
+        <v>1704</v>
       </c>
       <c r="D1000"/>
       <c r="E1000"/>
@@ -23179,10 +23203,10 @@
     <row r="1001">
       <c r="A1001"/>
       <c r="B1001" t="s">
-        <v>1699</v>
+        <v>1705</v>
       </c>
       <c r="C1001" t="s">
-        <v>1700</v>
+        <v>1706</v>
       </c>
       <c r="D1001"/>
       <c r="E1001"/>
@@ -23195,10 +23219,10 @@
     <row r="1002">
       <c r="A1002"/>
       <c r="B1002" t="s">
-        <v>1701</v>
+        <v>1707</v>
       </c>
       <c r="C1002" t="s">
-        <v>1702</v>
+        <v>1708</v>
       </c>
       <c r="D1002"/>
       <c r="E1002"/>
@@ -23211,10 +23235,10 @@
     <row r="1003">
       <c r="A1003"/>
       <c r="B1003" t="s">
-        <v>1703</v>
+        <v>1709</v>
       </c>
       <c r="C1003" t="s">
-        <v>1704</v>
+        <v>1710</v>
       </c>
       <c r="D1003"/>
       <c r="E1003"/>
@@ -23227,10 +23251,10 @@
     <row r="1004">
       <c r="A1004"/>
       <c r="B1004" t="s">
-        <v>1705</v>
+        <v>1711</v>
       </c>
       <c r="C1004" t="s">
-        <v>1706</v>
+        <v>1712</v>
       </c>
       <c r="D1004"/>
       <c r="E1004"/>
@@ -23243,10 +23267,10 @@
     <row r="1005">
       <c r="A1005"/>
       <c r="B1005" t="s">
-        <v>1707</v>
+        <v>1713</v>
       </c>
       <c r="C1005" t="s">
-        <v>1708</v>
+        <v>1714</v>
       </c>
       <c r="D1005"/>
       <c r="E1005"/>
@@ -23259,10 +23283,10 @@
     <row r="1006">
       <c r="A1006"/>
       <c r="B1006" t="s">
-        <v>1709</v>
+        <v>1715</v>
       </c>
       <c r="C1006" t="s">
-        <v>1710</v>
+        <v>1716</v>
       </c>
       <c r="D1006"/>
       <c r="E1006"/>
@@ -23275,10 +23299,10 @@
     <row r="1007">
       <c r="A1007"/>
       <c r="B1007" t="s">
-        <v>1711</v>
+        <v>1717</v>
       </c>
       <c r="C1007" t="s">
-        <v>1712</v>
+        <v>1718</v>
       </c>
       <c r="D1007"/>
       <c r="E1007"/>
@@ -23291,10 +23315,10 @@
     <row r="1008">
       <c r="A1008"/>
       <c r="B1008" t="s">
-        <v>1713</v>
+        <v>1719</v>
       </c>
       <c r="C1008" t="s">
-        <v>1714</v>
+        <v>1720</v>
       </c>
       <c r="D1008"/>
       <c r="E1008"/>
@@ -23307,10 +23331,10 @@
     <row r="1009">
       <c r="A1009"/>
       <c r="B1009" t="s">
-        <v>1715</v>
+        <v>1721</v>
       </c>
       <c r="C1009" t="s">
-        <v>1716</v>
+        <v>1722</v>
       </c>
       <c r="D1009"/>
       <c r="E1009"/>
@@ -23323,10 +23347,10 @@
     <row r="1010">
       <c r="A1010"/>
       <c r="B1010" t="s">
-        <v>1717</v>
+        <v>1723</v>
       </c>
       <c r="C1010" t="s">
-        <v>1718</v>
+        <v>1724</v>
       </c>
       <c r="D1010"/>
       <c r="E1010"/>
@@ -23339,10 +23363,10 @@
     <row r="1011">
       <c r="A1011"/>
       <c r="B1011" t="s">
-        <v>1719</v>
+        <v>1725</v>
       </c>
       <c r="C1011" t="s">
-        <v>1720</v>
+        <v>1726</v>
       </c>
       <c r="D1011"/>
       <c r="E1011" t="s">
@@ -23357,10 +23381,10 @@
     <row r="1012">
       <c r="A1012"/>
       <c r="B1012" t="s">
-        <v>1721</v>
+        <v>1727</v>
       </c>
       <c r="C1012" t="s">
-        <v>1722</v>
+        <v>1728</v>
       </c>
       <c r="D1012"/>
       <c r="E1012"/>
@@ -23373,10 +23397,10 @@
     <row r="1013">
       <c r="A1013"/>
       <c r="B1013" t="s">
-        <v>1723</v>
+        <v>1729</v>
       </c>
       <c r="C1013" t="s">
-        <v>1724</v>
+        <v>1730</v>
       </c>
       <c r="D1013"/>
       <c r="E1013"/>
@@ -23389,10 +23413,10 @@
     <row r="1014">
       <c r="A1014"/>
       <c r="B1014" t="s">
-        <v>1725</v>
+        <v>1731</v>
       </c>
       <c r="C1014" t="s">
-        <v>1726</v>
+        <v>1732</v>
       </c>
       <c r="D1014"/>
       <c r="E1014"/>
@@ -23405,10 +23429,10 @@
     <row r="1015">
       <c r="A1015"/>
       <c r="B1015" t="s">
-        <v>1727</v>
+        <v>1733</v>
       </c>
       <c r="C1015" t="s">
-        <v>1728</v>
+        <v>1734</v>
       </c>
       <c r="D1015"/>
       <c r="E1015" t="s">
@@ -23423,10 +23447,10 @@
     <row r="1016">
       <c r="A1016"/>
       <c r="B1016" t="s">
-        <v>1729</v>
+        <v>1735</v>
       </c>
       <c r="C1016" t="s">
-        <v>1730</v>
+        <v>1736</v>
       </c>
       <c r="D1016"/>
       <c r="E1016"/>
@@ -23439,10 +23463,10 @@
     <row r="1017">
       <c r="A1017"/>
       <c r="B1017" t="s">
-        <v>1731</v>
+        <v>1737</v>
       </c>
       <c r="C1017" t="s">
-        <v>1732</v>
+        <v>1738</v>
       </c>
       <c r="D1017"/>
       <c r="E1017"/>
@@ -23455,10 +23479,10 @@
     <row r="1018">
       <c r="A1018"/>
       <c r="B1018" t="s">
-        <v>1733</v>
+        <v>1739</v>
       </c>
       <c r="C1018" t="s">
-        <v>1734</v>
+        <v>1740</v>
       </c>
       <c r="D1018"/>
       <c r="E1018"/>
@@ -23471,10 +23495,10 @@
     <row r="1019">
       <c r="A1019"/>
       <c r="B1019" t="s">
-        <v>1735</v>
+        <v>1741</v>
       </c>
       <c r="C1019" t="s">
-        <v>1736</v>
+        <v>1742</v>
       </c>
       <c r="D1019"/>
       <c r="E1019"/>
@@ -23487,10 +23511,10 @@
     <row r="1020">
       <c r="A1020"/>
       <c r="B1020" t="s">
-        <v>1737</v>
+        <v>1743</v>
       </c>
       <c r="C1020" t="s">
-        <v>1738</v>
+        <v>1744</v>
       </c>
       <c r="D1020"/>
       <c r="E1020"/>
@@ -23503,10 +23527,10 @@
     <row r="1021">
       <c r="A1021"/>
       <c r="B1021" t="s">
-        <v>1739</v>
+        <v>1745</v>
       </c>
       <c r="C1021" t="s">
-        <v>1740</v>
+        <v>1746</v>
       </c>
       <c r="D1021"/>
       <c r="E1021"/>
@@ -23519,10 +23543,10 @@
     <row r="1022" ht="77" customHeight="1">
       <c r="A1022" s="1"/>
       <c r="B1022" s="1" t="s">
-        <v>1741</v>
+        <v>1747</v>
       </c>
       <c r="C1022" s="1" t="s">
-        <v>1742</v>
+        <v>1748</v>
       </c>
       <c r="D1022" s="1"/>
       <c r="E1022" s="1"/>
@@ -23535,10 +23559,10 @@
     <row r="1023" ht="77" customHeight="1">
       <c r="A1023" s="1"/>
       <c r="B1023" s="1" t="s">
-        <v>1743</v>
+        <v>1749</v>
       </c>
       <c r="C1023" s="1" t="s">
-        <v>1744</v>
+        <v>1750</v>
       </c>
       <c r="D1023" s="1"/>
       <c r="E1023" s="1"/>
@@ -23551,10 +23575,10 @@
     <row r="1024" ht="77" customHeight="1">
       <c r="A1024" s="1"/>
       <c r="B1024" s="1" t="s">
-        <v>1745</v>
+        <v>1751</v>
       </c>
       <c r="C1024" s="1" t="s">
-        <v>1746</v>
+        <v>1752</v>
       </c>
       <c r="D1024" s="1"/>
       <c r="E1024" s="1"/>
@@ -23567,10 +23591,10 @@
     <row r="1025" ht="77" customHeight="1">
       <c r="A1025" s="1"/>
       <c r="B1025" s="1" t="s">
-        <v>1747</v>
+        <v>1753</v>
       </c>
       <c r="C1025" s="1" t="s">
-        <v>1748</v>
+        <v>1754</v>
       </c>
       <c r="D1025" s="1"/>
       <c r="E1025" s="1"/>
@@ -23583,10 +23607,10 @@
     <row r="1026" ht="77" customHeight="1">
       <c r="A1026" s="1"/>
       <c r="B1026" s="1" t="s">
-        <v>1749</v>
+        <v>1755</v>
       </c>
       <c r="C1026" s="1" t="s">
-        <v>1750</v>
+        <v>1756</v>
       </c>
       <c r="D1026" s="1"/>
       <c r="E1026" s="1"/>
@@ -23599,10 +23623,10 @@
     <row r="1027" ht="77" customHeight="1">
       <c r="A1027" s="1"/>
       <c r="B1027" s="1" t="s">
-        <v>1751</v>
+        <v>1757</v>
       </c>
       <c r="C1027" s="1" t="s">
-        <v>1752</v>
+        <v>1758</v>
       </c>
       <c r="D1027" s="1"/>
       <c r="E1027" s="1"/>
@@ -23615,10 +23639,10 @@
     <row r="1028" ht="77" customHeight="1">
       <c r="A1028" s="1"/>
       <c r="B1028" s="1" t="s">
-        <v>1753</v>
+        <v>1759</v>
       </c>
       <c r="C1028" s="1" t="s">
-        <v>1754</v>
+        <v>1760</v>
       </c>
       <c r="D1028" s="1"/>
       <c r="E1028" s="1"/>
@@ -23631,10 +23655,10 @@
     <row r="1029" ht="77" customHeight="1">
       <c r="A1029" s="1"/>
       <c r="B1029" s="1" t="s">
-        <v>1755</v>
+        <v>1761</v>
       </c>
       <c r="C1029" s="1" t="s">
-        <v>1756</v>
+        <v>1762</v>
       </c>
       <c r="D1029" s="1"/>
       <c r="E1029" s="1"/>
@@ -23647,10 +23671,10 @@
     <row r="1030">
       <c r="A1030"/>
       <c r="B1030" t="s">
-        <v>1757</v>
+        <v>1763</v>
       </c>
       <c r="C1030" t="s">
-        <v>1758</v>
+        <v>1764</v>
       </c>
       <c r="D1030"/>
       <c r="E1030"/>
@@ -23672,10 +23696,10 @@
     </row>
     <row r="1032">
       <c r="A1032" t="s">
-        <v>1759</v>
+        <v>1765</v>
       </c>
       <c r="B1032" t="s">
-        <v>1760</v>
+        <v>1766</v>
       </c>
       <c r="C1032" t="s">
         <v>15</v>
@@ -23691,7 +23715,7 @@
     <row r="1033">
       <c r="A1033"/>
       <c r="B1033" t="s">
-        <v>1761</v>
+        <v>1767</v>
       </c>
       <c r="C1033" t="s">
         <v>18</v>
@@ -23707,7 +23731,7 @@
     <row r="1034">
       <c r="A1034"/>
       <c r="B1034" t="s">
-        <v>1762</v>
+        <v>1768</v>
       </c>
       <c r="C1034" t="s">
         <v>21</v>
@@ -23725,7 +23749,7 @@
     <row r="1035">
       <c r="A1035"/>
       <c r="B1035" t="s">
-        <v>1763</v>
+        <v>1769</v>
       </c>
       <c r="C1035" t="s">
         <v>24</v>
@@ -23741,7 +23765,7 @@
     <row r="1036" ht="77" customHeight="1">
       <c r="A1036" s="1"/>
       <c r="B1036" s="1" t="s">
-        <v>1764</v>
+        <v>1770</v>
       </c>
       <c r="C1036" s="1" t="s">
         <v>26</v>
@@ -23757,7 +23781,7 @@
     <row r="1037" ht="77" customHeight="1">
       <c r="A1037" s="1"/>
       <c r="B1037" s="1" t="s">
-        <v>1765</v>
+        <v>1771</v>
       </c>
       <c r="C1037" s="1" t="s">
         <v>29</v>
@@ -23773,7 +23797,7 @@
     <row r="1038" ht="77" customHeight="1">
       <c r="A1038" s="1"/>
       <c r="B1038" s="1" t="s">
-        <v>1766</v>
+        <v>1772</v>
       </c>
       <c r="C1038" s="1" t="s">
         <v>31</v>
@@ -23789,7 +23813,7 @@
     <row r="1039" ht="77" customHeight="1">
       <c r="A1039" s="1"/>
       <c r="B1039" s="1" t="s">
-        <v>1767</v>
+        <v>1773</v>
       </c>
       <c r="C1039" s="1" t="s">
         <v>33</v>
@@ -23805,7 +23829,7 @@
     <row r="1040" ht="77" customHeight="1">
       <c r="A1040" s="1"/>
       <c r="B1040" s="1" t="s">
-        <v>1768</v>
+        <v>1774</v>
       </c>
       <c r="C1040" s="1" t="s">
         <v>35</v>
@@ -23821,7 +23845,7 @@
     <row r="1041" ht="77" customHeight="1">
       <c r="A1041" s="1"/>
       <c r="B1041" s="1" t="s">
-        <v>1769</v>
+        <v>1775</v>
       </c>
       <c r="C1041" s="1" t="s">
         <v>37</v>
@@ -23837,7 +23861,7 @@
     <row r="1042" ht="77" customHeight="1">
       <c r="A1042" s="1"/>
       <c r="B1042" s="1" t="s">
-        <v>1770</v>
+        <v>1776</v>
       </c>
       <c r="C1042" s="1" t="s">
         <v>39</v>
@@ -23853,7 +23877,7 @@
     <row r="1043" ht="77" customHeight="1">
       <c r="A1043" s="1"/>
       <c r="B1043" s="1" t="s">
-        <v>1771</v>
+        <v>1777</v>
       </c>
       <c r="C1043" s="1" t="s">
         <v>41</v>
@@ -23869,7 +23893,7 @@
     <row r="1044" ht="77" customHeight="1">
       <c r="A1044" s="1"/>
       <c r="B1044" s="1" t="s">
-        <v>1772</v>
+        <v>1778</v>
       </c>
       <c r="C1044" s="1" t="s">
         <v>44</v>
@@ -23887,7 +23911,7 @@
     <row r="1045" ht="77" customHeight="1">
       <c r="A1045" s="1"/>
       <c r="B1045" s="1" t="s">
-        <v>1773</v>
+        <v>1779</v>
       </c>
       <c r="C1045" s="1" t="s">
         <v>46</v>
@@ -23905,7 +23929,7 @@
     <row r="1046">
       <c r="A1046"/>
       <c r="B1046" t="s">
-        <v>1774</v>
+        <v>1780</v>
       </c>
       <c r="C1046" t="s">
         <v>236</v>
@@ -23921,7 +23945,7 @@
     <row r="1047">
       <c r="A1047"/>
       <c r="B1047" t="s">
-        <v>1775</v>
+        <v>1781</v>
       </c>
       <c r="C1047" t="s">
         <v>238</v>
@@ -23937,7 +23961,7 @@
     <row r="1048">
       <c r="A1048"/>
       <c r="B1048" t="s">
-        <v>1776</v>
+        <v>1782</v>
       </c>
       <c r="C1048" t="s">
         <v>48</v>
@@ -23953,7 +23977,7 @@
     <row r="1049">
       <c r="A1049"/>
       <c r="B1049" t="s">
-        <v>1777</v>
+        <v>1783</v>
       </c>
       <c r="C1049" t="s">
         <v>50</v>
@@ -23969,10 +23993,10 @@
     <row r="1050">
       <c r="A1050"/>
       <c r="B1050" t="s">
-        <v>1778</v>
+        <v>1784</v>
       </c>
       <c r="C1050" t="s">
-        <v>1779</v>
+        <v>1785</v>
       </c>
       <c r="D1050"/>
       <c r="E1050"/>
@@ -23985,7 +24009,7 @@
     <row r="1051">
       <c r="A1051"/>
       <c r="B1051" t="s">
-        <v>1780</v>
+        <v>1786</v>
       </c>
       <c r="C1051" t="s">
         <v>718</v>
@@ -24001,7 +24025,7 @@
     <row r="1052">
       <c r="A1052"/>
       <c r="B1052" t="s">
-        <v>1781</v>
+        <v>1787</v>
       </c>
       <c r="C1052" t="s">
         <v>56</v>
@@ -24017,7 +24041,7 @@
     <row r="1053">
       <c r="A1053"/>
       <c r="B1053" t="s">
-        <v>1782</v>
+        <v>1788</v>
       </c>
       <c r="C1053" t="s">
         <v>261</v>
@@ -24033,7 +24057,7 @@
     <row r="1054">
       <c r="A1054"/>
       <c r="B1054" t="s">
-        <v>1783</v>
+        <v>1789</v>
       </c>
       <c r="C1054" t="s">
         <v>263</v>
@@ -24049,7 +24073,7 @@
     <row r="1055">
       <c r="A1055"/>
       <c r="B1055" t="s">
-        <v>1784</v>
+        <v>1790</v>
       </c>
       <c r="C1055" t="s">
         <v>265</v>
@@ -24065,7 +24089,7 @@
     <row r="1056">
       <c r="A1056"/>
       <c r="B1056" t="s">
-        <v>1785</v>
+        <v>1791</v>
       </c>
       <c r="C1056" t="s">
         <v>267</v>
@@ -24081,7 +24105,7 @@
     <row r="1057">
       <c r="A1057"/>
       <c r="B1057" t="s">
-        <v>1786</v>
+        <v>1792</v>
       </c>
       <c r="C1057" t="s">
         <v>269</v>
@@ -24097,7 +24121,7 @@
     <row r="1058">
       <c r="A1058"/>
       <c r="B1058" t="s">
-        <v>1787</v>
+        <v>1793</v>
       </c>
       <c r="C1058" t="s">
         <v>281</v>
@@ -24113,7 +24137,7 @@
     <row r="1059">
       <c r="A1059"/>
       <c r="B1059" t="s">
-        <v>1788</v>
+        <v>1794</v>
       </c>
       <c r="C1059" t="s">
         <v>283</v>
@@ -24129,7 +24153,7 @@
     <row r="1060">
       <c r="A1060"/>
       <c r="B1060" t="s">
-        <v>1789</v>
+        <v>1795</v>
       </c>
       <c r="C1060" t="s">
         <v>285</v>
@@ -24145,7 +24169,7 @@
     <row r="1061">
       <c r="A1061"/>
       <c r="B1061" t="s">
-        <v>1790</v>
+        <v>1796</v>
       </c>
       <c r="C1061" t="s">
         <v>287</v>
@@ -24161,7 +24185,7 @@
     <row r="1062">
       <c r="A1062"/>
       <c r="B1062" t="s">
-        <v>1791</v>
+        <v>1797</v>
       </c>
       <c r="C1062" t="s">
         <v>289</v>
@@ -24177,7 +24201,7 @@
     <row r="1063">
       <c r="A1063"/>
       <c r="B1063" t="s">
-        <v>1792</v>
+        <v>1798</v>
       </c>
       <c r="C1063" t="s">
         <v>1058</v>
@@ -24195,10 +24219,10 @@
     <row r="1064">
       <c r="A1064"/>
       <c r="B1064" t="s">
-        <v>1793</v>
+        <v>1799</v>
       </c>
       <c r="C1064" t="s">
-        <v>1570</v>
+        <v>1573</v>
       </c>
       <c r="D1064"/>
       <c r="E1064" t="s">
@@ -24213,10 +24237,10 @@
     <row r="1065">
       <c r="A1065"/>
       <c r="B1065" t="s">
-        <v>1794</v>
+        <v>1800</v>
       </c>
       <c r="C1065" t="s">
-        <v>1662</v>
+        <v>1668</v>
       </c>
       <c r="D1065"/>
       <c r="E1065"/>
@@ -24229,10 +24253,10 @@
     <row r="1066">
       <c r="A1066"/>
       <c r="B1066" t="s">
-        <v>1795</v>
+        <v>1801</v>
       </c>
       <c r="C1066" t="s">
-        <v>1664</v>
+        <v>1670</v>
       </c>
       <c r="D1066"/>
       <c r="E1066"/>
@@ -24245,10 +24269,10 @@
     <row r="1067" ht="77" customHeight="1">
       <c r="A1067" s="1"/>
       <c r="B1067" s="1" t="s">
-        <v>1796</v>
+        <v>1802</v>
       </c>
       <c r="C1067" s="1" t="s">
-        <v>1666</v>
+        <v>1672</v>
       </c>
       <c r="D1067" s="1"/>
       <c r="E1067" s="1"/>
@@ -24261,10 +24285,10 @@
     <row r="1068" ht="77" customHeight="1">
       <c r="A1068" s="1"/>
       <c r="B1068" s="1" t="s">
-        <v>1797</v>
+        <v>1803</v>
       </c>
       <c r="C1068" s="1" t="s">
-        <v>1668</v>
+        <v>1674</v>
       </c>
       <c r="D1068" s="1"/>
       <c r="E1068" s="1"/>
@@ -24277,10 +24301,10 @@
     <row r="1069" ht="77" customHeight="1">
       <c r="A1069" s="1"/>
       <c r="B1069" s="1" t="s">
-        <v>1798</v>
+        <v>1804</v>
       </c>
       <c r="C1069" s="1" t="s">
-        <v>1670</v>
+        <v>1676</v>
       </c>
       <c r="D1069" s="1"/>
       <c r="E1069" s="1"/>
@@ -24293,10 +24317,10 @@
     <row r="1070" ht="77" customHeight="1">
       <c r="A1070" s="1"/>
       <c r="B1070" s="1" t="s">
-        <v>1799</v>
+        <v>1805</v>
       </c>
       <c r="C1070" s="1" t="s">
-        <v>1672</v>
+        <v>1678</v>
       </c>
       <c r="D1070" s="1"/>
       <c r="E1070" s="1"/>
@@ -24309,10 +24333,10 @@
     <row r="1071" ht="77" customHeight="1">
       <c r="A1071" s="1"/>
       <c r="B1071" s="1" t="s">
-        <v>1800</v>
+        <v>1806</v>
       </c>
       <c r="C1071" s="1" t="s">
-        <v>1674</v>
+        <v>1680</v>
       </c>
       <c r="D1071" s="1"/>
       <c r="E1071" s="1"/>
@@ -24325,10 +24349,10 @@
     <row r="1072" ht="77" customHeight="1">
       <c r="A1072" s="1"/>
       <c r="B1072" s="1" t="s">
-        <v>1801</v>
+        <v>1807</v>
       </c>
       <c r="C1072" s="1" t="s">
-        <v>1676</v>
+        <v>1682</v>
       </c>
       <c r="D1072" s="1"/>
       <c r="E1072" s="1"/>
@@ -24341,10 +24365,10 @@
     <row r="1073" ht="77" customHeight="1">
       <c r="A1073" s="1"/>
       <c r="B1073" s="1" t="s">
-        <v>1802</v>
+        <v>1808</v>
       </c>
       <c r="C1073" s="1" t="s">
-        <v>1678</v>
+        <v>1684</v>
       </c>
       <c r="D1073" s="1"/>
       <c r="E1073" s="1"/>
@@ -24357,10 +24381,10 @@
     <row r="1074" ht="77" customHeight="1">
       <c r="A1074" s="1"/>
       <c r="B1074" s="1" t="s">
-        <v>1803</v>
+        <v>1809</v>
       </c>
       <c r="C1074" s="1" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="D1074" s="1"/>
       <c r="E1074" s="1"/>
@@ -24373,10 +24397,10 @@
     <row r="1075">
       <c r="A1075"/>
       <c r="B1075" t="s">
-        <v>1804</v>
+        <v>1810</v>
       </c>
       <c r="C1075" t="s">
-        <v>1682</v>
+        <v>1688</v>
       </c>
       <c r="D1075"/>
       <c r="E1075"/>
@@ -24389,10 +24413,10 @@
     <row r="1076">
       <c r="A1076"/>
       <c r="B1076" t="s">
-        <v>1805</v>
+        <v>1811</v>
       </c>
       <c r="C1076" t="s">
-        <v>1806</v>
+        <v>1812</v>
       </c>
       <c r="D1076"/>
       <c r="E1076"/>
@@ -24405,10 +24429,10 @@
     <row r="1077">
       <c r="A1077"/>
       <c r="B1077" t="s">
-        <v>1807</v>
+        <v>1813</v>
       </c>
       <c r="C1077" t="s">
-        <v>1808</v>
+        <v>1814</v>
       </c>
       <c r="D1077"/>
       <c r="E1077"/>
@@ -24421,10 +24445,10 @@
     <row r="1078">
       <c r="A1078"/>
       <c r="B1078" t="s">
-        <v>1809</v>
+        <v>1815</v>
       </c>
       <c r="C1078" t="s">
-        <v>1810</v>
+        <v>1816</v>
       </c>
       <c r="D1078"/>
       <c r="E1078"/>
@@ -24437,10 +24461,10 @@
     <row r="1079">
       <c r="A1079"/>
       <c r="B1079" t="s">
-        <v>1811</v>
+        <v>1817</v>
       </c>
       <c r="C1079" t="s">
-        <v>1812</v>
+        <v>1818</v>
       </c>
       <c r="D1079"/>
       <c r="E1079"/>
@@ -24453,10 +24477,10 @@
     <row r="1080">
       <c r="A1080"/>
       <c r="B1080" t="s">
-        <v>1813</v>
+        <v>1819</v>
       </c>
       <c r="C1080" t="s">
-        <v>1814</v>
+        <v>1820</v>
       </c>
       <c r="D1080"/>
       <c r="E1080"/>
@@ -24469,10 +24493,10 @@
     <row r="1081">
       <c r="A1081"/>
       <c r="B1081" t="s">
-        <v>1815</v>
+        <v>1821</v>
       </c>
       <c r="C1081" t="s">
-        <v>1816</v>
+        <v>1822</v>
       </c>
       <c r="D1081"/>
       <c r="E1081"/>
@@ -24494,10 +24518,10 @@
     </row>
     <row r="1083">
       <c r="A1083" t="s">
-        <v>1817</v>
+        <v>1823</v>
       </c>
       <c r="B1083" t="s">
-        <v>1818</v>
+        <v>1824</v>
       </c>
       <c r="C1083" t="s">
         <v>15</v>
@@ -24513,7 +24537,7 @@
     <row r="1084">
       <c r="A1084"/>
       <c r="B1084" t="s">
-        <v>1819</v>
+        <v>1825</v>
       </c>
       <c r="C1084" t="s">
         <v>18</v>
@@ -24529,7 +24553,7 @@
     <row r="1085">
       <c r="A1085"/>
       <c r="B1085" t="s">
-        <v>1820</v>
+        <v>1826</v>
       </c>
       <c r="C1085" t="s">
         <v>21</v>
@@ -24547,7 +24571,7 @@
     <row r="1086">
       <c r="A1086"/>
       <c r="B1086" t="s">
-        <v>1821</v>
+        <v>1827</v>
       </c>
       <c r="C1086" t="s">
         <v>24</v>
@@ -24563,7 +24587,7 @@
     <row r="1087" ht="77" customHeight="1">
       <c r="A1087" s="1"/>
       <c r="B1087" s="1" t="s">
-        <v>1822</v>
+        <v>1828</v>
       </c>
       <c r="C1087" s="1" t="s">
         <v>26</v>
@@ -24579,7 +24603,7 @@
     <row r="1088" ht="77" customHeight="1">
       <c r="A1088" s="1"/>
       <c r="B1088" s="1" t="s">
-        <v>1823</v>
+        <v>1829</v>
       </c>
       <c r="C1088" s="1" t="s">
         <v>29</v>
@@ -24595,7 +24619,7 @@
     <row r="1089" ht="77" customHeight="1">
       <c r="A1089" s="1"/>
       <c r="B1089" s="1" t="s">
-        <v>1824</v>
+        <v>1830</v>
       </c>
       <c r="C1089" s="1" t="s">
         <v>31</v>
@@ -24611,7 +24635,7 @@
     <row r="1090" ht="77" customHeight="1">
       <c r="A1090" s="1"/>
       <c r="B1090" s="1" t="s">
-        <v>1825</v>
+        <v>1831</v>
       </c>
       <c r="C1090" s="1" t="s">
         <v>33</v>
@@ -24627,7 +24651,7 @@
     <row r="1091" ht="77" customHeight="1">
       <c r="A1091" s="1"/>
       <c r="B1091" s="1" t="s">
-        <v>1826</v>
+        <v>1832</v>
       </c>
       <c r="C1091" s="1" t="s">
         <v>35</v>
@@ -24643,7 +24667,7 @@
     <row r="1092" ht="77" customHeight="1">
       <c r="A1092" s="1"/>
       <c r="B1092" s="1" t="s">
-        <v>1827</v>
+        <v>1833</v>
       </c>
       <c r="C1092" s="1" t="s">
         <v>37</v>
@@ -24659,7 +24683,7 @@
     <row r="1093" ht="77" customHeight="1">
       <c r="A1093" s="1"/>
       <c r="B1093" s="1" t="s">
-        <v>1828</v>
+        <v>1834</v>
       </c>
       <c r="C1093" s="1" t="s">
         <v>39</v>
@@ -24675,7 +24699,7 @@
     <row r="1094" ht="77" customHeight="1">
       <c r="A1094" s="1"/>
       <c r="B1094" s="1" t="s">
-        <v>1829</v>
+        <v>1835</v>
       </c>
       <c r="C1094" s="1" t="s">
         <v>41</v>
@@ -24691,7 +24715,7 @@
     <row r="1095" ht="77" customHeight="1">
       <c r="A1095" s="1"/>
       <c r="B1095" s="1" t="s">
-        <v>1830</v>
+        <v>1836</v>
       </c>
       <c r="C1095" s="1" t="s">
         <v>44</v>
@@ -24709,7 +24733,7 @@
     <row r="1096" ht="77" customHeight="1">
       <c r="A1096" s="1"/>
       <c r="B1096" s="1" t="s">
-        <v>1831</v>
+        <v>1837</v>
       </c>
       <c r="C1096" s="1" t="s">
         <v>46</v>
@@ -24727,7 +24751,7 @@
     <row r="1097">
       <c r="A1097"/>
       <c r="B1097" t="s">
-        <v>1832</v>
+        <v>1838</v>
       </c>
       <c r="C1097" t="s">
         <v>236</v>
@@ -24743,7 +24767,7 @@
     <row r="1098">
       <c r="A1098"/>
       <c r="B1098" t="s">
-        <v>1833</v>
+        <v>1839</v>
       </c>
       <c r="C1098" t="s">
         <v>238</v>
@@ -24759,7 +24783,7 @@
     <row r="1099">
       <c r="A1099"/>
       <c r="B1099" t="s">
-        <v>1834</v>
+        <v>1840</v>
       </c>
       <c r="C1099" t="s">
         <v>48</v>
@@ -24775,7 +24799,7 @@
     <row r="1100">
       <c r="A1100"/>
       <c r="B1100" t="s">
-        <v>1835</v>
+        <v>1841</v>
       </c>
       <c r="C1100" t="s">
         <v>718</v>
@@ -24791,7 +24815,7 @@
     <row r="1101">
       <c r="A1101"/>
       <c r="B1101" t="s">
-        <v>1836</v>
+        <v>1842</v>
       </c>
       <c r="C1101" t="s">
         <v>720</v>
@@ -24807,7 +24831,7 @@
     <row r="1102" ht="77" customHeight="1">
       <c r="A1102" s="1"/>
       <c r="B1102" s="1" t="s">
-        <v>1837</v>
+        <v>1843</v>
       </c>
       <c r="C1102" s="1" t="s">
         <v>722</v>
@@ -24823,7 +24847,7 @@
     <row r="1103" ht="77" customHeight="1">
       <c r="A1103" s="1"/>
       <c r="B1103" s="1" t="s">
-        <v>1838</v>
+        <v>1844</v>
       </c>
       <c r="C1103" s="1" t="s">
         <v>724</v>
@@ -24839,7 +24863,7 @@
     <row r="1104" ht="77" customHeight="1">
       <c r="A1104" s="1"/>
       <c r="B1104" s="1" t="s">
-        <v>1839</v>
+        <v>1845</v>
       </c>
       <c r="C1104" s="1" t="s">
         <v>726</v>
@@ -24855,7 +24879,7 @@
     <row r="1105" ht="77" customHeight="1">
       <c r="A1105" s="1"/>
       <c r="B1105" s="1" t="s">
-        <v>1840</v>
+        <v>1846</v>
       </c>
       <c r="C1105" s="1" t="s">
         <v>728</v>
@@ -24871,7 +24895,7 @@
     <row r="1106" ht="77" customHeight="1">
       <c r="A1106" s="1"/>
       <c r="B1106" s="1" t="s">
-        <v>1841</v>
+        <v>1847</v>
       </c>
       <c r="C1106" s="1" t="s">
         <v>730</v>
@@ -24887,7 +24911,7 @@
     <row r="1107" ht="77" customHeight="1">
       <c r="A1107" s="1"/>
       <c r="B1107" s="1" t="s">
-        <v>1842</v>
+        <v>1848</v>
       </c>
       <c r="C1107" s="1" t="s">
         <v>732</v>
@@ -24903,7 +24927,7 @@
     <row r="1108" ht="77" customHeight="1">
       <c r="A1108" s="1"/>
       <c r="B1108" s="1" t="s">
-        <v>1843</v>
+        <v>1849</v>
       </c>
       <c r="C1108" s="1" t="s">
         <v>734</v>
@@ -24919,7 +24943,7 @@
     <row r="1109" ht="77" customHeight="1">
       <c r="A1109" s="1"/>
       <c r="B1109" s="1" t="s">
-        <v>1844</v>
+        <v>1850</v>
       </c>
       <c r="C1109" s="1" t="s">
         <v>736</v>
@@ -24935,7 +24959,7 @@
     <row r="1110">
       <c r="A1110"/>
       <c r="B1110" t="s">
-        <v>1845</v>
+        <v>1851</v>
       </c>
       <c r="C1110" t="s">
         <v>738</v>
@@ -24951,7 +24975,7 @@
     <row r="1111">
       <c r="A1111"/>
       <c r="B1111" t="s">
-        <v>1846</v>
+        <v>1852</v>
       </c>
       <c r="C1111" t="s">
         <v>56</v>
@@ -24967,7 +24991,7 @@
     <row r="1112">
       <c r="A1112"/>
       <c r="B1112" t="s">
-        <v>1847</v>
+        <v>1853</v>
       </c>
       <c r="C1112" t="s">
         <v>597</v>
@@ -24983,7 +25007,7 @@
     <row r="1113">
       <c r="A1113"/>
       <c r="B1113" t="s">
-        <v>1848</v>
+        <v>1854</v>
       </c>
       <c r="C1113" t="s">
         <v>261</v>
@@ -24999,7 +25023,7 @@
     <row r="1114">
       <c r="A1114"/>
       <c r="B1114" t="s">
-        <v>1849</v>
+        <v>1855</v>
       </c>
       <c r="C1114" t="s">
         <v>263</v>
@@ -25015,7 +25039,7 @@
     <row r="1115">
       <c r="A1115"/>
       <c r="B1115" t="s">
-        <v>1850</v>
+        <v>1856</v>
       </c>
       <c r="C1115" t="s">
         <v>265</v>
@@ -25031,7 +25055,7 @@
     <row r="1116">
       <c r="A1116"/>
       <c r="B1116" t="s">
-        <v>1851</v>
+        <v>1857</v>
       </c>
       <c r="C1116" t="s">
         <v>267</v>
@@ -25047,7 +25071,7 @@
     <row r="1117">
       <c r="A1117"/>
       <c r="B1117" t="s">
-        <v>1852</v>
+        <v>1858</v>
       </c>
       <c r="C1117" t="s">
         <v>269</v>
@@ -25063,7 +25087,7 @@
     <row r="1118">
       <c r="A1118"/>
       <c r="B1118" t="s">
-        <v>1853</v>
+        <v>1859</v>
       </c>
       <c r="C1118" t="s">
         <v>281</v>
@@ -25079,7 +25103,7 @@
     <row r="1119">
       <c r="A1119"/>
       <c r="B1119" t="s">
-        <v>1854</v>
+        <v>1860</v>
       </c>
       <c r="C1119" t="s">
         <v>283</v>
@@ -25095,7 +25119,7 @@
     <row r="1120">
       <c r="A1120"/>
       <c r="B1120" t="s">
-        <v>1855</v>
+        <v>1861</v>
       </c>
       <c r="C1120" t="s">
         <v>285</v>
@@ -25111,7 +25135,7 @@
     <row r="1121">
       <c r="A1121"/>
       <c r="B1121" t="s">
-        <v>1856</v>
+        <v>1862</v>
       </c>
       <c r="C1121" t="s">
         <v>287</v>
@@ -25127,7 +25151,7 @@
     <row r="1122">
       <c r="A1122"/>
       <c r="B1122" t="s">
-        <v>1857</v>
+        <v>1863</v>
       </c>
       <c r="C1122" t="s">
         <v>289</v>
@@ -25143,7 +25167,7 @@
     <row r="1123">
       <c r="A1123"/>
       <c r="B1123" t="s">
-        <v>1858</v>
+        <v>1864</v>
       </c>
       <c r="C1123" t="s">
         <v>662</v>
@@ -25161,7 +25185,7 @@
     <row r="1124">
       <c r="A1124"/>
       <c r="B1124" t="s">
-        <v>1859</v>
+        <v>1865</v>
       </c>
       <c r="C1124" t="s">
         <v>664</v>
@@ -25177,7 +25201,7 @@
     <row r="1125">
       <c r="A1125"/>
       <c r="B1125" t="s">
-        <v>1860</v>
+        <v>1866</v>
       </c>
       <c r="C1125" t="s">
         <v>666</v>
@@ -25193,7 +25217,7 @@
     <row r="1126" ht="77" customHeight="1">
       <c r="A1126" s="1"/>
       <c r="B1126" s="1" t="s">
-        <v>1861</v>
+        <v>1867</v>
       </c>
       <c r="C1126" s="1" t="s">
         <v>668</v>
@@ -25209,7 +25233,7 @@
     <row r="1127" ht="77" customHeight="1">
       <c r="A1127" s="1"/>
       <c r="B1127" s="1" t="s">
-        <v>1862</v>
+        <v>1868</v>
       </c>
       <c r="C1127" s="1" t="s">
         <v>670</v>
@@ -25225,7 +25249,7 @@
     <row r="1128" ht="77" customHeight="1">
       <c r="A1128" s="1"/>
       <c r="B1128" s="1" t="s">
-        <v>1863</v>
+        <v>1869</v>
       </c>
       <c r="C1128" s="1" t="s">
         <v>672</v>
@@ -25241,7 +25265,7 @@
     <row r="1129" ht="77" customHeight="1">
       <c r="A1129" s="1"/>
       <c r="B1129" s="1" t="s">
-        <v>1864</v>
+        <v>1870</v>
       </c>
       <c r="C1129" s="1" t="s">
         <v>674</v>
@@ -25257,7 +25281,7 @@
     <row r="1130" ht="77" customHeight="1">
       <c r="A1130" s="1"/>
       <c r="B1130" s="1" t="s">
-        <v>1865</v>
+        <v>1871</v>
       </c>
       <c r="C1130" s="1" t="s">
         <v>676</v>
@@ -25273,7 +25297,7 @@
     <row r="1131" ht="77" customHeight="1">
       <c r="A1131" s="1"/>
       <c r="B1131" s="1" t="s">
-        <v>1866</v>
+        <v>1872</v>
       </c>
       <c r="C1131" s="1" t="s">
         <v>678</v>
@@ -25289,7 +25313,7 @@
     <row r="1132" ht="77" customHeight="1">
       <c r="A1132" s="1"/>
       <c r="B1132" s="1" t="s">
-        <v>1867</v>
+        <v>1873</v>
       </c>
       <c r="C1132" s="1" t="s">
         <v>680</v>
@@ -25305,7 +25329,7 @@
     <row r="1133" ht="77" customHeight="1">
       <c r="A1133" s="1"/>
       <c r="B1133" s="1" t="s">
-        <v>1868</v>
+        <v>1874</v>
       </c>
       <c r="C1133" s="1" t="s">
         <v>682</v>
@@ -25321,7 +25345,7 @@
     <row r="1134">
       <c r="A1134"/>
       <c r="B1134" t="s">
-        <v>1869</v>
+        <v>1875</v>
       </c>
       <c r="C1134" t="s">
         <v>684</v>
@@ -25337,10 +25361,10 @@
     <row r="1135">
       <c r="A1135"/>
       <c r="B1135" t="s">
-        <v>1870</v>
+        <v>1876</v>
       </c>
       <c r="C1135" t="s">
-        <v>1662</v>
+        <v>1668</v>
       </c>
       <c r="D1135"/>
       <c r="E1135"/>
@@ -25353,10 +25377,10 @@
     <row r="1136">
       <c r="A1136"/>
       <c r="B1136" t="s">
-        <v>1871</v>
+        <v>1877</v>
       </c>
       <c r="C1136" t="s">
-        <v>1664</v>
+        <v>1670</v>
       </c>
       <c r="D1136"/>
       <c r="E1136"/>
@@ -25369,10 +25393,10 @@
     <row r="1137" ht="77" customHeight="1">
       <c r="A1137" s="1"/>
       <c r="B1137" s="1" t="s">
-        <v>1872</v>
+        <v>1878</v>
       </c>
       <c r="C1137" s="1" t="s">
-        <v>1666</v>
+        <v>1672</v>
       </c>
       <c r="D1137" s="1"/>
       <c r="E1137" s="1"/>
@@ -25385,10 +25409,10 @@
     <row r="1138" ht="77" customHeight="1">
       <c r="A1138" s="1"/>
       <c r="B1138" s="1" t="s">
-        <v>1873</v>
+        <v>1879</v>
       </c>
       <c r="C1138" s="1" t="s">
-        <v>1668</v>
+        <v>1674</v>
       </c>
       <c r="D1138" s="1"/>
       <c r="E1138" s="1"/>
@@ -25401,10 +25425,10 @@
     <row r="1139" ht="77" customHeight="1">
       <c r="A1139" s="1"/>
       <c r="B1139" s="1" t="s">
-        <v>1874</v>
+        <v>1880</v>
       </c>
       <c r="C1139" s="1" t="s">
-        <v>1670</v>
+        <v>1676</v>
       </c>
       <c r="D1139" s="1"/>
       <c r="E1139" s="1"/>
@@ -25417,10 +25441,10 @@
     <row r="1140" ht="77" customHeight="1">
       <c r="A1140" s="1"/>
       <c r="B1140" s="1" t="s">
-        <v>1875</v>
+        <v>1881</v>
       </c>
       <c r="C1140" s="1" t="s">
-        <v>1672</v>
+        <v>1678</v>
       </c>
       <c r="D1140" s="1"/>
       <c r="E1140" s="1"/>
@@ -25433,10 +25457,10 @@
     <row r="1141" ht="77" customHeight="1">
       <c r="A1141" s="1"/>
       <c r="B1141" s="1" t="s">
-        <v>1876</v>
+        <v>1882</v>
       </c>
       <c r="C1141" s="1" t="s">
-        <v>1674</v>
+        <v>1680</v>
       </c>
       <c r="D1141" s="1"/>
       <c r="E1141" s="1"/>
@@ -25449,10 +25473,10 @@
     <row r="1142" ht="77" customHeight="1">
       <c r="A1142" s="1"/>
       <c r="B1142" s="1" t="s">
-        <v>1877</v>
+        <v>1883</v>
       </c>
       <c r="C1142" s="1" t="s">
-        <v>1676</v>
+        <v>1682</v>
       </c>
       <c r="D1142" s="1"/>
       <c r="E1142" s="1"/>
@@ -25465,10 +25489,10 @@
     <row r="1143" ht="77" customHeight="1">
       <c r="A1143" s="1"/>
       <c r="B1143" s="1" t="s">
-        <v>1878</v>
+        <v>1884</v>
       </c>
       <c r="C1143" s="1" t="s">
-        <v>1678</v>
+        <v>1684</v>
       </c>
       <c r="D1143" s="1"/>
       <c r="E1143" s="1"/>
@@ -25481,10 +25505,10 @@
     <row r="1144" ht="77" customHeight="1">
       <c r="A1144" s="1"/>
       <c r="B1144" s="1" t="s">
-        <v>1879</v>
+        <v>1885</v>
       </c>
       <c r="C1144" s="1" t="s">
-        <v>1680</v>
+        <v>1686</v>
       </c>
       <c r="D1144" s="1"/>
       <c r="E1144" s="1"/>
@@ -25497,10 +25521,10 @@
     <row r="1145">
       <c r="A1145"/>
       <c r="B1145" t="s">
-        <v>1880</v>
+        <v>1886</v>
       </c>
       <c r="C1145" t="s">
-        <v>1682</v>
+        <v>1688</v>
       </c>
       <c r="D1145"/>
       <c r="E1145"/>
@@ -25513,10 +25537,10 @@
     <row r="1146">
       <c r="A1146"/>
       <c r="B1146" t="s">
-        <v>1881</v>
+        <v>1887</v>
       </c>
       <c r="C1146" t="s">
-        <v>1882</v>
+        <v>1888</v>
       </c>
       <c r="D1146"/>
       <c r="E1146"/>
@@ -25529,10 +25553,10 @@
     <row r="1147">
       <c r="A1147"/>
       <c r="B1147" t="s">
-        <v>1883</v>
+        <v>1889</v>
       </c>
       <c r="C1147" t="s">
-        <v>1884</v>
+        <v>1890</v>
       </c>
       <c r="D1147"/>
       <c r="E1147"/>
@@ -25545,10 +25569,10 @@
     <row r="1148">
       <c r="A1148"/>
       <c r="B1148" t="s">
-        <v>1885</v>
+        <v>1891</v>
       </c>
       <c r="C1148" t="s">
-        <v>1886</v>
+        <v>1892</v>
       </c>
       <c r="D1148"/>
       <c r="E1148"/>
@@ -25561,10 +25585,10 @@
     <row r="1149">
       <c r="A1149"/>
       <c r="B1149" t="s">
-        <v>1887</v>
+        <v>1893</v>
       </c>
       <c r="C1149" t="s">
-        <v>1888</v>
+        <v>1894</v>
       </c>
       <c r="D1149"/>
       <c r="E1149"/>
@@ -25577,10 +25601,10 @@
     <row r="1150">
       <c r="A1150"/>
       <c r="B1150" t="s">
-        <v>1889</v>
+        <v>1895</v>
       </c>
       <c r="C1150" t="s">
-        <v>1890</v>
+        <v>1896</v>
       </c>
       <c r="D1150"/>
       <c r="E1150"/>
@@ -25602,10 +25626,10 @@
     </row>
     <row r="1152">
       <c r="A1152" t="s">
-        <v>1891</v>
+        <v>1897</v>
       </c>
       <c r="B1152" t="s">
-        <v>1892</v>
+        <v>1898</v>
       </c>
       <c r="C1152" t="s">
         <v>15</v>
@@ -25621,7 +25645,7 @@
     <row r="1153">
       <c r="A1153"/>
       <c r="B1153" t="s">
-        <v>1893</v>
+        <v>1899</v>
       </c>
       <c r="C1153" t="s">
         <v>18</v>
@@ -25637,7 +25661,7 @@
     <row r="1154">
       <c r="A1154"/>
       <c r="B1154" t="s">
-        <v>1894</v>
+        <v>1900</v>
       </c>
       <c r="C1154" t="s">
         <v>21</v>
@@ -25655,7 +25679,7 @@
     <row r="1155">
       <c r="A1155"/>
       <c r="B1155" t="s">
-        <v>1895</v>
+        <v>1901</v>
       </c>
       <c r="C1155" t="s">
         <v>24</v>
@@ -25671,7 +25695,7 @@
     <row r="1156" ht="77" customHeight="1">
       <c r="A1156" s="1"/>
       <c r="B1156" s="1" t="s">
-        <v>1896</v>
+        <v>1902</v>
       </c>
       <c r="C1156" s="1" t="s">
         <v>26</v>
@@ -25687,7 +25711,7 @@
     <row r="1157" ht="77" customHeight="1">
       <c r="A1157" s="1"/>
       <c r="B1157" s="1" t="s">
-        <v>1897</v>
+        <v>1903</v>
       </c>
       <c r="C1157" s="1" t="s">
         <v>29</v>
@@ -25703,7 +25727,7 @@
     <row r="1158" ht="77" customHeight="1">
       <c r="A1158" s="1"/>
       <c r="B1158" s="1" t="s">
-        <v>1898</v>
+        <v>1904</v>
       </c>
       <c r="C1158" s="1" t="s">
         <v>31</v>
@@ -25719,7 +25743,7 @@
     <row r="1159" ht="77" customHeight="1">
       <c r="A1159" s="1"/>
       <c r="B1159" s="1" t="s">
-        <v>1899</v>
+        <v>1905</v>
       </c>
       <c r="C1159" s="1" t="s">
         <v>33</v>
@@ -25735,7 +25759,7 @@
     <row r="1160" ht="77" customHeight="1">
       <c r="A1160" s="1"/>
       <c r="B1160" s="1" t="s">
-        <v>1900</v>
+        <v>1906</v>
       </c>
       <c r="C1160" s="1" t="s">
         <v>35</v>
@@ -25751,7 +25775,7 @@
     <row r="1161" ht="77" customHeight="1">
       <c r="A1161" s="1"/>
       <c r="B1161" s="1" t="s">
-        <v>1901</v>
+        <v>1907</v>
       </c>
       <c r="C1161" s="1" t="s">
         <v>37</v>
@@ -25767,7 +25791,7 @@
     <row r="1162" ht="77" customHeight="1">
       <c r="A1162" s="1"/>
       <c r="B1162" s="1" t="s">
-        <v>1902</v>
+        <v>1908</v>
       </c>
       <c r="C1162" s="1" t="s">
         <v>39</v>
@@ -25783,7 +25807,7 @@
     <row r="1163" ht="77" customHeight="1">
       <c r="A1163" s="1"/>
       <c r="B1163" s="1" t="s">
-        <v>1903</v>
+        <v>1909</v>
       </c>
       <c r="C1163" s="1" t="s">
         <v>41</v>
@@ -25799,7 +25823,7 @@
     <row r="1164" ht="77" customHeight="1">
       <c r="A1164" s="1"/>
       <c r="B1164" s="1" t="s">
-        <v>1904</v>
+        <v>1910</v>
       </c>
       <c r="C1164" s="1" t="s">
         <v>44</v>
@@ -25817,7 +25841,7 @@
     <row r="1165" ht="77" customHeight="1">
       <c r="A1165" s="1"/>
       <c r="B1165" s="1" t="s">
-        <v>1905</v>
+        <v>1911</v>
       </c>
       <c r="C1165" s="1" t="s">
         <v>46</v>
@@ -25835,7 +25859,7 @@
     <row r="1166">
       <c r="A1166"/>
       <c r="B1166" t="s">
-        <v>1906</v>
+        <v>1912</v>
       </c>
       <c r="C1166" t="s">
         <v>236</v>
@@ -25851,7 +25875,7 @@
     <row r="1167">
       <c r="A1167"/>
       <c r="B1167" t="s">
-        <v>1907</v>
+        <v>1913</v>
       </c>
       <c r="C1167" t="s">
         <v>238</v>
@@ -25867,7 +25891,7 @@
     <row r="1168">
       <c r="A1168"/>
       <c r="B1168" t="s">
-        <v>1908</v>
+        <v>1914</v>
       </c>
       <c r="C1168" t="s">
         <v>48</v>
@@ -25883,7 +25907,7 @@
     <row r="1169">
       <c r="A1169"/>
       <c r="B1169" t="s">
-        <v>1909</v>
+        <v>1915</v>
       </c>
       <c r="C1169" t="s">
         <v>50</v>
@@ -25899,7 +25923,7 @@
     <row r="1170">
       <c r="A1170"/>
       <c r="B1170" t="s">
-        <v>1910</v>
+        <v>1916</v>
       </c>
       <c r="C1170" t="s">
         <v>718</v>
@@ -25915,7 +25939,7 @@
     <row r="1171">
       <c r="A1171"/>
       <c r="B1171" t="s">
-        <v>1911</v>
+        <v>1917</v>
       </c>
       <c r="C1171" t="s">
         <v>720</v>
@@ -25931,7 +25955,7 @@
     <row r="1172" ht="77" customHeight="1">
       <c r="A1172" s="1"/>
       <c r="B1172" s="1" t="s">
-        <v>1912</v>
+        <v>1918</v>
       </c>
       <c r="C1172" s="1" t="s">
         <v>722</v>
@@ -25947,7 +25971,7 @@
     <row r="1173" ht="77" customHeight="1">
       <c r="A1173" s="1"/>
       <c r="B1173" s="1" t="s">
-        <v>1913</v>
+        <v>1919</v>
       </c>
       <c r="C1173" s="1" t="s">
         <v>724</v>
@@ -25963,7 +25987,7 @@
     <row r="1174" ht="77" customHeight="1">
       <c r="A1174" s="1"/>
       <c r="B1174" s="1" t="s">
-        <v>1914</v>
+        <v>1920</v>
       </c>
       <c r="C1174" s="1" t="s">
         <v>726</v>
@@ -25979,7 +26003,7 @@
     <row r="1175" ht="77" customHeight="1">
       <c r="A1175" s="1"/>
       <c r="B1175" s="1" t="s">
-        <v>1915</v>
+        <v>1921</v>
       </c>
       <c r="C1175" s="1" t="s">
         <v>728</v>
@@ -25995,7 +26019,7 @@
     <row r="1176" ht="77" customHeight="1">
       <c r="A1176" s="1"/>
       <c r="B1176" s="1" t="s">
-        <v>1916</v>
+        <v>1922</v>
       </c>
       <c r="C1176" s="1" t="s">
         <v>730</v>
@@ -26011,7 +26035,7 @@
     <row r="1177" ht="77" customHeight="1">
       <c r="A1177" s="1"/>
       <c r="B1177" s="1" t="s">
-        <v>1917</v>
+        <v>1923</v>
       </c>
       <c r="C1177" s="1" t="s">
         <v>732</v>
@@ -26027,7 +26051,7 @@
     <row r="1178" ht="77" customHeight="1">
       <c r="A1178" s="1"/>
       <c r="B1178" s="1" t="s">
-        <v>1918</v>
+        <v>1924</v>
       </c>
       <c r="C1178" s="1" t="s">
         <v>734</v>
@@ -26043,7 +26067,7 @@
     <row r="1179" ht="77" customHeight="1">
       <c r="A1179" s="1"/>
       <c r="B1179" s="1" t="s">
-        <v>1919</v>
+        <v>1925</v>
       </c>
       <c r="C1179" s="1" t="s">
         <v>736</v>
@@ -26059,7 +26083,7 @@
     <row r="1180">
       <c r="A1180"/>
       <c r="B1180" t="s">
-        <v>1920</v>
+        <v>1926</v>
       </c>
       <c r="C1180" t="s">
         <v>738</v>
@@ -26075,7 +26099,7 @@
     <row r="1181">
       <c r="A1181"/>
       <c r="B1181" t="s">
-        <v>1921</v>
+        <v>1927</v>
       </c>
       <c r="C1181" t="s">
         <v>56</v>
@@ -26091,7 +26115,7 @@
     <row r="1182">
       <c r="A1182"/>
       <c r="B1182" t="s">
-        <v>1922</v>
+        <v>1928</v>
       </c>
       <c r="C1182" t="s">
         <v>585</v>
@@ -26107,7 +26131,7 @@
     <row r="1183">
       <c r="A1183"/>
       <c r="B1183" t="s">
-        <v>1923</v>
+        <v>1929</v>
       </c>
       <c r="C1183" t="s">
         <v>587</v>
@@ -26123,7 +26147,7 @@
     <row r="1184">
       <c r="A1184"/>
       <c r="B1184" t="s">
-        <v>1924</v>
+        <v>1930</v>
       </c>
       <c r="C1184" t="s">
         <v>589</v>
@@ -26139,7 +26163,7 @@
     <row r="1185">
       <c r="A1185"/>
       <c r="B1185" t="s">
-        <v>1925</v>
+        <v>1931</v>
       </c>
       <c r="C1185" t="s">
         <v>591</v>
@@ -26155,7 +26179,7 @@
     <row r="1186">
       <c r="A1186"/>
       <c r="B1186" t="s">
-        <v>1926</v>
+        <v>1932</v>
       </c>
       <c r="C1186" t="s">
         <v>593</v>
@@ -26171,7 +26195,7 @@
     <row r="1187">
       <c r="A1187"/>
       <c r="B1187" t="s">
-        <v>1927</v>
+        <v>1933</v>
       </c>
       <c r="C1187" t="s">
         <v>261</v>
@@ -26187,7 +26211,7 @@
     <row r="1188">
       <c r="A1188"/>
       <c r="B1188" t="s">
-        <v>1928</v>
+        <v>1934</v>
       </c>
       <c r="C1188" t="s">
         <v>263</v>
@@ -26203,7 +26227,7 @@
     <row r="1189">
       <c r="A1189"/>
       <c r="B1189" t="s">
-        <v>1929</v>
+        <v>1935</v>
       </c>
       <c r="C1189" t="s">
         <v>265</v>
@@ -26219,7 +26243,7 @@
     <row r="1190">
       <c r="A1190"/>
       <c r="B1190" t="s">
-        <v>1930</v>
+        <v>1936</v>
       </c>
       <c r="C1190" t="s">
         <v>267</v>
@@ -26235,7 +26259,7 @@
     <row r="1191">
       <c r="A1191"/>
       <c r="B1191" t="s">
-        <v>1931</v>
+        <v>1937</v>
       </c>
       <c r="C1191" t="s">
         <v>269</v>
@@ -26251,7 +26275,7 @@
     <row r="1192">
       <c r="A1192"/>
       <c r="B1192" t="s">
-        <v>1932</v>
+        <v>1938</v>
       </c>
       <c r="C1192" t="s">
         <v>281</v>
@@ -26267,7 +26291,7 @@
     <row r="1193">
       <c r="A1193"/>
       <c r="B1193" t="s">
-        <v>1933</v>
+        <v>1939</v>
       </c>
       <c r="C1193" t="s">
         <v>283</v>
@@ -26283,7 +26307,7 @@
     <row r="1194">
       <c r="A1194"/>
       <c r="B1194" t="s">
-        <v>1934</v>
+        <v>1940</v>
       </c>
       <c r="C1194" t="s">
         <v>285</v>
@@ -26299,7 +26323,7 @@
     <row r="1195">
       <c r="A1195"/>
       <c r="B1195" t="s">
-        <v>1935</v>
+        <v>1941</v>
       </c>
       <c r="C1195" t="s">
         <v>287</v>
@@ -26315,7 +26339,7 @@
     <row r="1196">
       <c r="A1196"/>
       <c r="B1196" t="s">
-        <v>1936</v>
+        <v>1942</v>
       </c>
       <c r="C1196" t="s">
         <v>289</v>
@@ -26331,10 +26355,10 @@
     <row r="1197">
       <c r="A1197"/>
       <c r="B1197" t="s">
-        <v>1937</v>
+        <v>1943</v>
       </c>
       <c r="C1197" t="s">
-        <v>1938</v>
+        <v>1944</v>
       </c>
       <c r="D1197"/>
       <c r="E1197" t="s">
@@ -26349,10 +26373,10 @@
     <row r="1198">
       <c r="A1198"/>
       <c r="B1198" t="s">
-        <v>1939</v>
+        <v>1945</v>
       </c>
       <c r="C1198" t="s">
-        <v>1940</v>
+        <v>1946</v>
       </c>
       <c r="D1198"/>
       <c r="E1198" t="s">
@@ -26367,10 +26391,10 @@
     <row r="1199">
       <c r="A1199"/>
       <c r="B1199" t="s">
-        <v>1941</v>
+        <v>1947</v>
       </c>
       <c r="C1199" t="s">
-        <v>1942</v>
+        <v>1948</v>
       </c>
       <c r="D1199"/>
       <c r="E1199" t="s">
@@ -26385,7 +26409,7 @@
     <row r="1200">
       <c r="A1200"/>
       <c r="B1200" t="s">
-        <v>1943</v>
+        <v>1949</v>
       </c>
       <c r="C1200" t="s">
         <v>686</v>
@@ -26401,7 +26425,7 @@
     <row r="1201">
       <c r="A1201"/>
       <c r="B1201" t="s">
-        <v>1944</v>
+        <v>1950</v>
       </c>
       <c r="C1201" t="s">
         <v>688</v>
@@ -26417,7 +26441,7 @@
     <row r="1202">
       <c r="A1202"/>
       <c r="B1202" t="s">
-        <v>1945</v>
+        <v>1951</v>
       </c>
       <c r="C1202" t="s">
         <v>690</v>
@@ -26433,7 +26457,7 @@
     <row r="1203">
       <c r="A1203"/>
       <c r="B1203" t="s">
-        <v>1946</v>
+        <v>1952</v>
       </c>
       <c r="C1203" t="s">
         <v>692</v>
@@ -26449,7 +26473,7 @@
     <row r="1204">
       <c r="A1204"/>
       <c r="B1204" t="s">
-        <v>1947</v>
+        <v>1953</v>
       </c>
       <c r="C1204" t="s">
         <v>694</v>
@@ -26465,7 +26489,7 @@
     <row r="1205">
       <c r="A1205"/>
       <c r="B1205" t="s">
-        <v>1948</v>
+        <v>1954</v>
       </c>
       <c r="C1205" t="s">
         <v>696</v>
@@ -26481,7 +26505,7 @@
     <row r="1206">
       <c r="A1206"/>
       <c r="B1206" t="s">
-        <v>1949</v>
+        <v>1955</v>
       </c>
       <c r="C1206" t="s">
         <v>698</v>
@@ -26497,7 +26521,7 @@
     <row r="1207" ht="77" customHeight="1">
       <c r="A1207" s="1"/>
       <c r="B1207" s="1" t="s">
-        <v>1950</v>
+        <v>1956</v>
       </c>
       <c r="C1207" s="1" t="s">
         <v>700</v>
@@ -26513,7 +26537,7 @@
     <row r="1208" ht="77" customHeight="1">
       <c r="A1208" s="1"/>
       <c r="B1208" s="1" t="s">
-        <v>1951</v>
+        <v>1957</v>
       </c>
       <c r="C1208" s="1" t="s">
         <v>702</v>
@@ -26529,7 +26553,7 @@
     <row r="1209" ht="77" customHeight="1">
       <c r="A1209" s="1"/>
       <c r="B1209" s="1" t="s">
-        <v>1952</v>
+        <v>1958</v>
       </c>
       <c r="C1209" s="1" t="s">
         <v>704</v>
@@ -26545,7 +26569,7 @@
     <row r="1210" ht="77" customHeight="1">
       <c r="A1210" s="1"/>
       <c r="B1210" s="1" t="s">
-        <v>1953</v>
+        <v>1959</v>
       </c>
       <c r="C1210" s="1" t="s">
         <v>706</v>
@@ -26561,7 +26585,7 @@
     <row r="1211" ht="77" customHeight="1">
       <c r="A1211" s="1"/>
       <c r="B1211" s="1" t="s">
-        <v>1954</v>
+        <v>1960</v>
       </c>
       <c r="C1211" s="1" t="s">
         <v>708</v>
@@ -26577,7 +26601,7 @@
     <row r="1212" ht="77" customHeight="1">
       <c r="A1212" s="1"/>
       <c r="B1212" s="1" t="s">
-        <v>1955</v>
+        <v>1961</v>
       </c>
       <c r="C1212" s="1" t="s">
         <v>710</v>
@@ -26593,7 +26617,7 @@
     <row r="1213" ht="77" customHeight="1">
       <c r="A1213" s="1"/>
       <c r="B1213" s="1" t="s">
-        <v>1956</v>
+        <v>1962</v>
       </c>
       <c r="C1213" s="1" t="s">
         <v>712</v>
@@ -26609,7 +26633,7 @@
     <row r="1214" ht="77" customHeight="1">
       <c r="A1214" s="1"/>
       <c r="B1214" s="1" t="s">
-        <v>1957</v>
+        <v>1963</v>
       </c>
       <c r="C1214" s="1" t="s">
         <v>714</v>
@@ -26625,7 +26649,7 @@
     <row r="1215">
       <c r="A1215"/>
       <c r="B1215" t="s">
-        <v>1958</v>
+        <v>1964</v>
       </c>
       <c r="C1215" t="s">
         <v>716</v>
@@ -26641,7 +26665,7 @@
     <row r="1216">
       <c r="A1216"/>
       <c r="B1216" t="s">
-        <v>1959</v>
+        <v>1965</v>
       </c>
       <c r="C1216" t="s">
         <v>430</v>
@@ -26657,7 +26681,7 @@
     <row r="1217">
       <c r="A1217"/>
       <c r="B1217" t="s">
-        <v>1960</v>
+        <v>1966</v>
       </c>
       <c r="C1217" t="s">
         <v>432</v>
@@ -26673,7 +26697,7 @@
     <row r="1218">
       <c r="A1218"/>
       <c r="B1218" t="s">
-        <v>1961</v>
+        <v>1967</v>
       </c>
       <c r="C1218" t="s">
         <v>434</v>
@@ -26689,7 +26713,7 @@
     <row r="1219" ht="77" customHeight="1">
       <c r="A1219" s="1"/>
       <c r="B1219" s="1" t="s">
-        <v>1962</v>
+        <v>1968</v>
       </c>
       <c r="C1219" s="1" t="s">
         <v>436</v>
@@ -26705,7 +26729,7 @@
     <row r="1220" ht="77" customHeight="1">
       <c r="A1220" s="1"/>
       <c r="B1220" s="1" t="s">
-        <v>1963</v>
+        <v>1969</v>
       </c>
       <c r="C1220" s="1" t="s">
         <v>438</v>
@@ -26721,7 +26745,7 @@
     <row r="1221" ht="77" customHeight="1">
       <c r="A1221" s="1"/>
       <c r="B1221" s="1" t="s">
-        <v>1964</v>
+        <v>1970</v>
       </c>
       <c r="C1221" s="1" t="s">
         <v>440</v>
@@ -26737,7 +26761,7 @@
     <row r="1222" ht="77" customHeight="1">
       <c r="A1222" s="1"/>
       <c r="B1222" s="1" t="s">
-        <v>1965</v>
+        <v>1971</v>
       </c>
       <c r="C1222" s="1" t="s">
         <v>442</v>
@@ -26753,7 +26777,7 @@
     <row r="1223" ht="77" customHeight="1">
       <c r="A1223" s="1"/>
       <c r="B1223" s="1" t="s">
-        <v>1966</v>
+        <v>1972</v>
       </c>
       <c r="C1223" s="1" t="s">
         <v>444</v>
@@ -26769,7 +26793,7 @@
     <row r="1224" ht="77" customHeight="1">
       <c r="A1224" s="1"/>
       <c r="B1224" s="1" t="s">
-        <v>1967</v>
+        <v>1973</v>
       </c>
       <c r="C1224" s="1" t="s">
         <v>446</v>
@@ -26785,7 +26809,7 @@
     <row r="1225" ht="77" customHeight="1">
       <c r="A1225" s="1"/>
       <c r="B1225" s="1" t="s">
-        <v>1968</v>
+        <v>1974</v>
       </c>
       <c r="C1225" s="1" t="s">
         <v>448</v>
@@ -26801,7 +26825,7 @@
     <row r="1226" ht="77" customHeight="1">
       <c r="A1226" s="1"/>
       <c r="B1226" s="1" t="s">
-        <v>1969</v>
+        <v>1975</v>
       </c>
       <c r="C1226" s="1" t="s">
         <v>450</v>
@@ -26817,7 +26841,7 @@
     <row r="1227">
       <c r="A1227"/>
       <c r="B1227" t="s">
-        <v>1970</v>
+        <v>1976</v>
       </c>
       <c r="C1227" t="s">
         <v>452</v>
@@ -26833,7 +26857,7 @@
     <row r="1228">
       <c r="A1228"/>
       <c r="B1228" t="s">
-        <v>1971</v>
+        <v>1977</v>
       </c>
       <c r="C1228" t="s">
         <v>454</v>
@@ -26851,7 +26875,7 @@
     <row r="1229">
       <c r="A1229"/>
       <c r="B1229" t="s">
-        <v>1972</v>
+        <v>1978</v>
       </c>
       <c r="C1229" t="s">
         <v>456</v>
@@ -26876,10 +26900,10 @@
     </row>
     <row r="1231">
       <c r="A1231" t="s">
-        <v>1973</v>
+        <v>1979</v>
       </c>
       <c r="B1231" t="s">
-        <v>1974</v>
+        <v>1980</v>
       </c>
       <c r="C1231" t="s">
         <v>15</v>
@@ -26895,7 +26919,7 @@
     <row r="1232">
       <c r="A1232"/>
       <c r="B1232" t="s">
-        <v>1975</v>
+        <v>1981</v>
       </c>
       <c r="C1232" t="s">
         <v>18</v>
@@ -26911,7 +26935,7 @@
     <row r="1233">
       <c r="A1233"/>
       <c r="B1233" t="s">
-        <v>1976</v>
+        <v>1982</v>
       </c>
       <c r="C1233" t="s">
         <v>21</v>
@@ -26929,7 +26953,7 @@
     <row r="1234">
       <c r="A1234"/>
       <c r="B1234" t="s">
-        <v>1977</v>
+        <v>1983</v>
       </c>
       <c r="C1234" t="s">
         <v>24</v>
@@ -26945,7 +26969,7 @@
     <row r="1235" ht="77" customHeight="1">
       <c r="A1235" s="1"/>
       <c r="B1235" s="1" t="s">
-        <v>1978</v>
+        <v>1984</v>
       </c>
       <c r="C1235" s="1" t="s">
         <v>26</v>
@@ -26961,7 +26985,7 @@
     <row r="1236" ht="77" customHeight="1">
       <c r="A1236" s="1"/>
       <c r="B1236" s="1" t="s">
-        <v>1979</v>
+        <v>1985</v>
       </c>
       <c r="C1236" s="1" t="s">
         <v>29</v>
@@ -26977,7 +27001,7 @@
     <row r="1237" ht="77" customHeight="1">
       <c r="A1237" s="1"/>
       <c r="B1237" s="1" t="s">
-        <v>1980</v>
+        <v>1986</v>
       </c>
       <c r="C1237" s="1" t="s">
         <v>31</v>
@@ -26993,7 +27017,7 @@
     <row r="1238" ht="77" customHeight="1">
       <c r="A1238" s="1"/>
       <c r="B1238" s="1" t="s">
-        <v>1981</v>
+        <v>1987</v>
       </c>
       <c r="C1238" s="1" t="s">
         <v>33</v>
@@ -27009,7 +27033,7 @@
     <row r="1239" ht="77" customHeight="1">
       <c r="A1239" s="1"/>
       <c r="B1239" s="1" t="s">
-        <v>1982</v>
+        <v>1988</v>
       </c>
       <c r="C1239" s="1" t="s">
         <v>35</v>
@@ -27025,7 +27049,7 @@
     <row r="1240" ht="77" customHeight="1">
       <c r="A1240" s="1"/>
       <c r="B1240" s="1" t="s">
-        <v>1983</v>
+        <v>1989</v>
       </c>
       <c r="C1240" s="1" t="s">
         <v>37</v>
@@ -27041,7 +27065,7 @@
     <row r="1241" ht="77" customHeight="1">
       <c r="A1241" s="1"/>
       <c r="B1241" s="1" t="s">
-        <v>1984</v>
+        <v>1990</v>
       </c>
       <c r="C1241" s="1" t="s">
         <v>39</v>
@@ -27057,7 +27081,7 @@
     <row r="1242" ht="77" customHeight="1">
       <c r="A1242" s="1"/>
       <c r="B1242" s="1" t="s">
-        <v>1985</v>
+        <v>1991</v>
       </c>
       <c r="C1242" s="1" t="s">
         <v>41</v>
@@ -27073,7 +27097,7 @@
     <row r="1243" ht="77" customHeight="1">
       <c r="A1243" s="1"/>
       <c r="B1243" s="1" t="s">
-        <v>1986</v>
+        <v>1992</v>
       </c>
       <c r="C1243" s="1" t="s">
         <v>44</v>
@@ -27091,7 +27115,7 @@
     <row r="1244" ht="77" customHeight="1">
       <c r="A1244" s="1"/>
       <c r="B1244" s="1" t="s">
-        <v>1987</v>
+        <v>1993</v>
       </c>
       <c r="C1244" s="1" t="s">
         <v>46</v>
@@ -27109,10 +27133,10 @@
     <row r="1245">
       <c r="A1245"/>
       <c r="B1245" t="s">
-        <v>1988</v>
+        <v>1994</v>
       </c>
       <c r="C1245" t="s">
-        <v>1989</v>
+        <v>1995</v>
       </c>
       <c r="D1245"/>
       <c r="E1245"/>
@@ -27125,7 +27149,7 @@
     <row r="1246">
       <c r="A1246"/>
       <c r="B1246" t="s">
-        <v>1990</v>
+        <v>1996</v>
       </c>
       <c r="C1246" t="s">
         <v>56</v>
@@ -27141,10 +27165,10 @@
     <row r="1247">
       <c r="A1247"/>
       <c r="B1247" t="s">
-        <v>1991</v>
+        <v>1997</v>
       </c>
       <c r="C1247" t="s">
-        <v>1992</v>
+        <v>1998</v>
       </c>
       <c r="D1247"/>
       <c r="E1247"/>
@@ -27157,10 +27181,10 @@
     <row r="1248">
       <c r="A1248"/>
       <c r="B1248" t="s">
-        <v>1993</v>
+        <v>1999</v>
       </c>
       <c r="C1248" t="s">
-        <v>1994</v>
+        <v>2000</v>
       </c>
       <c r="D1248"/>
       <c r="E1248"/>
@@ -27173,10 +27197,10 @@
     <row r="1249">
       <c r="A1249"/>
       <c r="B1249" t="s">
-        <v>1995</v>
+        <v>2001</v>
       </c>
       <c r="C1249" t="s">
-        <v>1996</v>
+        <v>2002</v>
       </c>
       <c r="D1249"/>
       <c r="E1249"/>
@@ -27189,10 +27213,10 @@
     <row r="1250">
       <c r="A1250"/>
       <c r="B1250" t="s">
-        <v>1997</v>
+        <v>2003</v>
       </c>
       <c r="C1250" t="s">
-        <v>1998</v>
+        <v>2004</v>
       </c>
       <c r="D1250"/>
       <c r="E1250"/>
@@ -27205,10 +27229,10 @@
     <row r="1251">
       <c r="A1251"/>
       <c r="B1251" t="s">
-        <v>1999</v>
+        <v>2005</v>
       </c>
       <c r="C1251" t="s">
-        <v>2000</v>
+        <v>2006</v>
       </c>
       <c r="D1251"/>
       <c r="E1251"/>
@@ -27221,7 +27245,7 @@
     <row r="1252">
       <c r="A1252"/>
       <c r="B1252" t="s">
-        <v>2001</v>
+        <v>2007</v>
       </c>
       <c r="C1252" t="s">
         <v>261</v>
@@ -27237,7 +27261,7 @@
     <row r="1253">
       <c r="A1253"/>
       <c r="B1253" t="s">
-        <v>2002</v>
+        <v>2008</v>
       </c>
       <c r="C1253" t="s">
         <v>263</v>
@@ -27253,7 +27277,7 @@
     <row r="1254">
       <c r="A1254"/>
       <c r="B1254" t="s">
-        <v>2003</v>
+        <v>2009</v>
       </c>
       <c r="C1254" t="s">
         <v>265</v>
@@ -27269,7 +27293,7 @@
     <row r="1255">
       <c r="A1255"/>
       <c r="B1255" t="s">
-        <v>2004</v>
+        <v>2010</v>
       </c>
       <c r="C1255" t="s">
         <v>267</v>
@@ -27285,7 +27309,7 @@
     <row r="1256">
       <c r="A1256"/>
       <c r="B1256" t="s">
-        <v>2005</v>
+        <v>2011</v>
       </c>
       <c r="C1256" t="s">
         <v>269</v>
@@ -27301,10 +27325,10 @@
     <row r="1257">
       <c r="A1257"/>
       <c r="B1257" t="s">
-        <v>2006</v>
+        <v>2012</v>
       </c>
       <c r="C1257" t="s">
-        <v>2007</v>
+        <v>2013</v>
       </c>
       <c r="D1257"/>
       <c r="E1257" t="s">
@@ -27319,10 +27343,10 @@
     <row r="1258">
       <c r="A1258"/>
       <c r="B1258" t="s">
-        <v>2008</v>
+        <v>2014</v>
       </c>
       <c r="C1258" t="s">
-        <v>2009</v>
+        <v>2015</v>
       </c>
       <c r="D1258"/>
       <c r="E1258"/>
@@ -27335,10 +27359,10 @@
     <row r="1259">
       <c r="A1259"/>
       <c r="B1259" t="s">
-        <v>2010</v>
+        <v>2016</v>
       </c>
       <c r="C1259" t="s">
-        <v>2011</v>
+        <v>2017</v>
       </c>
       <c r="D1259"/>
       <c r="E1259"/>
@@ -27351,10 +27375,10 @@
     <row r="1260">
       <c r="A1260"/>
       <c r="B1260" t="s">
-        <v>2012</v>
+        <v>2018</v>
       </c>
       <c r="C1260" t="s">
-        <v>2013</v>
+        <v>2019</v>
       </c>
       <c r="D1260"/>
       <c r="E1260"/>
@@ -27367,10 +27391,10 @@
     <row r="1261">
       <c r="A1261"/>
       <c r="B1261" t="s">
-        <v>2014</v>
+        <v>2020</v>
       </c>
       <c r="C1261" t="s">
-        <v>2015</v>
+        <v>2021</v>
       </c>
       <c r="D1261"/>
       <c r="E1261" t="s">
@@ -27385,10 +27409,10 @@
     <row r="1262">
       <c r="A1262"/>
       <c r="B1262" t="s">
-        <v>2016</v>
+        <v>2022</v>
       </c>
       <c r="C1262" t="s">
-        <v>2017</v>
+        <v>2023</v>
       </c>
       <c r="D1262"/>
       <c r="E1262" t="s">
@@ -27403,10 +27427,10 @@
     <row r="1263">
       <c r="A1263"/>
       <c r="B1263" t="s">
-        <v>2018</v>
+        <v>2024</v>
       </c>
       <c r="C1263" t="s">
-        <v>2019</v>
+        <v>2025</v>
       </c>
       <c r="D1263"/>
       <c r="E1263"/>
@@ -27419,10 +27443,10 @@
     <row r="1264">
       <c r="A1264"/>
       <c r="B1264" t="s">
-        <v>2020</v>
+        <v>2026</v>
       </c>
       <c r="C1264" t="s">
-        <v>2021</v>
+        <v>2027</v>
       </c>
       <c r="D1264"/>
       <c r="E1264"/>
@@ -27435,10 +27459,10 @@
     <row r="1265">
       <c r="A1265"/>
       <c r="B1265" t="s">
-        <v>2022</v>
+        <v>2028</v>
       </c>
       <c r="C1265" t="s">
-        <v>2023</v>
+        <v>2029</v>
       </c>
       <c r="D1265"/>
       <c r="E1265"/>
@@ -27451,10 +27475,10 @@
     <row r="1266">
       <c r="A1266"/>
       <c r="B1266" t="s">
-        <v>2024</v>
+        <v>2030</v>
       </c>
       <c r="C1266" t="s">
-        <v>2025</v>
+        <v>2031</v>
       </c>
       <c r="D1266"/>
       <c r="E1266"/>
@@ -27467,10 +27491,10 @@
     <row r="1267">
       <c r="A1267"/>
       <c r="B1267" t="s">
-        <v>2026</v>
+        <v>2032</v>
       </c>
       <c r="C1267" t="s">
-        <v>2027</v>
+        <v>2033</v>
       </c>
       <c r="D1267"/>
       <c r="E1267"/>
@@ -27483,10 +27507,10 @@
     <row r="1268">
       <c r="A1268"/>
       <c r="B1268" t="s">
-        <v>2028</v>
+        <v>2034</v>
       </c>
       <c r="C1268" t="s">
-        <v>2029</v>
+        <v>2035</v>
       </c>
       <c r="D1268"/>
       <c r="E1268"/>
@@ -27499,10 +27523,10 @@
     <row r="1269">
       <c r="A1269"/>
       <c r="B1269" t="s">
-        <v>2030</v>
+        <v>2036</v>
       </c>
       <c r="C1269" t="s">
-        <v>2031</v>
+        <v>2037</v>
       </c>
       <c r="D1269"/>
       <c r="E1269"/>
@@ -27515,10 +27539,10 @@
     <row r="1270" ht="77" customHeight="1">
       <c r="A1270" s="1"/>
       <c r="B1270" s="1" t="s">
-        <v>2032</v>
+        <v>2038</v>
       </c>
       <c r="C1270" s="1" t="s">
-        <v>2033</v>
+        <v>2039</v>
       </c>
       <c r="D1270" s="1"/>
       <c r="E1270" s="1"/>
@@ -27531,10 +27555,10 @@
     <row r="1271" ht="77" customHeight="1">
       <c r="A1271" s="1"/>
       <c r="B1271" s="1" t="s">
-        <v>2034</v>
+        <v>2040</v>
       </c>
       <c r="C1271" s="1" t="s">
-        <v>2035</v>
+        <v>2041</v>
       </c>
       <c r="D1271" s="1"/>
       <c r="E1271" s="1"/>
@@ -27547,10 +27571,10 @@
     <row r="1272" ht="77" customHeight="1">
       <c r="A1272" s="1"/>
       <c r="B1272" s="1" t="s">
-        <v>2036</v>
+        <v>2042</v>
       </c>
       <c r="C1272" s="1" t="s">
-        <v>2037</v>
+        <v>2043</v>
       </c>
       <c r="D1272" s="1"/>
       <c r="E1272" s="1"/>
@@ -27563,10 +27587,10 @@
     <row r="1273" ht="77" customHeight="1">
       <c r="A1273" s="1"/>
       <c r="B1273" s="1" t="s">
-        <v>2038</v>
+        <v>2044</v>
       </c>
       <c r="C1273" s="1" t="s">
-        <v>2039</v>
+        <v>2045</v>
       </c>
       <c r="D1273" s="1"/>
       <c r="E1273" s="1"/>
@@ -27579,10 +27603,10 @@
     <row r="1274" ht="77" customHeight="1">
       <c r="A1274" s="1"/>
       <c r="B1274" s="1" t="s">
-        <v>2040</v>
+        <v>2046</v>
       </c>
       <c r="C1274" s="1" t="s">
-        <v>2041</v>
+        <v>2047</v>
       </c>
       <c r="D1274" s="1"/>
       <c r="E1274" s="1"/>
@@ -27595,10 +27619,10 @@
     <row r="1275" ht="77" customHeight="1">
       <c r="A1275" s="1"/>
       <c r="B1275" s="1" t="s">
-        <v>2042</v>
+        <v>2048</v>
       </c>
       <c r="C1275" s="1" t="s">
-        <v>2043</v>
+        <v>2049</v>
       </c>
       <c r="D1275" s="1"/>
       <c r="E1275" s="1"/>
@@ -27611,10 +27635,10 @@
     <row r="1276" ht="77" customHeight="1">
       <c r="A1276" s="1"/>
       <c r="B1276" s="1" t="s">
-        <v>2044</v>
+        <v>2050</v>
       </c>
       <c r="C1276" s="1" t="s">
-        <v>2045</v>
+        <v>2051</v>
       </c>
       <c r="D1276" s="1"/>
       <c r="E1276" s="1"/>
@@ -27627,10 +27651,10 @@
     <row r="1277" ht="77" customHeight="1">
       <c r="A1277" s="1"/>
       <c r="B1277" s="1" t="s">
-        <v>2046</v>
+        <v>2052</v>
       </c>
       <c r="C1277" s="1" t="s">
-        <v>2047</v>
+        <v>2053</v>
       </c>
       <c r="D1277" s="1"/>
       <c r="E1277" s="1"/>
@@ -27643,10 +27667,10 @@
     <row r="1278">
       <c r="A1278"/>
       <c r="B1278" t="s">
-        <v>2048</v>
+        <v>2054</v>
       </c>
       <c r="C1278" t="s">
-        <v>2049</v>
+        <v>2055</v>
       </c>
       <c r="D1278"/>
       <c r="E1278"/>
@@ -27659,10 +27683,10 @@
     <row r="1279">
       <c r="A1279"/>
       <c r="B1279" t="s">
-        <v>2050</v>
+        <v>2056</v>
       </c>
       <c r="C1279" t="s">
-        <v>2051</v>
+        <v>2057</v>
       </c>
       <c r="D1279"/>
       <c r="E1279"/>
@@ -27675,10 +27699,10 @@
     <row r="1280">
       <c r="A1280"/>
       <c r="B1280" t="s">
-        <v>2052</v>
+        <v>2058</v>
       </c>
       <c r="C1280" t="s">
-        <v>2053</v>
+        <v>2059</v>
       </c>
       <c r="D1280"/>
       <c r="E1280"/>
@@ -27691,10 +27715,10 @@
     <row r="1281">
       <c r="A1281"/>
       <c r="B1281" t="s">
-        <v>2054</v>
+        <v>2060</v>
       </c>
       <c r="C1281" t="s">
-        <v>2055</v>
+        <v>2061</v>
       </c>
       <c r="D1281"/>
       <c r="E1281"/>
@@ -27707,10 +27731,10 @@
     <row r="1282">
       <c r="A1282"/>
       <c r="B1282" t="s">
-        <v>2056</v>
+        <v>2062</v>
       </c>
       <c r="C1282" t="s">
-        <v>2057</v>
+        <v>2063</v>
       </c>
       <c r="D1282"/>
       <c r="E1282"/>
@@ -27723,10 +27747,10 @@
     <row r="1283">
       <c r="A1283"/>
       <c r="B1283" t="s">
-        <v>2058</v>
+        <v>2064</v>
       </c>
       <c r="C1283" t="s">
-        <v>2059</v>
+        <v>2065</v>
       </c>
       <c r="D1283"/>
       <c r="E1283"/>
@@ -27739,10 +27763,10 @@
     <row r="1284">
       <c r="A1284"/>
       <c r="B1284" t="s">
-        <v>2060</v>
+        <v>2066</v>
       </c>
       <c r="C1284" t="s">
-        <v>2061</v>
+        <v>2067</v>
       </c>
       <c r="D1284"/>
       <c r="E1284" t="s">
@@ -27757,10 +27781,10 @@
     <row r="1285">
       <c r="A1285"/>
       <c r="B1285" t="s">
-        <v>2062</v>
+        <v>2068</v>
       </c>
       <c r="C1285" t="s">
-        <v>2063</v>
+        <v>2069</v>
       </c>
       <c r="D1285"/>
       <c r="E1285" t="s">
@@ -27775,10 +27799,10 @@
     <row r="1286">
       <c r="A1286"/>
       <c r="B1286" t="s">
-        <v>2064</v>
+        <v>2070</v>
       </c>
       <c r="C1286" t="s">
-        <v>2065</v>
+        <v>2071</v>
       </c>
       <c r="D1286"/>
       <c r="E1286"/>
@@ -27791,10 +27815,10 @@
     <row r="1287">
       <c r="A1287"/>
       <c r="B1287" t="s">
-        <v>2066</v>
+        <v>2072</v>
       </c>
       <c r="C1287" t="s">
-        <v>2067</v>
+        <v>2073</v>
       </c>
       <c r="D1287"/>
       <c r="E1287" t="s">
@@ -27809,10 +27833,10 @@
     <row r="1288">
       <c r="A1288"/>
       <c r="B1288" t="s">
-        <v>2068</v>
+        <v>2074</v>
       </c>
       <c r="C1288" t="s">
-        <v>2069</v>
+        <v>2075</v>
       </c>
       <c r="D1288"/>
       <c r="E1288" t="s">
@@ -27827,10 +27851,10 @@
     <row r="1289">
       <c r="A1289"/>
       <c r="B1289" t="s">
-        <v>2070</v>
+        <v>2076</v>
       </c>
       <c r="C1289" t="s">
-        <v>2071</v>
+        <v>2077</v>
       </c>
       <c r="D1289"/>
       <c r="E1289"/>
@@ -27843,10 +27867,10 @@
     <row r="1290">
       <c r="A1290"/>
       <c r="B1290" t="s">
-        <v>2072</v>
+        <v>2078</v>
       </c>
       <c r="C1290" t="s">
-        <v>2073</v>
+        <v>2079</v>
       </c>
       <c r="D1290"/>
       <c r="E1290"/>
@@ -27859,10 +27883,10 @@
     <row r="1291">
       <c r="A1291"/>
       <c r="B1291" t="s">
-        <v>2074</v>
+        <v>2080</v>
       </c>
       <c r="C1291" t="s">
-        <v>2075</v>
+        <v>2081</v>
       </c>
       <c r="D1291"/>
       <c r="E1291"/>
@@ -27875,10 +27899,10 @@
     <row r="1292">
       <c r="A1292"/>
       <c r="B1292" t="s">
-        <v>2076</v>
+        <v>2082</v>
       </c>
       <c r="C1292" t="s">
-        <v>2077</v>
+        <v>2083</v>
       </c>
       <c r="D1292"/>
       <c r="E1292"/>
@@ -27891,10 +27915,10 @@
     <row r="1293">
       <c r="A1293"/>
       <c r="B1293" t="s">
-        <v>2078</v>
+        <v>2084</v>
       </c>
       <c r="C1293" t="s">
-        <v>2079</v>
+        <v>2085</v>
       </c>
       <c r="D1293"/>
       <c r="E1293"/>
@@ -27907,10 +27931,10 @@
     <row r="1294">
       <c r="A1294"/>
       <c r="B1294" t="s">
-        <v>2080</v>
+        <v>2086</v>
       </c>
       <c r="C1294" t="s">
-        <v>2081</v>
+        <v>2087</v>
       </c>
       <c r="D1294"/>
       <c r="E1294"/>
@@ -27923,10 +27947,10 @@
     <row r="1295">
       <c r="A1295"/>
       <c r="B1295" t="s">
-        <v>2082</v>
+        <v>2088</v>
       </c>
       <c r="C1295" t="s">
-        <v>2083</v>
+        <v>2089</v>
       </c>
       <c r="D1295"/>
       <c r="E1295"/>
@@ -27939,10 +27963,10 @@
     <row r="1296" ht="77" customHeight="1">
       <c r="A1296" s="1"/>
       <c r="B1296" s="1" t="s">
-        <v>2084</v>
+        <v>2090</v>
       </c>
       <c r="C1296" s="1" t="s">
-        <v>2085</v>
+        <v>2091</v>
       </c>
       <c r="D1296" s="1"/>
       <c r="E1296" s="1"/>
@@ -27955,10 +27979,10 @@
     <row r="1297" ht="77" customHeight="1">
       <c r="A1297" s="1"/>
       <c r="B1297" s="1" t="s">
-        <v>2086</v>
+        <v>2092</v>
       </c>
       <c r="C1297" s="1" t="s">
-        <v>2087</v>
+        <v>2093</v>
       </c>
       <c r="D1297" s="1"/>
       <c r="E1297" s="1"/>
@@ -27971,10 +27995,10 @@
     <row r="1298" ht="77" customHeight="1">
       <c r="A1298" s="1"/>
       <c r="B1298" s="1" t="s">
-        <v>2088</v>
+        <v>2094</v>
       </c>
       <c r="C1298" s="1" t="s">
-        <v>2089</v>
+        <v>2095</v>
       </c>
       <c r="D1298" s="1"/>
       <c r="E1298" s="1"/>
@@ -27987,10 +28011,10 @@
     <row r="1299" ht="77" customHeight="1">
       <c r="A1299" s="1"/>
       <c r="B1299" s="1" t="s">
-        <v>2090</v>
+        <v>2096</v>
       </c>
       <c r="C1299" s="1" t="s">
-        <v>2091</v>
+        <v>2097</v>
       </c>
       <c r="D1299" s="1"/>
       <c r="E1299" s="1"/>
@@ -28003,10 +28027,10 @@
     <row r="1300" ht="77" customHeight="1">
       <c r="A1300" s="1"/>
       <c r="B1300" s="1" t="s">
-        <v>2092</v>
+        <v>2098</v>
       </c>
       <c r="C1300" s="1" t="s">
-        <v>2093</v>
+        <v>2099</v>
       </c>
       <c r="D1300" s="1"/>
       <c r="E1300" s="1"/>
@@ -28019,10 +28043,10 @@
     <row r="1301" ht="77" customHeight="1">
       <c r="A1301" s="1"/>
       <c r="B1301" s="1" t="s">
-        <v>2094</v>
+        <v>2100</v>
       </c>
       <c r="C1301" s="1" t="s">
-        <v>2095</v>
+        <v>2101</v>
       </c>
       <c r="D1301" s="1"/>
       <c r="E1301" s="1"/>
@@ -28035,10 +28059,10 @@
     <row r="1302" ht="77" customHeight="1">
       <c r="A1302" s="1"/>
       <c r="B1302" s="1" t="s">
-        <v>2096</v>
+        <v>2102</v>
       </c>
       <c r="C1302" s="1" t="s">
-        <v>2097</v>
+        <v>2103</v>
       </c>
       <c r="D1302" s="1"/>
       <c r="E1302" s="1"/>
@@ -28051,10 +28075,10 @@
     <row r="1303" ht="77" customHeight="1">
       <c r="A1303" s="1"/>
       <c r="B1303" s="1" t="s">
-        <v>2098</v>
+        <v>2104</v>
       </c>
       <c r="C1303" s="1" t="s">
-        <v>2099</v>
+        <v>2105</v>
       </c>
       <c r="D1303" s="1"/>
       <c r="E1303" s="1"/>
@@ -28067,10 +28091,10 @@
     <row r="1304">
       <c r="A1304"/>
       <c r="B1304" t="s">
-        <v>2100</v>
+        <v>2106</v>
       </c>
       <c r="C1304" t="s">
-        <v>2101</v>
+        <v>2107</v>
       </c>
       <c r="D1304"/>
       <c r="E1304"/>
@@ -28083,10 +28107,10 @@
     <row r="1305">
       <c r="A1305"/>
       <c r="B1305" t="s">
-        <v>2102</v>
+        <v>2108</v>
       </c>
       <c r="C1305" t="s">
-        <v>2103</v>
+        <v>2109</v>
       </c>
       <c r="D1305"/>
       <c r="E1305"/>
@@ -28099,10 +28123,10 @@
     <row r="1306">
       <c r="A1306"/>
       <c r="B1306" t="s">
-        <v>2104</v>
+        <v>2110</v>
       </c>
       <c r="C1306" t="s">
-        <v>2105</v>
+        <v>2111</v>
       </c>
       <c r="D1306"/>
       <c r="E1306"/>
@@ -28115,10 +28139,10 @@
     <row r="1307">
       <c r="A1307"/>
       <c r="B1307" t="s">
-        <v>2106</v>
+        <v>2112</v>
       </c>
       <c r="C1307" t="s">
-        <v>2107</v>
+        <v>2113</v>
       </c>
       <c r="D1307"/>
       <c r="E1307"/>
@@ -28131,10 +28155,10 @@
     <row r="1308">
       <c r="A1308"/>
       <c r="B1308" t="s">
-        <v>2108</v>
+        <v>2114</v>
       </c>
       <c r="C1308" t="s">
-        <v>2109</v>
+        <v>2115</v>
       </c>
       <c r="D1308"/>
       <c r="E1308"/>
@@ -28147,10 +28171,10 @@
     <row r="1309">
       <c r="A1309"/>
       <c r="B1309" t="s">
-        <v>2110</v>
+        <v>2116</v>
       </c>
       <c r="C1309" t="s">
-        <v>2111</v>
+        <v>2117</v>
       </c>
       <c r="D1309"/>
       <c r="E1309"/>
@@ -28163,10 +28187,10 @@
     <row r="1310">
       <c r="A1310"/>
       <c r="B1310" t="s">
-        <v>2112</v>
+        <v>2118</v>
       </c>
       <c r="C1310" t="s">
-        <v>2113</v>
+        <v>2119</v>
       </c>
       <c r="D1310"/>
       <c r="E1310" t="s">
@@ -28181,10 +28205,10 @@
     <row r="1311">
       <c r="A1311"/>
       <c r="B1311" t="s">
-        <v>2114</v>
+        <v>2120</v>
       </c>
       <c r="C1311" t="s">
-        <v>2115</v>
+        <v>2121</v>
       </c>
       <c r="D1311"/>
       <c r="E1311" t="s">
@@ -28227,7 +28251,7 @@
     <row r="1314">
       <c r="A1314"/>
       <c r="B1314" t="s">
-        <v>2116</v>
+        <v>2122</v>
       </c>
       <c r="C1314" t="s">
         <v>18</v>
@@ -28243,7 +28267,7 @@
     <row r="1315">
       <c r="A1315"/>
       <c r="B1315" t="s">
-        <v>2117</v>
+        <v>2123</v>
       </c>
       <c r="C1315" t="s">
         <v>21</v>
@@ -28261,7 +28285,7 @@
     <row r="1316">
       <c r="A1316"/>
       <c r="B1316" t="s">
-        <v>2118</v>
+        <v>2124</v>
       </c>
       <c r="C1316" t="s">
         <v>24</v>
@@ -28277,7 +28301,7 @@
     <row r="1317" ht="77" customHeight="1">
       <c r="A1317" s="1"/>
       <c r="B1317" s="1" t="s">
-        <v>2119</v>
+        <v>2125</v>
       </c>
       <c r="C1317" s="1" t="s">
         <v>26</v>
@@ -28293,7 +28317,7 @@
     <row r="1318" ht="77" customHeight="1">
       <c r="A1318" s="1"/>
       <c r="B1318" s="1" t="s">
-        <v>2120</v>
+        <v>2126</v>
       </c>
       <c r="C1318" s="1" t="s">
         <v>29</v>
@@ -28309,7 +28333,7 @@
     <row r="1319" ht="77" customHeight="1">
       <c r="A1319" s="1"/>
       <c r="B1319" s="1" t="s">
-        <v>2121</v>
+        <v>2127</v>
       </c>
       <c r="C1319" s="1" t="s">
         <v>31</v>
@@ -28325,7 +28349,7 @@
     <row r="1320" ht="77" customHeight="1">
       <c r="A1320" s="1"/>
       <c r="B1320" s="1" t="s">
-        <v>2122</v>
+        <v>2128</v>
       </c>
       <c r="C1320" s="1" t="s">
         <v>33</v>
@@ -28341,7 +28365,7 @@
     <row r="1321" ht="77" customHeight="1">
       <c r="A1321" s="1"/>
       <c r="B1321" s="1" t="s">
-        <v>2123</v>
+        <v>2129</v>
       </c>
       <c r="C1321" s="1" t="s">
         <v>35</v>
@@ -28357,7 +28381,7 @@
     <row r="1322" ht="77" customHeight="1">
       <c r="A1322" s="1"/>
       <c r="B1322" s="1" t="s">
-        <v>2124</v>
+        <v>2130</v>
       </c>
       <c r="C1322" s="1" t="s">
         <v>37</v>
@@ -28373,7 +28397,7 @@
     <row r="1323" ht="77" customHeight="1">
       <c r="A1323" s="1"/>
       <c r="B1323" s="1" t="s">
-        <v>2125</v>
+        <v>2131</v>
       </c>
       <c r="C1323" s="1" t="s">
         <v>39</v>
@@ -28389,7 +28413,7 @@
     <row r="1324" ht="77" customHeight="1">
       <c r="A1324" s="1"/>
       <c r="B1324" s="1" t="s">
-        <v>2126</v>
+        <v>2132</v>
       </c>
       <c r="C1324" s="1" t="s">
         <v>41</v>
@@ -28405,7 +28429,7 @@
     <row r="1325" ht="77" customHeight="1">
       <c r="A1325" s="1"/>
       <c r="B1325" s="1" t="s">
-        <v>2127</v>
+        <v>2133</v>
       </c>
       <c r="C1325" s="1" t="s">
         <v>44</v>
@@ -28423,7 +28447,7 @@
     <row r="1326" ht="77" customHeight="1">
       <c r="A1326" s="1"/>
       <c r="B1326" s="1" t="s">
-        <v>2128</v>
+        <v>2134</v>
       </c>
       <c r="C1326" s="1" t="s">
         <v>46</v>
@@ -28441,7 +28465,7 @@
     <row r="1327">
       <c r="A1327"/>
       <c r="B1327" t="s">
-        <v>2129</v>
+        <v>2135</v>
       </c>
       <c r="C1327" t="s">
         <v>56</v>
@@ -28457,10 +28481,10 @@
     <row r="1328">
       <c r="A1328"/>
       <c r="B1328" t="s">
-        <v>2130</v>
+        <v>2136</v>
       </c>
       <c r="C1328" t="s">
-        <v>2131</v>
+        <v>2137</v>
       </c>
       <c r="D1328"/>
       <c r="E1328"/>
@@ -28473,10 +28497,10 @@
     <row r="1329">
       <c r="A1329"/>
       <c r="B1329" t="s">
-        <v>2132</v>
+        <v>2138</v>
       </c>
       <c r="C1329" t="s">
-        <v>2133</v>
+        <v>2139</v>
       </c>
       <c r="D1329"/>
       <c r="E1329"/>
@@ -28489,10 +28513,10 @@
     <row r="1330">
       <c r="A1330"/>
       <c r="B1330" t="s">
-        <v>2134</v>
+        <v>2140</v>
       </c>
       <c r="C1330" t="s">
-        <v>2135</v>
+        <v>2141</v>
       </c>
       <c r="D1330"/>
       <c r="E1330"/>
@@ -28505,10 +28529,10 @@
     <row r="1331">
       <c r="A1331"/>
       <c r="B1331" t="s">
-        <v>2136</v>
+        <v>2142</v>
       </c>
       <c r="C1331" t="s">
-        <v>2137</v>
+        <v>2143</v>
       </c>
       <c r="D1331"/>
       <c r="E1331"/>
@@ -28521,10 +28545,10 @@
     <row r="1332">
       <c r="A1332"/>
       <c r="B1332" t="s">
-        <v>2138</v>
+        <v>2144</v>
       </c>
       <c r="C1332" t="s">
-        <v>2139</v>
+        <v>2145</v>
       </c>
       <c r="D1332"/>
       <c r="E1332"/>
@@ -28537,10 +28561,10 @@
     <row r="1333">
       <c r="A1333"/>
       <c r="B1333" t="s">
-        <v>2140</v>
+        <v>2146</v>
       </c>
       <c r="C1333" t="s">
-        <v>2141</v>
+        <v>2147</v>
       </c>
       <c r="D1333"/>
       <c r="E1333"/>
@@ -28553,10 +28577,10 @@
     <row r="1334">
       <c r="A1334"/>
       <c r="B1334" t="s">
-        <v>2142</v>
+        <v>2148</v>
       </c>
       <c r="C1334" t="s">
-        <v>2143</v>
+        <v>2149</v>
       </c>
       <c r="D1334"/>
       <c r="E1334"/>
@@ -28569,10 +28593,10 @@
     <row r="1335">
       <c r="A1335"/>
       <c r="B1335" t="s">
-        <v>2144</v>
+        <v>2150</v>
       </c>
       <c r="C1335" t="s">
-        <v>2145</v>
+        <v>2151</v>
       </c>
       <c r="D1335"/>
       <c r="E1335"/>
@@ -28584,17 +28608,17 @@
     </row>
     <row r="1336">
       <c r="A1336" t="s">
-        <v>2146</v>
+        <v>2152</v>
       </c>
       <c r="B1336" t="s">
-        <v>2147</v>
+        <v>2153</v>
       </c>
       <c r="C1336" t="s">
-        <v>2147</v>
+        <v>2153</v>
       </c>
       <c r="D1336"/>
       <c r="E1336" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="F1336"/>
       <c r="G1336"/>
@@ -28605,14 +28629,14 @@
     <row r="1337">
       <c r="A1337"/>
       <c r="B1337" t="s">
-        <v>2149</v>
+        <v>2155</v>
       </c>
       <c r="C1337" t="s">
-        <v>2149</v>
+        <v>2155</v>
       </c>
       <c r="D1337"/>
       <c r="E1337" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="F1337"/>
       <c r="G1337"/>
@@ -28623,14 +28647,14 @@
     <row r="1338">
       <c r="A1338"/>
       <c r="B1338" t="s">
-        <v>2150</v>
+        <v>2156</v>
       </c>
       <c r="C1338" t="s">
-        <v>2150</v>
+        <v>2156</v>
       </c>
       <c r="D1338"/>
       <c r="E1338" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="F1338"/>
       <c r="G1338"/>
@@ -28660,7 +28684,7 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>2151</v>
+        <v>2157</v>
       </c>
       <c r="B2"/>
       <c r="C2"/>
@@ -28669,7 +28693,7 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>2152</v>
+        <v>2158</v>
       </c>
       <c r="B3"/>
       <c r="C3"/>
@@ -28678,7 +28702,7 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>2153</v>
+        <v>2159</v>
       </c>
       <c r="B4"/>
       <c r="C4"/>
@@ -28694,16 +28718,16 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>2154</v>
+        <v>2160</v>
       </c>
       <c r="B6" t="s">
         <v>6</v>
       </c>
       <c r="C6" t="s">
-        <v>2155</v>
+        <v>2161</v>
       </c>
       <c r="D6" t="s">
-        <v>2156</v>
+        <v>2162</v>
       </c>
       <c r="E6" t="s">
         <v>12</v>
@@ -28711,16 +28735,16 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>2157</v>
+        <v>2163</v>
       </c>
       <c r="B7" t="s">
-        <v>2158</v>
+        <v>2164</v>
       </c>
       <c r="C7" t="s">
-        <v>2159</v>
+        <v>2165</v>
       </c>
       <c r="D7" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E7" t="s">
         <v>19</v>
@@ -28728,16 +28752,16 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>2157</v>
+        <v>2163</v>
       </c>
       <c r="B8" t="s">
-        <v>2160</v>
+        <v>2166</v>
       </c>
       <c r="C8" t="s">
-        <v>2161</v>
+        <v>2167</v>
       </c>
       <c r="D8" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E8" t="s">
         <v>19</v>
@@ -28745,16 +28769,16 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>2162</v>
+        <v>2168</v>
       </c>
       <c r="B9" t="s">
-        <v>2163</v>
+        <v>2169</v>
       </c>
       <c r="C9" t="s">
-        <v>2159</v>
+        <v>2165</v>
       </c>
       <c r="D9" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E9" t="s">
         <v>19</v>
@@ -28762,16 +28786,16 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>2162</v>
+        <v>2168</v>
       </c>
       <c r="B10" t="s">
-        <v>2164</v>
+        <v>2170</v>
       </c>
       <c r="C10" t="s">
-        <v>2161</v>
+        <v>2167</v>
       </c>
       <c r="D10" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E10" t="s">
         <v>19</v>
@@ -28779,16 +28803,16 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
+        <v>2171</v>
+      </c>
+      <c r="B11" t="s">
+        <v>2172</v>
+      </c>
+      <c r="C11" t="s">
         <v>2165</v>
       </c>
-      <c r="B11" t="s">
-        <v>2166</v>
-      </c>
-      <c r="C11" t="s">
-        <v>2159</v>
-      </c>
       <c r="D11" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E11" t="s">
         <v>19</v>
@@ -28796,16 +28820,16 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>2165</v>
+        <v>2171</v>
       </c>
       <c r="B12" t="s">
+        <v>2173</v>
+      </c>
+      <c r="C12" t="s">
         <v>2167</v>
       </c>
-      <c r="C12" t="s">
-        <v>2161</v>
-      </c>
       <c r="D12" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E12" t="s">
         <v>19</v>
@@ -28813,13 +28837,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>2168</v>
+        <v>2174</v>
       </c>
       <c r="B13" t="s">
-        <v>2169</v>
+        <v>2175</v>
       </c>
       <c r="C13" t="s">
-        <v>2170</v>
+        <v>2176</v>
       </c>
       <c r="D13" t="s">
         <v>105</v>
@@ -28830,13 +28854,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>2171</v>
+        <v>2177</v>
       </c>
       <c r="B14" t="s">
-        <v>2172</v>
+        <v>2178</v>
       </c>
       <c r="C14" t="s">
-        <v>2173</v>
+        <v>2179</v>
       </c>
       <c r="D14" t="s">
         <v>105</v>
@@ -28847,16 +28871,16 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
       <c r="B15" t="s">
-        <v>2175</v>
+        <v>2181</v>
       </c>
       <c r="C15" t="s">
-        <v>2176</v>
+        <v>2182</v>
       </c>
       <c r="D15" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E15" t="s">
         <v>19</v>
@@ -28864,16 +28888,16 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
       <c r="B16" t="s">
-        <v>2177</v>
+        <v>2183</v>
       </c>
       <c r="C16" t="s">
-        <v>2178</v>
+        <v>2184</v>
       </c>
       <c r="D16" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E16" t="s">
         <v>19</v>
@@ -28881,16 +28905,16 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
       <c r="B17" t="s">
-        <v>2179</v>
+        <v>2185</v>
       </c>
       <c r="C17" t="s">
-        <v>2180</v>
+        <v>2186</v>
       </c>
       <c r="D17" t="s">
-        <v>2181</v>
+        <v>2187</v>
       </c>
       <c r="E17" t="s">
         <v>19</v>
@@ -28898,16 +28922,16 @@
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>2174</v>
+        <v>2180</v>
       </c>
       <c r="B18" t="s">
-        <v>2182</v>
+        <v>2188</v>
       </c>
       <c r="C18" t="s">
-        <v>2183</v>
+        <v>2189</v>
       </c>
       <c r="D18" t="s">
-        <v>2148</v>
+        <v>2154</v>
       </c>
       <c r="E18" t="s">
         <v>19</v>

</xml_diff>